<commit_message>
Update Squash sheet in matchups workbook for U15/U25/Above-25 split
Mirrors the index.html restructure: Under 15 knockout unchanged,
new Under 25 round robin + final section, Above 25 regrouped into
two 3-player pools with crossover semis and a final on Aug 16.
</commit_message>
<xml_diff>
--- a/Ekta_Schedule_With_Matchups.xlsx
+++ b/Ekta_Schedule_With_Matchups.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TT Women's Singles" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table Tennis Singles Men" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table Tennis Doubles" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carrom Singles Men" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carrom Singles Women" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carrom Doubles" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pool" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chess" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Squash" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TT Women's Singles" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Table Tennis Singles Men" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Table Tennis Doubles" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Carrom Singles Men" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Carrom Singles Women" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Carrom Doubles" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Pool" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Chess" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Squash" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,8 +79,12 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font/>
+    <font>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="17">
+  <fills count="23">
     <fill>
       <patternFill/>
     </fill>
@@ -174,8 +178,38 @@
         <bgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00203864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B4C7E7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00366092"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0070AD47"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -231,11 +265,12 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -303,6 +338,35 @@
     <xf numFmtId="0" fontId="10" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="21" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="22" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1391,7 +1455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1404,1337 +1468,1426 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>SQUASH TOURNAMENT - PLAYER GROUPS</t>
         </is>
       </c>
+      <c r="B1" s="30" t="n"/>
+      <c r="C1" s="30" t="n"/>
+      <c r="D1" s="30" t="n"/>
+      <c r="E1" s="31" t="n"/>
+      <c r="F1" s="31" t="n"/>
+      <c r="G1" s="31" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="31" t="n"/>
+      <c r="B2" s="31" t="n"/>
+      <c r="C2" s="31" t="n"/>
+      <c r="D2" s="31" t="n"/>
+      <c r="E2" s="31" t="n"/>
+      <c r="F2" s="31" t="n"/>
+      <c r="G2" s="31" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="32" t="inlineStr">
         <is>
           <t>UNDER 15 (7 Players) - SINGLE ELIMINATION KNOCKOUT</t>
         </is>
       </c>
+      <c r="B3" s="33" t="n"/>
+      <c r="C3" s="33" t="n"/>
+      <c r="D3" s="33" t="n"/>
+      <c r="E3" s="31" t="n"/>
+      <c r="F3" s="31" t="n"/>
+      <c r="G3" s="31" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="34" t="inlineStr">
         <is>
           <t>S.No</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="34" t="inlineStr">
         <is>
           <t>Player Name</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="34" t="inlineStr">
         <is>
           <t>Age</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="34" t="inlineStr">
         <is>
           <t>Group/Seed</t>
         </is>
       </c>
+      <c r="E4" s="31" t="n"/>
+      <c r="F4" s="31" t="n"/>
+      <c r="G4" s="31" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="n">
+      <c r="A5" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="35" t="inlineStr">
         <is>
           <t>Shaurya Tripathi</t>
         </is>
       </c>
-      <c r="C5" s="8" t="n">
+      <c r="C5" s="35" t="n">
         <v>10</v>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="35" t="inlineStr">
         <is>
           <t>Round 1</t>
         </is>
       </c>
+      <c r="E5" s="31" t="n"/>
+      <c r="F5" s="31" t="n"/>
+      <c r="G5" s="31" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="n">
+      <c r="A6" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="35" t="inlineStr">
         <is>
           <t>Parth yadav</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="35" t="n">
         <v>10</v>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="35" t="inlineStr">
         <is>
           <t>Round 1</t>
         </is>
       </c>
+      <c r="E6" s="31" t="n"/>
+      <c r="F6" s="31" t="n"/>
+      <c r="G6" s="31" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="35" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="35" t="inlineStr">
         <is>
           <t>Peher Krunal Shah</t>
         </is>
       </c>
-      <c r="C7" s="8" t="n">
+      <c r="C7" s="35" t="n">
         <v>12</v>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="35" t="inlineStr">
         <is>
           <t>Round 1</t>
         </is>
       </c>
+      <c r="E7" s="31" t="n"/>
+      <c r="F7" s="31" t="n"/>
+      <c r="G7" s="31" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="n">
+      <c r="A8" s="35" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="35" t="inlineStr">
         <is>
           <t>Aadit Joshi</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="35" t="n">
         <v>12</v>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="35" t="inlineStr">
         <is>
           <t>Round 1</t>
         </is>
       </c>
+      <c r="E8" s="31" t="n"/>
+      <c r="F8" s="31" t="n"/>
+      <c r="G8" s="31" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="n">
+      <c r="A9" s="35" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="35" t="inlineStr">
         <is>
           <t>Viaan Neema</t>
         </is>
       </c>
-      <c r="C9" s="8" t="n">
+      <c r="C9" s="35" t="n">
         <v>12</v>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="35" t="inlineStr">
         <is>
           <t>Round 1</t>
         </is>
       </c>
+      <c r="E9" s="31" t="n"/>
+      <c r="F9" s="31" t="n"/>
+      <c r="G9" s="31" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="n">
+      <c r="A10" s="35" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="35" t="inlineStr">
         <is>
           <t>Yash agarwal</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n">
+      <c r="C10" s="35" t="n">
         <v>13</v>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="35" t="inlineStr">
         <is>
           <t>Round 1</t>
         </is>
       </c>
+      <c r="E10" s="31" t="n"/>
+      <c r="F10" s="31" t="n"/>
+      <c r="G10" s="31" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="n">
+      <c r="A11" s="35" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="35" t="inlineStr">
         <is>
           <t>Hridh jhala</t>
         </is>
       </c>
-      <c r="C11" s="8" t="n">
+      <c r="C11" s="35" t="n">
         <v>13</v>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="35" t="inlineStr">
         <is>
           <t>BYE (Semifinal)</t>
         </is>
       </c>
+      <c r="E11" s="31" t="n"/>
+      <c r="F11" s="31" t="n"/>
+      <c r="G11" s="31" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="31" t="n"/>
+      <c r="B12" s="31" t="n"/>
+      <c r="C12" s="31" t="n"/>
+      <c r="D12" s="31" t="n"/>
+      <c r="E12" s="31" t="n"/>
+      <c r="F12" s="31" t="n"/>
+      <c r="G12" s="31" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>ABOVE 15 (9 Players) - TWO POOL GROUPS</t>
-        </is>
-      </c>
+      <c r="A13" s="32" t="inlineStr">
+        <is>
+          <t>UNDER 25 (3 Players) - ROUND ROBIN + FINAL</t>
+        </is>
+      </c>
+      <c r="B13" s="33" t="n"/>
+      <c r="C13" s="33" t="n"/>
+      <c r="D13" s="33" t="n"/>
+      <c r="E13" s="31" t="n"/>
+      <c r="F13" s="31" t="n"/>
+      <c r="G13" s="31" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>GROUP A (5 Players) - Round Robin Pool</t>
-        </is>
-      </c>
+      <c r="A14" s="34" t="inlineStr">
+        <is>
+          <t>S.No</t>
+        </is>
+      </c>
+      <c r="B14" s="34" t="inlineStr">
+        <is>
+          <t>Player Name</t>
+        </is>
+      </c>
+      <c r="C14" s="34" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="D14" s="34" t="inlineStr">
+        <is>
+          <t>Group/Seed</t>
+        </is>
+      </c>
+      <c r="E14" s="31" t="n"/>
+      <c r="F14" s="31" t="n"/>
+      <c r="G14" s="31" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" s="35" t="inlineStr">
+        <is>
+          <t>Aaditya Kumar</t>
+        </is>
+      </c>
+      <c r="C15" s="35" t="n">
+        <v>17</v>
+      </c>
+      <c r="D15" s="35" t="inlineStr">
+        <is>
+          <t>Round Robin</t>
+        </is>
+      </c>
+      <c r="E15" s="31" t="n"/>
+      <c r="F15" s="31" t="n"/>
+      <c r="G15" s="31" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" s="35" t="inlineStr">
+        <is>
+          <t>Hryday Goyal</t>
+        </is>
+      </c>
+      <c r="C16" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="D16" s="35" t="inlineStr">
+        <is>
+          <t>Round Robin</t>
+        </is>
+      </c>
+      <c r="E16" s="31" t="n"/>
+      <c r="F16" s="31" t="n"/>
+      <c r="G16" s="31" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="35" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" s="35" t="inlineStr">
+        <is>
+          <t>Shravan Gajera</t>
+        </is>
+      </c>
+      <c r="C17" s="35" t="n">
+        <v>23</v>
+      </c>
+      <c r="D17" s="35" t="inlineStr">
+        <is>
+          <t>Round Robin</t>
+        </is>
+      </c>
+      <c r="E17" s="31" t="n"/>
+      <c r="F17" s="31" t="n"/>
+      <c r="G17" s="31" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="31" t="n"/>
+      <c r="B18" s="31" t="n"/>
+      <c r="C18" s="31" t="n"/>
+      <c r="D18" s="31" t="n"/>
+      <c r="E18" s="31" t="n"/>
+      <c r="F18" s="31" t="n"/>
+      <c r="G18" s="31" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="32" t="inlineStr">
+        <is>
+          <t>ABOVE 25 (6 Players) - TWO POOL GROUPS</t>
+        </is>
+      </c>
+      <c r="B19" s="33" t="n"/>
+      <c r="C19" s="33" t="n"/>
+      <c r="D19" s="33" t="n"/>
+      <c r="E19" s="31" t="n"/>
+      <c r="F19" s="31" t="n"/>
+      <c r="G19" s="31" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="36" t="inlineStr">
+        <is>
+          <t>GROUP A (3 Players) - Round Robin Pool</t>
+        </is>
+      </c>
+      <c r="B20" s="37" t="n"/>
+      <c r="C20" s="37" t="n"/>
+      <c r="D20" s="37" t="n"/>
+      <c r="E20" s="31" t="n"/>
+      <c r="F20" s="31" t="n"/>
+      <c r="G20" s="31" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="34" t="inlineStr">
         <is>
           <t>S.No</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B21" s="34" t="inlineStr">
         <is>
           <t>Player Name</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C21" s="34" t="inlineStr">
         <is>
           <t>Age</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="n">
+      <c r="D21" s="34" t="inlineStr">
+        <is>
+          <t>Group/Seed</t>
+        </is>
+      </c>
+      <c r="E21" s="31" t="n"/>
+      <c r="F21" s="31" t="n"/>
+      <c r="G21" s="31" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Shravan Gajera</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="n">
-        <v>23</v>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="B22" s="35" t="inlineStr">
+        <is>
+          <t>Ravi Modi</t>
+        </is>
+      </c>
+      <c r="C22" s="35" t="n">
+        <v>29</v>
+      </c>
+      <c r="D22" s="35" t="inlineStr">
         <is>
           <t>Group A</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="n">
+      <c r="E22" s="31" t="n"/>
+      <c r="F22" s="31" t="n"/>
+      <c r="G22" s="31" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Hryday Goyal</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="B23" s="35" t="inlineStr">
+        <is>
+          <t>Mayank Aggarwal</t>
+        </is>
+      </c>
+      <c r="C23" s="35" t="n">
+        <v>40</v>
+      </c>
+      <c r="D23" s="35" t="inlineStr">
         <is>
           <t>Group A</t>
         </is>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="n">
+      <c r="E23" s="31" t="n"/>
+      <c r="F23" s="31" t="n"/>
+      <c r="G23" s="31" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="35" t="n">
         <v>3</v>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B24" s="35" t="inlineStr">
+        <is>
+          <t>Tejas doshi</t>
+        </is>
+      </c>
+      <c r="C24" s="35" t="n">
+        <v>40</v>
+      </c>
+      <c r="D24" s="35" t="inlineStr">
+        <is>
+          <t>Group A</t>
+        </is>
+      </c>
+      <c r="E24" s="31" t="n"/>
+      <c r="F24" s="31" t="n"/>
+      <c r="G24" s="31" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="31" t="n"/>
+      <c r="B25" s="31" t="n"/>
+      <c r="C25" s="31" t="n"/>
+      <c r="D25" s="31" t="n"/>
+      <c r="E25" s="31" t="n"/>
+      <c r="F25" s="31" t="n"/>
+      <c r="G25" s="31" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="36" t="inlineStr">
+        <is>
+          <t>GROUP B (3 Players) - Round Robin Pool</t>
+        </is>
+      </c>
+      <c r="B26" s="37" t="n"/>
+      <c r="C26" s="37" t="n"/>
+      <c r="D26" s="37" t="n"/>
+      <c r="E26" s="31" t="n"/>
+      <c r="F26" s="31" t="n"/>
+      <c r="G26" s="31" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="34" t="inlineStr">
+        <is>
+          <t>S.No</t>
+        </is>
+      </c>
+      <c r="B27" s="34" t="inlineStr">
+        <is>
+          <t>Player Name</t>
+        </is>
+      </c>
+      <c r="C27" s="34" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="D27" s="34" t="inlineStr">
+        <is>
+          <t>Group/Seed</t>
+        </is>
+      </c>
+      <c r="E27" s="31" t="n"/>
+      <c r="F27" s="31" t="n"/>
+      <c r="G27" s="31" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="B28" s="35" t="inlineStr">
         <is>
           <t>Dr Rahul Modi</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C28" s="35" t="n">
         <v>36</v>
       </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>Group A</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="D28" s="35" t="inlineStr">
+        <is>
+          <t>Group B</t>
+        </is>
+      </c>
+      <c r="E28" s="31" t="n"/>
+      <c r="F28" s="31" t="n"/>
+      <c r="G28" s="31" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="B29" s="35" t="inlineStr">
         <is>
           <t>Tanmay Sharma</t>
         </is>
       </c>
-      <c r="C19" s="8" t="n">
+      <c r="C29" s="35" t="n">
         <v>39</v>
       </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>Group A</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>Mayank Aggarwal</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="n">
-        <v>40</v>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>Group A</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>GROUP B (4 Players) - Round Robin Pool</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>S.No</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Player Name</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>Age</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Aaditya Kumar</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D29" s="35" t="inlineStr">
         <is>
           <t>Group B</t>
         </is>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>Ravi Modi</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="n">
-        <v>29</v>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
+      <c r="E29" s="31" t="n"/>
+      <c r="F29" s="31" t="n"/>
+      <c r="G29" s="31" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="35" t="n">
+        <v>3</v>
+      </c>
+      <c r="B30" s="35" t="inlineStr">
+        <is>
+          <t>Vinit Padia</t>
+        </is>
+      </c>
+      <c r="C30" s="35" t="n">
+        <v>44</v>
+      </c>
+      <c r="D30" s="35" t="inlineStr">
         <is>
           <t>Group B</t>
         </is>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>Tejas doshi</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="n">
-        <v>40</v>
-      </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>Group B</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>Vinit Padia</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="n">
-        <v>44</v>
-      </c>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>Group B</t>
-        </is>
-      </c>
-    </row>
-    <row r="29"/>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="E30" s="31" t="n"/>
+      <c r="F30" s="31" t="n"/>
+      <c r="G30" s="31" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="31" t="n"/>
+      <c r="B31" s="31" t="n"/>
+      <c r="C31" s="31" t="n"/>
+      <c r="D31" s="31" t="n"/>
+      <c r="E31" s="31" t="n"/>
+      <c r="F31" s="31" t="n"/>
+      <c r="G31" s="31" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="31" t="n"/>
+      <c r="B32" s="31" t="n"/>
+      <c r="C32" s="31" t="n"/>
+      <c r="D32" s="31" t="n"/>
+      <c r="E32" s="31" t="n"/>
+      <c r="F32" s="31" t="n"/>
+      <c r="G32" s="31" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="32" t="inlineStr">
         <is>
           <t>SQUASH TOURNAMENT SCHEDULE</t>
         </is>
       </c>
-    </row>
-    <row r="31"/>
-    <row r="32">
-      <c r="A32" s="11" t="inlineStr">
+      <c r="B33" s="33" t="n"/>
+      <c r="C33" s="33" t="n"/>
+      <c r="D33" s="33" t="n"/>
+      <c r="E33" s="33" t="n"/>
+      <c r="F33" s="33" t="n"/>
+      <c r="G33" s="31" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="31" t="n"/>
+      <c r="B34" s="31" t="n"/>
+      <c r="C34" s="31" t="n"/>
+      <c r="D34" s="31" t="n"/>
+      <c r="E34" s="31" t="n"/>
+      <c r="F34" s="31" t="n"/>
+      <c r="G34" s="31" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="38" t="inlineStr">
         <is>
           <t>AUGUST 15 - POOLS &amp; KNOCKOUTS</t>
         </is>
       </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="12" t="inlineStr">
+      <c r="B35" s="30" t="n"/>
+      <c r="C35" s="30" t="n"/>
+      <c r="D35" s="30" t="n"/>
+      <c r="E35" s="30" t="n"/>
+      <c r="F35" s="30" t="n"/>
+      <c r="G35" s="31" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="39" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
+      <c r="B36" s="39" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
       </c>
-      <c r="C33" s="12" t="inlineStr">
+      <c r="C36" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D33" s="12" t="inlineStr">
+      <c r="D36" s="39" t="inlineStr">
         <is>
           <t>Player A</t>
         </is>
       </c>
-      <c r="E33" s="12" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F33" s="12" t="inlineStr">
+      <c r="E36" s="39" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F36" s="39" t="inlineStr">
         <is>
           <t>Player B</t>
         </is>
       </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="G36" s="31" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="35" t="inlineStr">
         <is>
           <t>8:30 AM</t>
         </is>
       </c>
-      <c r="B34" s="8" t="inlineStr">
+      <c r="B37" s="35" t="inlineStr">
         <is>
           <t>U15-R1-M1</t>
         </is>
       </c>
-      <c r="C34" s="8" t="inlineStr">
+      <c r="C37" s="35" t="inlineStr">
         <is>
           <t>U15-R1</t>
         </is>
       </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="D37" s="35" t="inlineStr">
         <is>
           <t>Shaurya Tripathi (10)</t>
         </is>
       </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
+      <c r="E37" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F37" s="35" t="inlineStr">
         <is>
           <t>Parth yadav (10)</t>
         </is>
       </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="G37" s="31" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="35" t="inlineStr">
         <is>
           <t>8:48 AM</t>
         </is>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B38" s="35" t="inlineStr">
+        <is>
+          <t>U25-1</t>
+        </is>
+      </c>
+      <c r="C38" s="35" t="inlineStr">
+        <is>
+          <t>U25</t>
+        </is>
+      </c>
+      <c r="D38" s="35" t="inlineStr">
+        <is>
+          <t>Aaditya Kumar (17)</t>
+        </is>
+      </c>
+      <c r="E38" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F38" s="35" t="inlineStr">
+        <is>
+          <t>Hryday Goyal (20)</t>
+        </is>
+      </c>
+      <c r="G38" s="31" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="35" t="inlineStr">
+        <is>
+          <t>9:06 AM</t>
+        </is>
+      </c>
+      <c r="B39" s="35" t="inlineStr">
+        <is>
+          <t>U15-R1-M2</t>
+        </is>
+      </c>
+      <c r="C39" s="35" t="inlineStr">
+        <is>
+          <t>U15-R1</t>
+        </is>
+      </c>
+      <c r="D39" s="35" t="inlineStr">
+        <is>
+          <t>Peher Krunal Shah (12)</t>
+        </is>
+      </c>
+      <c r="E39" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F39" s="35" t="inlineStr">
+        <is>
+          <t>Aadit Joshi (12)</t>
+        </is>
+      </c>
+      <c r="G39" s="31" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="35" t="inlineStr">
+        <is>
+          <t>9:24 AM</t>
+        </is>
+      </c>
+      <c r="B40" s="35" t="inlineStr">
+        <is>
+          <t>U25-2</t>
+        </is>
+      </c>
+      <c r="C40" s="35" t="inlineStr">
+        <is>
+          <t>U25</t>
+        </is>
+      </c>
+      <c r="D40" s="35" t="inlineStr">
+        <is>
+          <t>Aaditya Kumar (17)</t>
+        </is>
+      </c>
+      <c r="E40" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F40" s="35" t="inlineStr">
+        <is>
+          <t>Shravan Gajera (23)</t>
+        </is>
+      </c>
+      <c r="G40" s="31" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="35" t="inlineStr">
+        <is>
+          <t>9:42 AM</t>
+        </is>
+      </c>
+      <c r="B41" s="35" t="inlineStr">
         <is>
           <t>GA-1</t>
         </is>
       </c>
-      <c r="C35" s="8" t="inlineStr">
+      <c r="C41" s="35" t="inlineStr">
         <is>
           <t>GA</t>
         </is>
       </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="D41" s="35" t="inlineStr">
+        <is>
+          <t>Ravi Modi (29)</t>
+        </is>
+      </c>
+      <c r="E41" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F41" s="35" t="inlineStr">
+        <is>
+          <t>Mayank Aggarwal (40)</t>
+        </is>
+      </c>
+      <c r="G41" s="31" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="35" t="inlineStr">
+        <is>
+          <t>11:00 AM</t>
+        </is>
+      </c>
+      <c r="B42" s="35" t="inlineStr">
+        <is>
+          <t>U15-R1-M3</t>
+        </is>
+      </c>
+      <c r="C42" s="35" t="inlineStr">
+        <is>
+          <t>U15-R1</t>
+        </is>
+      </c>
+      <c r="D42" s="35" t="inlineStr">
+        <is>
+          <t>Viaan Neema (12)</t>
+        </is>
+      </c>
+      <c r="E42" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F42" s="35" t="inlineStr">
+        <is>
+          <t>Yash agarwal (13)</t>
+        </is>
+      </c>
+      <c r="G42" s="31" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="35" t="inlineStr">
+        <is>
+          <t>11:18 AM</t>
+        </is>
+      </c>
+      <c r="B43" s="35" t="inlineStr">
+        <is>
+          <t>U25-3</t>
+        </is>
+      </c>
+      <c r="C43" s="35" t="inlineStr">
+        <is>
+          <t>U25</t>
+        </is>
+      </c>
+      <c r="D43" s="35" t="inlineStr">
+        <is>
+          <t>Hryday Goyal (20)</t>
+        </is>
+      </c>
+      <c r="E43" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F43" s="35" t="inlineStr">
         <is>
           <t>Shravan Gajera (23)</t>
         </is>
       </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>Hryday Goyal (20)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>9:06 AM</t>
-        </is>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>U15-R1-M2</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>U15-R1</t>
-        </is>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>Peher Krunal Shah (12)</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
-        <is>
-          <t>Aadit Joshi (12)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t>9:24 AM</t>
-        </is>
-      </c>
-      <c r="B37" s="8" t="inlineStr">
+      <c r="G43" s="31" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="35" t="inlineStr">
+        <is>
+          <t>11:36 AM</t>
+        </is>
+      </c>
+      <c r="B44" s="35" t="inlineStr">
+        <is>
+          <t>GB-1</t>
+        </is>
+      </c>
+      <c r="C44" s="35" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="D44" s="35" t="inlineStr">
+        <is>
+          <t>Dr Rahul Modi (36)</t>
+        </is>
+      </c>
+      <c r="E44" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F44" s="35" t="inlineStr">
+        <is>
+          <t>Tanmay Sharma (39)</t>
+        </is>
+      </c>
+      <c r="G44" s="31" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="35" t="inlineStr">
+        <is>
+          <t>11:54 AM</t>
+        </is>
+      </c>
+      <c r="B45" s="35" t="inlineStr">
         <is>
           <t>GA-2</t>
         </is>
       </c>
-      <c r="C37" s="8" t="inlineStr">
+      <c r="C45" s="35" t="inlineStr">
         <is>
           <t>GA</t>
         </is>
       </c>
-      <c r="D37" s="9" t="inlineStr">
-        <is>
-          <t>Shravan Gajera (23)</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="inlineStr">
+      <c r="D45" s="35" t="inlineStr">
+        <is>
+          <t>Ravi Modi (29)</t>
+        </is>
+      </c>
+      <c r="E45" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F45" s="35" t="inlineStr">
+        <is>
+          <t>Tejas doshi (40)</t>
+        </is>
+      </c>
+      <c r="G45" s="31" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="35" t="inlineStr">
+        <is>
+          <t>3:00 PM</t>
+        </is>
+      </c>
+      <c r="B46" s="35" t="inlineStr">
+        <is>
+          <t>GB-2</t>
+        </is>
+      </c>
+      <c r="C46" s="35" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="D46" s="35" t="inlineStr">
         <is>
           <t>Dr Rahul Modi (36)</t>
         </is>
       </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>9:42 AM</t>
-        </is>
-      </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>GB-1</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
+      <c r="E46" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F46" s="35" t="inlineStr">
+        <is>
+          <t>Vinit Padia (44)</t>
+        </is>
+      </c>
+      <c r="G46" s="31" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="35" t="inlineStr">
+        <is>
+          <t>3:18 PM</t>
+        </is>
+      </c>
+      <c r="B47" s="35" t="inlineStr">
+        <is>
+          <t>GA-3</t>
+        </is>
+      </c>
+      <c r="C47" s="35" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D47" s="35" t="inlineStr">
+        <is>
+          <t>Mayank Aggarwal (40)</t>
+        </is>
+      </c>
+      <c r="E47" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F47" s="35" t="inlineStr">
+        <is>
+          <t>Tejas doshi (40)</t>
+        </is>
+      </c>
+      <c r="G47" s="31" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="35" t="inlineStr">
+        <is>
+          <t>3:36 PM</t>
+        </is>
+      </c>
+      <c r="B48" s="35" t="inlineStr">
+        <is>
+          <t>GB-3</t>
+        </is>
+      </c>
+      <c r="C48" s="35" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>Aaditya Kumar (17)</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="inlineStr">
-        <is>
-          <t>Ravi Modi (29)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t>11:00 AM</t>
-        </is>
-      </c>
-      <c r="B39" s="8" t="inlineStr">
-        <is>
-          <t>U15-R1-M3</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>U15-R1</t>
-        </is>
-      </c>
-      <c r="D39" s="9" t="inlineStr">
-        <is>
-          <t>Viaan Neema (12)</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="inlineStr">
-        <is>
-          <t>Yash agarwal (13)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
-        <is>
-          <t>11:18 AM</t>
-        </is>
-      </c>
-      <c r="B40" s="8" t="inlineStr">
-        <is>
-          <t>GA-3</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>GA</t>
-        </is>
-      </c>
-      <c r="D40" s="9" t="inlineStr">
-        <is>
-          <t>Shravan Gajera (23)</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F40" s="9" t="inlineStr">
+      <c r="D48" s="35" t="inlineStr">
         <is>
           <t>Tanmay Sharma (39)</t>
         </is>
       </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
-        <is>
-          <t>11:36 AM</t>
-        </is>
-      </c>
-      <c r="B41" s="8" t="inlineStr">
-        <is>
-          <t>GB-2</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="D41" s="9" t="inlineStr">
-        <is>
-          <t>Aaditya Kumar (17)</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="inlineStr">
-        <is>
-          <t>Tejas doshi (40)</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
-        <is>
-          <t>11:54 AM</t>
-        </is>
-      </c>
-      <c r="B42" s="8" t="inlineStr">
-        <is>
-          <t>GA-4</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>GA</t>
-        </is>
-      </c>
-      <c r="D42" s="9" t="inlineStr">
-        <is>
-          <t>Shravan Gajera (23)</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="inlineStr">
-        <is>
-          <t>Mayank Aggarwal (40)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
-        <is>
-          <t>3:00 PM</t>
-        </is>
-      </c>
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>GB-3</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="D43" s="9" t="inlineStr">
-        <is>
-          <t>Aaditya Kumar (17)</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="inlineStr">
+      <c r="E48" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F48" s="35" t="inlineStr">
         <is>
           <t>Vinit Padia (44)</t>
         </is>
       </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
-        <is>
-          <t>3:18 PM</t>
-        </is>
-      </c>
-      <c r="B44" s="8" t="inlineStr">
-        <is>
-          <t>GA-5</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>GA</t>
-        </is>
-      </c>
-      <c r="D44" s="9" t="inlineStr">
-        <is>
-          <t>Hryday Goyal (20)</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="inlineStr">
-        <is>
-          <t>Dr Rahul Modi (36)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
-        <is>
-          <t>3:36 PM</t>
-        </is>
-      </c>
-      <c r="B45" s="8" t="inlineStr">
-        <is>
-          <t>GB-4</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="D45" s="9" t="inlineStr">
-        <is>
-          <t>Ravi Modi (29)</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="inlineStr">
-        <is>
-          <t>Tejas doshi (40)</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="G48" s="31" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="31" t="n"/>
+      <c r="B49" s="31" t="n"/>
+      <c r="C49" s="31" t="n"/>
+      <c r="D49" s="31" t="n"/>
+      <c r="E49" s="31" t="n"/>
+      <c r="F49" s="31" t="n"/>
+      <c r="G49" s="31" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="40" t="inlineStr">
+        <is>
+          <t>KNOCKOUTS - AUGUST 15</t>
+        </is>
+      </c>
+      <c r="B50" s="41" t="n"/>
+      <c r="C50" s="41" t="n"/>
+      <c r="D50" s="41" t="n"/>
+      <c r="E50" s="41" t="n"/>
+      <c r="F50" s="41" t="n"/>
+      <c r="G50" s="31" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="39" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="B51" s="39" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="C51" s="39" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D51" s="39" t="inlineStr">
+        <is>
+          <t>Player A</t>
+        </is>
+      </c>
+      <c r="E51" s="39" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F51" s="39" t="inlineStr">
+        <is>
+          <t>Player B</t>
+        </is>
+      </c>
+      <c r="G51" s="31" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="35" t="inlineStr">
         <is>
           <t>3:54 PM</t>
         </is>
       </c>
-      <c r="B46" s="8" t="inlineStr">
-        <is>
-          <t>GA-6</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>GA</t>
-        </is>
-      </c>
-      <c r="D46" s="9" t="inlineStr">
-        <is>
-          <t>Hryday Goyal (20)</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="inlineStr">
-        <is>
-          <t>Tanmay Sharma (39)</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="B52" s="35" t="inlineStr">
+        <is>
+          <t>U15-SF-1</t>
+        </is>
+      </c>
+      <c r="C52" s="35" t="inlineStr">
+        <is>
+          <t>U15-SF</t>
+        </is>
+      </c>
+      <c r="D52" s="35" t="inlineStr">
+        <is>
+          <t>Winner U15-R1-M1</t>
+        </is>
+      </c>
+      <c r="E52" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F52" s="35" t="inlineStr">
+        <is>
+          <t>Hridh jhala (BYE)</t>
+        </is>
+      </c>
+      <c r="G52" s="31" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="35" t="inlineStr">
         <is>
           <t>4:12 PM</t>
         </is>
       </c>
-      <c r="B47" s="8" t="inlineStr">
-        <is>
-          <t>GB-5</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="D47" s="9" t="inlineStr">
-        <is>
-          <t>Ravi Modi (29)</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="inlineStr">
-        <is>
-          <t>Vinit Padia (44)</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="B53" s="35" t="inlineStr">
+        <is>
+          <t>U15-SF-2</t>
+        </is>
+      </c>
+      <c r="C53" s="35" t="inlineStr">
+        <is>
+          <t>U15-SF</t>
+        </is>
+      </c>
+      <c r="D53" s="35" t="inlineStr">
+        <is>
+          <t>Winner U15-R1-M2</t>
+        </is>
+      </c>
+      <c r="E53" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F53" s="35" t="inlineStr">
+        <is>
+          <t>Winner U15-R1-M3</t>
+        </is>
+      </c>
+      <c r="G53" s="31" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="35" t="inlineStr">
         <is>
           <t>4:30 PM</t>
         </is>
       </c>
-      <c r="B48" s="8" t="inlineStr">
-        <is>
-          <t>GA-7</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>GA</t>
-        </is>
-      </c>
-      <c r="D48" s="9" t="inlineStr">
-        <is>
-          <t>Hryday Goyal (20)</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F48" s="9" t="inlineStr">
-        <is>
-          <t>Mayank Aggarwal (40)</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="B54" s="35" t="inlineStr">
+        <is>
+          <t>U25-FINAL</t>
+        </is>
+      </c>
+      <c r="C54" s="35" t="inlineStr">
+        <is>
+          <t>U25-F</t>
+        </is>
+      </c>
+      <c r="D54" s="35" t="inlineStr">
+        <is>
+          <t>U25 RR Winner</t>
+        </is>
+      </c>
+      <c r="E54" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F54" s="35" t="inlineStr">
+        <is>
+          <t>U25 RR Runner-up</t>
+        </is>
+      </c>
+      <c r="G54" s="31" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="35" t="inlineStr">
         <is>
           <t>4:48 PM</t>
         </is>
       </c>
-      <c r="B49" s="8" t="inlineStr">
-        <is>
-          <t>GB-6</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="D49" s="9" t="inlineStr">
-        <is>
-          <t>Tejas doshi (40)</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="inlineStr">
-        <is>
-          <t>Vinit Padia (44)</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="B55" s="35" t="inlineStr">
+        <is>
+          <t>U15-FINAL</t>
+        </is>
+      </c>
+      <c r="C55" s="35" t="inlineStr">
+        <is>
+          <t>U15-F</t>
+        </is>
+      </c>
+      <c r="D55" s="35" t="inlineStr">
+        <is>
+          <t>Winner U15-SF-1</t>
+        </is>
+      </c>
+      <c r="E55" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F55" s="35" t="inlineStr">
+        <is>
+          <t>Winner U15-SF-2</t>
+        </is>
+      </c>
+      <c r="G55" s="31" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="35" t="inlineStr">
         <is>
           <t>5:06 PM</t>
         </is>
       </c>
-      <c r="B50" s="8" t="inlineStr">
-        <is>
-          <t>GA-8</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>GA</t>
-        </is>
-      </c>
-      <c r="D50" s="9" t="inlineStr">
-        <is>
-          <t>Dr Rahul Modi (36)</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="inlineStr">
-        <is>
-          <t>Tanmay Sharma (39)</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="B56" s="35" t="inlineStr">
+        <is>
+          <t>A25-SF-1</t>
+        </is>
+      </c>
+      <c r="C56" s="35" t="inlineStr">
+        <is>
+          <t>A25-SF</t>
+        </is>
+      </c>
+      <c r="D56" s="35" t="inlineStr">
+        <is>
+          <t>GA Pool Winner</t>
+        </is>
+      </c>
+      <c r="E56" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F56" s="35" t="inlineStr">
+        <is>
+          <t>GB Pool 2nd</t>
+        </is>
+      </c>
+      <c r="G56" s="31" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="35" t="inlineStr">
         <is>
           <t>5:24 PM</t>
         </is>
       </c>
-      <c r="B51" s="8" t="inlineStr">
-        <is>
-          <t>GA-9</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>GA</t>
-        </is>
-      </c>
-      <c r="D51" s="9" t="inlineStr">
-        <is>
-          <t>Dr Rahul Modi (36)</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="inlineStr">
-        <is>
-          <t>Mayank Aggarwal (40)</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
-        <is>
-          <t>5:42 PM</t>
-        </is>
-      </c>
-      <c r="B52" s="8" t="inlineStr">
-        <is>
-          <t>GA-10</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>GA</t>
-        </is>
-      </c>
-      <c r="D52" s="9" t="inlineStr">
-        <is>
-          <t>Tanmay Sharma (39)</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="inlineStr">
-        <is>
-          <t>Mayank Aggarwal (40)</t>
-        </is>
-      </c>
-    </row>
-    <row r="53"/>
-    <row r="54">
-      <c r="A54" s="13" t="inlineStr">
-        <is>
-          <t>KNOCKOUTS - AUGUST 15</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="12" t="inlineStr">
+      <c r="B57" s="35" t="inlineStr">
+        <is>
+          <t>A25-SF-2</t>
+        </is>
+      </c>
+      <c r="C57" s="35" t="inlineStr">
+        <is>
+          <t>A25-SF</t>
+        </is>
+      </c>
+      <c r="D57" s="35" t="inlineStr">
+        <is>
+          <t>GB Pool Winner</t>
+        </is>
+      </c>
+      <c r="E57" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F57" s="35" t="inlineStr">
+        <is>
+          <t>GA Pool 2nd</t>
+        </is>
+      </c>
+      <c r="G57" s="31" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="31" t="n"/>
+      <c r="B58" s="31" t="n"/>
+      <c r="C58" s="31" t="n"/>
+      <c r="D58" s="31" t="n"/>
+      <c r="E58" s="31" t="n"/>
+      <c r="F58" s="31" t="n"/>
+      <c r="G58" s="31" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="38" t="inlineStr">
+        <is>
+          <t>AUGUST 16 - A25 FINAL</t>
+        </is>
+      </c>
+      <c r="B59" s="30" t="n"/>
+      <c r="C59" s="30" t="n"/>
+      <c r="D59" s="30" t="n"/>
+      <c r="E59" s="30" t="n"/>
+      <c r="F59" s="30" t="n"/>
+      <c r="G59" s="31" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="39" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B60" s="39" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
       </c>
-      <c r="C55" s="12" t="inlineStr">
+      <c r="C60" s="39" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D55" s="12" t="inlineStr">
+      <c r="D60" s="39" t="inlineStr">
         <is>
           <t>Player A</t>
         </is>
       </c>
-      <c r="E55" s="12" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F55" s="12" t="inlineStr">
+      <c r="E60" s="39" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F60" s="39" t="inlineStr">
         <is>
           <t>Player B</t>
         </is>
       </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
-        <is>
-          <t>6:30 PM</t>
-        </is>
-      </c>
-      <c r="B56" s="8" t="inlineStr">
-        <is>
-          <t>U15-SF-1</t>
-        </is>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>U15-SF</t>
-        </is>
-      </c>
-      <c r="D56" s="9" t="inlineStr">
-        <is>
-          <t>Winner U15-R1-M1</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F56" s="9" t="inlineStr">
-        <is>
-          <t>Hridh jhala (BYE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="inlineStr">
-        <is>
-          <t>6:48 PM</t>
-        </is>
-      </c>
-      <c r="B57" s="8" t="inlineStr">
-        <is>
-          <t>U15-SF-2</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>U15-SF</t>
-        </is>
-      </c>
-      <c r="D57" s="9" t="inlineStr">
-        <is>
-          <t>Winner U15-R1-M2</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="inlineStr">
-        <is>
-          <t>Winner U15-R1-M3</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="8" t="inlineStr">
-        <is>
-          <t>7:06 PM</t>
-        </is>
-      </c>
-      <c r="B58" s="8" t="inlineStr">
-        <is>
-          <t>A15-SF-1</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>A15-SF</t>
-        </is>
-      </c>
-      <c r="D58" s="9" t="inlineStr">
-        <is>
-          <t>GA Pool Winner</t>
-        </is>
-      </c>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F58" s="9" t="inlineStr">
-        <is>
-          <t>GB Pool Winner</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="8" t="inlineStr">
-        <is>
-          <t>7:24 PM</t>
-        </is>
-      </c>
-      <c r="B59" s="8" t="inlineStr">
-        <is>
-          <t>A15-SF-2</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="inlineStr">
-        <is>
-          <t>A15-SF</t>
-        </is>
-      </c>
-      <c r="D59" s="9" t="inlineStr">
-        <is>
-          <t>GA Pool 2nd</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F59" s="9" t="inlineStr">
-        <is>
-          <t>GB Pool 2nd</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="8" t="inlineStr">
-        <is>
-          <t>7:42 PM</t>
-        </is>
-      </c>
-      <c r="B60" s="8" t="inlineStr">
-        <is>
-          <t>U15-FINAL</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>U15-F</t>
-        </is>
-      </c>
-      <c r="D60" s="9" t="inlineStr">
-        <is>
-          <t>Winner U15-SF-1</t>
-        </is>
-      </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F60" s="9" t="inlineStr">
-        <is>
-          <t>Winner U15-SF-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="62"/>
+      <c r="G60" s="31" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="35" t="inlineStr">
+        <is>
+          <t>5:00 PM</t>
+        </is>
+      </c>
+      <c r="B61" s="35" t="inlineStr">
+        <is>
+          <t>A25-FINAL</t>
+        </is>
+      </c>
+      <c r="C61" s="35" t="inlineStr">
+        <is>
+          <t>A25-F</t>
+        </is>
+      </c>
+      <c r="D61" s="35" t="inlineStr">
+        <is>
+          <t>Winner A25-SF-1</t>
+        </is>
+      </c>
+      <c r="E61" s="35" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F61" s="35" t="inlineStr">
+        <is>
+          <t>Winner A25-SF-2</t>
+        </is>
+      </c>
+      <c r="G61" s="31" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="31" t="n"/>
+      <c r="B62" s="31" t="n"/>
+      <c r="C62" s="31" t="n"/>
+      <c r="D62" s="31" t="n"/>
+      <c r="E62" s="31" t="n"/>
+      <c r="F62" s="31" t="n"/>
+      <c r="G62" s="31" t="n"/>
+    </row>
     <row r="63">
-      <c r="A63" s="11" t="inlineStr">
-        <is>
-          <t>AUGUST 16 - A15 FINAL</t>
-        </is>
-      </c>
+      <c r="A63" s="31" t="n"/>
+      <c r="B63" s="31" t="n"/>
+      <c r="C63" s="31" t="n"/>
+      <c r="D63" s="31" t="n"/>
+      <c r="E63" s="31" t="n"/>
+      <c r="F63" s="31" t="n"/>
+      <c r="G63" s="31" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="12" t="inlineStr">
-        <is>
-          <t>Time</t>
-        </is>
-      </c>
-      <c r="B64" s="12" t="inlineStr">
-        <is>
-          <t>Match</t>
-        </is>
-      </c>
-      <c r="C64" s="12" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="D64" s="12" t="inlineStr">
-        <is>
-          <t>Player A</t>
-        </is>
-      </c>
-      <c r="E64" s="12" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F64" s="12" t="inlineStr">
-        <is>
-          <t>Player B</t>
-        </is>
-      </c>
+      <c r="A64" s="31" t="n"/>
+      <c r="B64" s="31" t="n"/>
+      <c r="C64" s="31" t="n"/>
+      <c r="D64" s="31" t="n"/>
+      <c r="E64" s="31" t="n"/>
+      <c r="F64" s="31" t="n"/>
+      <c r="G64" s="31" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="8" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
-      <c r="B65" s="8" t="inlineStr">
-        <is>
-          <t>A15-FINAL</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>A15-F</t>
-        </is>
-      </c>
-      <c r="D65" s="9" t="inlineStr">
-        <is>
-          <t>Winner A15-SF-1</t>
-        </is>
-      </c>
-      <c r="E65" s="8" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F65" s="9" t="inlineStr">
-        <is>
-          <t>Winner A15-SF-2</t>
-        </is>
-      </c>
+      <c r="A65" s="31" t="n"/>
+      <c r="B65" s="31" t="n"/>
+      <c r="C65" s="31" t="n"/>
+      <c r="D65" s="31" t="n"/>
+      <c r="E65" s="31" t="n"/>
+      <c r="F65" s="31" t="n"/>
+      <c r="G65" s="31" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="10">
+    <mergeCell ref="A33:F33"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A63:F63"/>
-    <mergeCell ref="A54:F54"/>
-    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A20:D20"/>
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A62:F62"/>
-    <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A53:F53"/>
-    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="A59:F59"/>
     <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A14:D14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add a hard 12-3pm break on Aug 16 to the schedule
No match of any kind is now scheduled between 12:00 PM and 3:00 PM on
Aug 16 - anything that would otherwise land there rolls to 3:00 PM.
Combined with the existing overnight closure and break-insertion
rules, tournament now finishes Aug 16, 5:00 PM (up from 2:05 PM).

Updates index.html's SEED_DATA and every sheet in
Ekta_Schedule_With_Matchups.xlsx to match; documents the new rule and
the Firestore re-sync requirement in CLAUDE.md.
</commit_message>
<xml_diff>
--- a/Ekta_Schedule_With_Matchups.xlsx
+++ b/Ekta_Schedule_With_Matchups.xlsx
@@ -795,32 +795,52 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>11:50 AM - 2:05 PM</t>
+          <t>11:50 AM - 12:00 PM</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Semis + Finals for every singles event, plus both Doubles events in full (TT Doubles, Carrom Doubles) — none of this starts until every group/pool match everywhere is done</t>
+          <t>Semis + Finals begin, plus both Doubles events in full (TT Doubles, Carrom Doubles) — none of this starts until every group/pool match everywhere is done</t>
         </is>
       </c>
       <c r="D10" s="4" t="n"/>
       <c r="E10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Aug 16</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>12:00 - 3:00 PM</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>BREAK</t>
+        </is>
+      </c>
       <c r="D11" s="10" t="n"/>
       <c r="E11" s="10" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>No matches are scheduled between 10:00 PM and 8:00 AM — any match that would otherwise land in that window rolls to 8:00 AM the next day.</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
+          <t>Aug 16</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>3:00 - 5:00 PM</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Semis + Finals + Doubles resume and wrap up</t>
+        </is>
+      </c>
       <c r="D12" s="4" t="n"/>
       <c r="E12" s="4" t="n"/>
     </row>
@@ -832,7 +852,11 @@
       <c r="E13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n"/>
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>No matches are scheduled between 10:00 PM and 8:00 AM, or between 12:00 PM and 3:00 PM on Aug 16 — any match that would otherwise land in those windows rolls to the end of the window.</t>
+        </is>
+      </c>
       <c r="B14" s="10" t="n"/>
       <c r="C14" s="10" t="n"/>
       <c r="D14" s="10" t="n"/>
@@ -907,7 +931,7 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Aug16 12:20PM</t>
+          <t>Aug16 3:15PM</t>
         </is>
       </c>
     </row>
@@ -932,7 +956,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Aug16 1:35PM</t>
+          <t>Aug16 4:30PM</t>
         </is>
       </c>
     </row>
@@ -952,12 +976,12 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Aug16 12:35PM</t>
+          <t>Aug16 3:30PM</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Aug16 2:05PM</t>
+          <t>Aug16 5:00PM</t>
         </is>
       </c>
     </row>
@@ -982,7 +1006,7 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Aug16 1:30PM</t>
+          <t>Aug16 4:20PM</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1031,7 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Aug16 1:30PM</t>
+          <t>Aug16 4:20PM</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1056,7 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Aug16 12:35PM</t>
+          <t>Aug16 3:30PM</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1106,7 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Aug16 1:20PM</t>
+          <t>Aug16 4:15PM</t>
         </is>
       </c>
     </row>
@@ -1107,14 +1131,14 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Aug16 1:56PM</t>
+          <t>Aug16 4:48PM</t>
         </is>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="19" t="inlineStr">
         <is>
-          <t>Overall tournament span: Aug 15, 8:00 AM start → Aug 16, 2:05 PM finish — comfortably inside the Aug 16, 10 PM cap.</t>
+          <t>Overall tournament span: Aug 15, 8:00 AM start → Aug 16, 5:00 PM finish — comfortably inside the Aug 16, 10 PM cap.</t>
         </is>
       </c>
     </row>
@@ -2289,12 +2313,12 @@
       </c>
       <c r="B44" s="28" t="inlineStr">
         <is>
-          <t>12:08PM</t>
+          <t>3:00PM</t>
         </is>
       </c>
       <c r="C44" s="28" t="inlineStr">
         <is>
-          <t>12:26PM</t>
+          <t>3:18PM</t>
         </is>
       </c>
       <c r="D44" s="28" t="inlineStr">
@@ -2339,12 +2363,12 @@
       </c>
       <c r="B45" s="27" t="inlineStr">
         <is>
-          <t>12:26PM</t>
+          <t>3:18PM</t>
         </is>
       </c>
       <c r="C45" s="27" t="inlineStr">
         <is>
-          <t>12:44PM</t>
+          <t>3:36PM</t>
         </is>
       </c>
       <c r="D45" s="27" t="inlineStr">
@@ -2389,12 +2413,12 @@
       </c>
       <c r="B46" s="28" t="inlineStr">
         <is>
-          <t>12:44PM</t>
+          <t>3:36PM</t>
         </is>
       </c>
       <c r="C46" s="28" t="inlineStr">
         <is>
-          <t>1:02PM</t>
+          <t>3:54PM</t>
         </is>
       </c>
       <c r="D46" s="28" t="inlineStr">
@@ -2439,12 +2463,12 @@
       </c>
       <c r="B47" s="27" t="inlineStr">
         <is>
-          <t>1:02PM</t>
+          <t>3:54PM</t>
         </is>
       </c>
       <c r="C47" s="27" t="inlineStr">
         <is>
-          <t>1:20PM</t>
+          <t>4:12PM</t>
         </is>
       </c>
       <c r="D47" s="27" t="inlineStr">
@@ -2489,12 +2513,12 @@
       </c>
       <c r="B48" s="28" t="inlineStr">
         <is>
-          <t>1:20PM</t>
+          <t>4:12PM</t>
         </is>
       </c>
       <c r="C48" s="28" t="inlineStr">
         <is>
-          <t>1:38PM</t>
+          <t>4:30PM</t>
         </is>
       </c>
       <c r="D48" s="28" t="inlineStr">
@@ -2539,12 +2563,12 @@
       </c>
       <c r="B49" s="27" t="inlineStr">
         <is>
-          <t>1:38PM</t>
+          <t>4:30PM</t>
         </is>
       </c>
       <c r="C49" s="27" t="inlineStr">
         <is>
-          <t>1:56PM</t>
+          <t>4:48PM</t>
         </is>
       </c>
       <c r="D49" s="27" t="inlineStr">
@@ -3498,12 +3522,12 @@
       </c>
       <c r="B30" s="27" t="inlineStr">
         <is>
-          <t>12:05PM</t>
+          <t>3:00PM</t>
         </is>
       </c>
       <c r="C30" s="27" t="inlineStr">
         <is>
-          <t>12:20PM</t>
+          <t>3:15PM</t>
         </is>
       </c>
       <c r="D30" s="27" t="inlineStr">
@@ -7091,12 +7115,12 @@
       </c>
       <c r="B105" s="27" t="inlineStr">
         <is>
-          <t>12:05PM</t>
+          <t>3:00PM</t>
         </is>
       </c>
       <c r="C105" s="27" t="inlineStr">
         <is>
-          <t>12:20PM</t>
+          <t>3:15PM</t>
         </is>
       </c>
       <c r="D105" s="27" t="inlineStr">
@@ -7141,12 +7165,12 @@
       </c>
       <c r="B106" s="28" t="inlineStr">
         <is>
-          <t>12:05PM</t>
+          <t>3:00PM</t>
         </is>
       </c>
       <c r="C106" s="28" t="inlineStr">
         <is>
-          <t>12:20PM</t>
+          <t>3:15PM</t>
         </is>
       </c>
       <c r="D106" s="28" t="inlineStr">
@@ -7191,12 +7215,12 @@
       </c>
       <c r="B107" s="27" t="inlineStr">
         <is>
-          <t>12:20PM</t>
+          <t>3:15PM</t>
         </is>
       </c>
       <c r="C107" s="27" t="inlineStr">
         <is>
-          <t>12:35PM</t>
+          <t>3:30PM</t>
         </is>
       </c>
       <c r="D107" s="27" t="inlineStr">
@@ -7241,12 +7265,12 @@
       </c>
       <c r="B108" s="28" t="inlineStr">
         <is>
-          <t>12:20PM</t>
+          <t>3:15PM</t>
         </is>
       </c>
       <c r="C108" s="28" t="inlineStr">
         <is>
-          <t>12:35PM</t>
+          <t>3:30PM</t>
         </is>
       </c>
       <c r="D108" s="28" t="inlineStr">
@@ -7291,12 +7315,12 @@
       </c>
       <c r="B109" s="27" t="inlineStr">
         <is>
-          <t>12:35PM</t>
+          <t>3:30PM</t>
         </is>
       </c>
       <c r="C109" s="27" t="inlineStr">
         <is>
-          <t>12:50PM</t>
+          <t>3:45PM</t>
         </is>
       </c>
       <c r="D109" s="27" t="inlineStr">
@@ -7341,12 +7365,12 @@
       </c>
       <c r="B110" s="28" t="inlineStr">
         <is>
-          <t>12:35PM</t>
+          <t>3:30PM</t>
         </is>
       </c>
       <c r="C110" s="28" t="inlineStr">
         <is>
-          <t>12:50PM</t>
+          <t>3:45PM</t>
         </is>
       </c>
       <c r="D110" s="28" t="inlineStr">
@@ -7391,12 +7415,12 @@
       </c>
       <c r="B111" s="27" t="inlineStr">
         <is>
-          <t>12:50PM</t>
+          <t>3:45PM</t>
         </is>
       </c>
       <c r="C111" s="27" t="inlineStr">
         <is>
-          <t>1:05PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="D111" s="27" t="inlineStr">
@@ -7441,12 +7465,12 @@
       </c>
       <c r="B112" s="28" t="inlineStr">
         <is>
-          <t>12:50PM</t>
+          <t>3:45PM</t>
         </is>
       </c>
       <c r="C112" s="28" t="inlineStr">
         <is>
-          <t>1:05PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="D112" s="28" t="inlineStr">
@@ -7491,12 +7515,12 @@
       </c>
       <c r="B113" s="27" t="inlineStr">
         <is>
-          <t>1:05PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="C113" s="27" t="inlineStr">
         <is>
-          <t>1:20PM</t>
+          <t>4:15PM</t>
         </is>
       </c>
       <c r="D113" s="27" t="inlineStr">
@@ -7541,12 +7565,12 @@
       </c>
       <c r="B114" s="28" t="inlineStr">
         <is>
-          <t>1:05PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="C114" s="28" t="inlineStr">
         <is>
-          <t>1:20PM</t>
+          <t>4:15PM</t>
         </is>
       </c>
       <c r="D114" s="28" t="inlineStr">
@@ -7591,12 +7615,12 @@
       </c>
       <c r="B115" s="27" t="inlineStr">
         <is>
-          <t>1:20PM</t>
+          <t>4:15PM</t>
         </is>
       </c>
       <c r="C115" s="27" t="inlineStr">
         <is>
-          <t>1:35PM</t>
+          <t>4:30PM</t>
         </is>
       </c>
       <c r="D115" s="27" t="inlineStr">
@@ -7865,12 +7889,12 @@
       </c>
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>12:35PM</t>
+          <t>3:30PM</t>
         </is>
       </c>
       <c r="C20" s="27" t="inlineStr">
         <is>
-          <t>12:50PM</t>
+          <t>3:45PM</t>
         </is>
       </c>
       <c r="D20" s="27" t="inlineStr">
@@ -7915,12 +7939,12 @@
       </c>
       <c r="B21" s="28" t="inlineStr">
         <is>
-          <t>12:50PM</t>
+          <t>3:45PM</t>
         </is>
       </c>
       <c r="C21" s="28" t="inlineStr">
         <is>
-          <t>1:05PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="D21" s="28" t="inlineStr">
@@ -7965,12 +7989,12 @@
       </c>
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>12:50PM</t>
+          <t>3:45PM</t>
         </is>
       </c>
       <c r="C22" s="27" t="inlineStr">
         <is>
-          <t>1:05PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="D22" s="27" t="inlineStr">
@@ -8015,12 +8039,12 @@
       </c>
       <c r="B23" s="28" t="inlineStr">
         <is>
-          <t>1:05PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="C23" s="28" t="inlineStr">
         <is>
-          <t>1:20PM</t>
+          <t>4:15PM</t>
         </is>
       </c>
       <c r="D23" s="28" t="inlineStr">
@@ -8065,12 +8089,12 @@
       </c>
       <c r="B24" s="27" t="inlineStr">
         <is>
-          <t>1:20PM</t>
+          <t>4:15PM</t>
         </is>
       </c>
       <c r="C24" s="27" t="inlineStr">
         <is>
-          <t>1:35PM</t>
+          <t>4:30PM</t>
         </is>
       </c>
       <c r="D24" s="27" t="inlineStr">
@@ -8115,12 +8139,12 @@
       </c>
       <c r="B25" s="28" t="inlineStr">
         <is>
-          <t>1:35PM</t>
+          <t>4:30PM</t>
         </is>
       </c>
       <c r="C25" s="28" t="inlineStr">
         <is>
-          <t>1:50PM</t>
+          <t>4:45PM</t>
         </is>
       </c>
       <c r="D25" s="28" t="inlineStr">
@@ -8165,12 +8189,12 @@
       </c>
       <c r="B26" s="27" t="inlineStr">
         <is>
-          <t>1:50PM</t>
+          <t>4:45PM</t>
         </is>
       </c>
       <c r="C26" s="27" t="inlineStr">
         <is>
-          <t>2:05PM</t>
+          <t>5:00PM</t>
         </is>
       </c>
       <c r="D26" s="27" t="inlineStr">
@@ -10996,12 +11020,12 @@
       </c>
       <c r="B79" s="27" t="inlineStr">
         <is>
-          <t>12:05PM</t>
+          <t>3:00PM</t>
         </is>
       </c>
       <c r="C79" s="27" t="inlineStr">
         <is>
-          <t>12:20PM</t>
+          <t>3:15PM</t>
         </is>
       </c>
       <c r="D79" s="27" t="inlineStr">
@@ -11046,12 +11070,12 @@
       </c>
       <c r="B80" s="28" t="inlineStr">
         <is>
-          <t>12:05PM</t>
+          <t>3:00PM</t>
         </is>
       </c>
       <c r="C80" s="28" t="inlineStr">
         <is>
-          <t>12:20PM</t>
+          <t>3:15PM</t>
         </is>
       </c>
       <c r="D80" s="28" t="inlineStr">
@@ -11096,12 +11120,12 @@
       </c>
       <c r="B81" s="27" t="inlineStr">
         <is>
-          <t>12:05PM</t>
+          <t>3:00PM</t>
         </is>
       </c>
       <c r="C81" s="27" t="inlineStr">
         <is>
-          <t>12:20PM</t>
+          <t>3:15PM</t>
         </is>
       </c>
       <c r="D81" s="27" t="inlineStr">
@@ -11146,12 +11170,12 @@
       </c>
       <c r="B82" s="28" t="inlineStr">
         <is>
-          <t>12:20PM</t>
+          <t>3:15PM</t>
         </is>
       </c>
       <c r="C82" s="28" t="inlineStr">
         <is>
-          <t>12:35PM</t>
+          <t>3:30PM</t>
         </is>
       </c>
       <c r="D82" s="28" t="inlineStr">
@@ -12374,12 +12398,12 @@
       </c>
       <c r="B31" s="28" t="inlineStr">
         <is>
-          <t>12:05PM</t>
+          <t>3:00PM</t>
         </is>
       </c>
       <c r="C31" s="28" t="inlineStr">
         <is>
-          <t>12:20PM</t>
+          <t>3:15PM</t>
         </is>
       </c>
       <c r="D31" s="28" t="inlineStr">
@@ -12424,12 +12448,12 @@
       </c>
       <c r="B32" s="27" t="inlineStr">
         <is>
-          <t>12:05PM</t>
+          <t>3:00PM</t>
         </is>
       </c>
       <c r="C32" s="27" t="inlineStr">
         <is>
-          <t>12:20PM</t>
+          <t>3:15PM</t>
         </is>
       </c>
       <c r="D32" s="27" t="inlineStr">
@@ -12474,12 +12498,12 @@
       </c>
       <c r="B33" s="28" t="inlineStr">
         <is>
-          <t>12:05PM</t>
+          <t>3:00PM</t>
         </is>
       </c>
       <c r="C33" s="28" t="inlineStr">
         <is>
-          <t>12:20PM</t>
+          <t>3:15PM</t>
         </is>
       </c>
       <c r="D33" s="28" t="inlineStr">
@@ -12524,12 +12548,12 @@
       </c>
       <c r="B34" s="27" t="inlineStr">
         <is>
-          <t>12:20PM</t>
+          <t>3:15PM</t>
         </is>
       </c>
       <c r="C34" s="27" t="inlineStr">
         <is>
-          <t>12:35PM</t>
+          <t>3:30PM</t>
         </is>
       </c>
       <c r="D34" s="27" t="inlineStr">
@@ -12574,12 +12598,12 @@
       </c>
       <c r="B35" s="28" t="inlineStr">
         <is>
-          <t>12:20PM</t>
+          <t>3:15PM</t>
         </is>
       </c>
       <c r="C35" s="28" t="inlineStr">
         <is>
-          <t>12:35PM</t>
+          <t>3:30PM</t>
         </is>
       </c>
       <c r="D35" s="28" t="inlineStr">
@@ -12624,12 +12648,12 @@
       </c>
       <c r="B36" s="27" t="inlineStr">
         <is>
-          <t>12:20PM</t>
+          <t>3:15PM</t>
         </is>
       </c>
       <c r="C36" s="27" t="inlineStr">
         <is>
-          <t>12:35PM</t>
+          <t>3:30PM</t>
         </is>
       </c>
       <c r="D36" s="27" t="inlineStr">
@@ -12674,12 +12698,12 @@
       </c>
       <c r="B37" s="28" t="inlineStr">
         <is>
-          <t>12:35PM</t>
+          <t>3:30PM</t>
         </is>
       </c>
       <c r="C37" s="28" t="inlineStr">
         <is>
-          <t>12:50PM</t>
+          <t>3:45PM</t>
         </is>
       </c>
       <c r="D37" s="28" t="inlineStr">
@@ -12724,12 +12748,12 @@
       </c>
       <c r="B38" s="27" t="inlineStr">
         <is>
-          <t>12:35PM</t>
+          <t>3:30PM</t>
         </is>
       </c>
       <c r="C38" s="27" t="inlineStr">
         <is>
-          <t>12:50PM</t>
+          <t>3:45PM</t>
         </is>
       </c>
       <c r="D38" s="27" t="inlineStr">
@@ -12774,12 +12798,12 @@
       </c>
       <c r="B39" s="28" t="inlineStr">
         <is>
-          <t>12:50PM</t>
+          <t>3:45PM</t>
         </is>
       </c>
       <c r="C39" s="28" t="inlineStr">
         <is>
-          <t>1:05PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="D39" s="28" t="inlineStr">
@@ -12824,12 +12848,12 @@
       </c>
       <c r="B40" s="27" t="inlineStr">
         <is>
-          <t>12:50PM</t>
+          <t>3:45PM</t>
         </is>
       </c>
       <c r="C40" s="27" t="inlineStr">
         <is>
-          <t>1:05PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="D40" s="27" t="inlineStr">
@@ -12874,12 +12898,12 @@
       </c>
       <c r="B41" s="28" t="inlineStr">
         <is>
-          <t>1:05PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="C41" s="28" t="inlineStr">
         <is>
-          <t>1:20PM</t>
+          <t>4:15PM</t>
         </is>
       </c>
       <c r="D41" s="28" t="inlineStr">
@@ -16047,12 +16071,12 @@
       </c>
       <c r="B86" s="27" t="inlineStr">
         <is>
-          <t>12:10PM</t>
+          <t>3:00PM</t>
         </is>
       </c>
       <c r="C86" s="27" t="inlineStr">
         <is>
-          <t>12:30PM</t>
+          <t>3:20PM</t>
         </is>
       </c>
       <c r="D86" s="27" t="inlineStr">
@@ -16097,12 +16121,12 @@
       </c>
       <c r="B87" s="28" t="inlineStr">
         <is>
-          <t>12:10PM</t>
+          <t>3:00PM</t>
         </is>
       </c>
       <c r="C87" s="28" t="inlineStr">
         <is>
-          <t>12:30PM</t>
+          <t>3:20PM</t>
         </is>
       </c>
       <c r="D87" s="28" t="inlineStr">
@@ -16147,12 +16171,12 @@
       </c>
       <c r="B88" s="27" t="inlineStr">
         <is>
-          <t>12:30PM</t>
+          <t>3:20PM</t>
         </is>
       </c>
       <c r="C88" s="27" t="inlineStr">
         <is>
-          <t>12:50PM</t>
+          <t>3:40PM</t>
         </is>
       </c>
       <c r="D88" s="27" t="inlineStr">
@@ -16197,12 +16221,12 @@
       </c>
       <c r="B89" s="28" t="inlineStr">
         <is>
-          <t>12:30PM</t>
+          <t>3:20PM</t>
         </is>
       </c>
       <c r="C89" s="28" t="inlineStr">
         <is>
-          <t>12:50PM</t>
+          <t>3:40PM</t>
         </is>
       </c>
       <c r="D89" s="28" t="inlineStr">
@@ -16247,12 +16271,12 @@
       </c>
       <c r="B90" s="27" t="inlineStr">
         <is>
-          <t>12:50PM</t>
+          <t>3:40PM</t>
         </is>
       </c>
       <c r="C90" s="27" t="inlineStr">
         <is>
-          <t>1:10PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="D90" s="27" t="inlineStr">
@@ -16297,12 +16321,12 @@
       </c>
       <c r="B91" s="28" t="inlineStr">
         <is>
-          <t>12:50PM</t>
+          <t>3:40PM</t>
         </is>
       </c>
       <c r="C91" s="28" t="inlineStr">
         <is>
-          <t>1:10PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="D91" s="28" t="inlineStr">
@@ -16347,12 +16371,12 @@
       </c>
       <c r="B92" s="27" t="inlineStr">
         <is>
-          <t>1:10PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="C92" s="27" t="inlineStr">
         <is>
-          <t>1:30PM</t>
+          <t>4:20PM</t>
         </is>
       </c>
       <c r="D92" s="27" t="inlineStr">
@@ -19773,12 +19797,12 @@
       </c>
       <c r="B97" s="27" t="inlineStr">
         <is>
-          <t>12:10PM</t>
+          <t>3:00PM</t>
         </is>
       </c>
       <c r="C97" s="27" t="inlineStr">
         <is>
-          <t>12:30PM</t>
+          <t>3:20PM</t>
         </is>
       </c>
       <c r="D97" s="27" t="inlineStr">
@@ -19823,12 +19847,12 @@
       </c>
       <c r="B98" s="28" t="inlineStr">
         <is>
-          <t>12:30PM</t>
+          <t>3:20PM</t>
         </is>
       </c>
       <c r="C98" s="28" t="inlineStr">
         <is>
-          <t>12:50PM</t>
+          <t>3:40PM</t>
         </is>
       </c>
       <c r="D98" s="28" t="inlineStr">
@@ -19873,12 +19897,12 @@
       </c>
       <c r="B99" s="27" t="inlineStr">
         <is>
-          <t>12:50PM</t>
+          <t>3:40PM</t>
         </is>
       </c>
       <c r="C99" s="27" t="inlineStr">
         <is>
-          <t>1:10PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="D99" s="27" t="inlineStr">
@@ -19923,12 +19947,12 @@
       </c>
       <c r="B100" s="28" t="inlineStr">
         <is>
-          <t>1:10PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="C100" s="28" t="inlineStr">
         <is>
-          <t>1:30PM</t>
+          <t>4:20PM</t>
         </is>
       </c>
       <c r="D100" s="28" t="inlineStr">

</xml_diff>

<commit_message>
Fix overlapping text in Overview sheet's Day Structure table
The Activity column's long descriptions weren't merged or wrapped, so
they overflowed past column C into the neighboring Day/Time cells of
adjacent rows, producing garbled overlapping text on mobile viewers.
Merge each Activity cell across C:G, enable text wrapping, and set
explicit row heights sized to the text length. Also fixes the
standalone closure-window note (row 14), which wasn't merged either.
</commit_message>
<xml_diff>
--- a/Ekta_Schedule_With_Matchups.xlsx
+++ b/Ekta_Schedule_With_Matchups.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -116,6 +116,11 @@
       <color rgb="FFCBD5E1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF64748B"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -165,7 +170,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -203,11 +208,55 @@
         <color rgb="FFCBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -314,6 +363,23 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -680,7 +746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="21" min="1" max="1"/>
@@ -746,103 +812,115 @@
           <t>Activity</t>
         </is>
       </c>
-      <c r="D7" s="17" t="n"/>
-      <c r="E7" s="17" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Aug 15</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="D7" s="37" t="n"/>
+      <c r="E7" s="37" t="n"/>
+      <c r="F7" s="37" t="n"/>
+      <c r="G7" s="38" t="n"/>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="39" t="inlineStr">
+        <is>
+          <t>Aug 15</t>
+        </is>
+      </c>
+      <c r="B8" s="39" t="inlineStr">
         <is>
           <t>8:00 AM - 9:00 PM</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="40" t="inlineStr">
         <is>
           <t>Group / pool ("Americano") stage for all 7 non-doubles events, running concurrently on their own tables/boards/court</t>
         </is>
       </c>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="D8" s="37" t="n"/>
+      <c r="E8" s="37" t="n"/>
+      <c r="F8" s="37" t="n"/>
+      <c r="G8" s="38" t="n"/>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="41" t="inlineStr">
         <is>
           <t>Aug 16</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="41" t="inlineStr">
         <is>
           <t>8:00 - 11:50 AM</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="42" t="inlineStr">
         <is>
           <t>Remaining group-stage matches (Chess, TT Men's Singles, Pool) wrap up — held over from Aug 15 by the player rest-break rule</t>
         </is>
       </c>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="D9" s="37" t="n"/>
+      <c r="E9" s="37" t="n"/>
+      <c r="F9" s="37" t="n"/>
+      <c r="G9" s="38" t="n"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="39" t="inlineStr">
         <is>
           <t>Aug 16</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="39" t="inlineStr">
         <is>
           <t>11:50 AM - 12:00 PM</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="40" t="inlineStr">
         <is>
           <t>Semis + Finals begin, plus both Doubles events in full (TT Doubles, Carrom Doubles) — none of this starts until every group/pool match everywhere is done</t>
         </is>
       </c>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="D10" s="37" t="n"/>
+      <c r="E10" s="37" t="n"/>
+      <c r="F10" s="37" t="n"/>
+      <c r="G10" s="38" t="n"/>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="41" t="inlineStr">
         <is>
           <t>Aug 16</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="41" t="inlineStr">
         <is>
           <t>12:00 - 3:00 PM</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="42" t="inlineStr">
         <is>
           <t>BREAK</t>
         </is>
       </c>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="D11" s="37" t="n"/>
+      <c r="E11" s="37" t="n"/>
+      <c r="F11" s="37" t="n"/>
+      <c r="G11" s="38" t="n"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="39" t="inlineStr">
         <is>
           <t>Aug 16</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="39" t="inlineStr">
         <is>
           <t>3:00 - 5:00 PM</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="40" t="inlineStr">
         <is>
           <t>Semis + Finals + Doubles resume and wrap up</t>
         </is>
       </c>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="n"/>
+      <c r="D12" s="37" t="n"/>
+      <c r="E12" s="37" t="n"/>
+      <c r="F12" s="37" t="n"/>
+      <c r="G12" s="38" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n"/>
@@ -851,16 +929,18 @@
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="6" t="n"/>
     </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="43" t="inlineStr">
         <is>
           <t>No matches are scheduled between 10:00 PM and 8:00 AM, or between 12:00 PM and 3:00 PM on Aug 16 — any match that would otherwise land in those windows rolls to the end of the window.</t>
         </is>
       </c>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
+      <c r="B14" s="37" t="n"/>
+      <c r="C14" s="37" t="n"/>
+      <c r="D14" s="37" t="n"/>
+      <c r="E14" s="37" t="n"/>
+      <c r="F14" s="37" t="n"/>
+      <c r="G14" s="38" t="n"/>
     </row>
     <row r="15" ht="33" customHeight="1">
       <c r="A15" s="6" t="n"/>
@@ -1157,15 +1237,22 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="17">
+    <mergeCell ref="C9:G9"/>
     <mergeCell ref="A34:E34"/>
+    <mergeCell ref="C7:G7"/>
     <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="C12:G12"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="C10:G10"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="A19:E19"/>
+    <mergeCell ref="C11:G11"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A31:E31"/>
     <mergeCell ref="A6:E6"/>
+    <mergeCell ref="C8:G8"/>
     <mergeCell ref="A17:E17"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>

</xml_diff>

<commit_message>
Decouple Doubles events from the all-groups-done gate
TT Doubles and Carrom Doubles no longer wait for every event's
group/pool stage to finish - they only need their own players free,
starting no earlier than 9:00 AM Aug 16 (per request, since both
events combined only take ~2h15m). Carrom Doubles now runs
9:00-10:30 AM and TT Doubles 9:45-11:15 AM, both done well before
league stage wraps up (~3:20 PM). Semis/finals for singles events
still wait for every group match everywhere to finish. Tournament
now finishes Aug 16, 5:26 PM.

Also fixes a fresh Overview-sheet corruption from this change: the
Day Structure table grew by a row for the new Doubles entry, and a
naive clear-and-rewrite collided with the fixed EVENTS section header
below it. Rebuilt via proper row insertion instead, and fixed stale
merged-cell ranges that openpyxl's insert_rows() left behind (which
had wiped Squash's Matches/Equipment/Starts/Finishes columns).
</commit_message>
<xml_diff>
--- a/Ekta_Schedule_With_Matchups.xlsx
+++ b/Ekta_Schedule_With_Matchups.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -130,8 +130,13 @@
       <color rgb="000F172A"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -176,6 +181,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000E7490"/>
       </patternFill>
     </fill>
   </fills>
@@ -265,7 +275,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -420,6 +430,13 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -785,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="21" min="1" max="1"/>
@@ -824,7 +841,7 @@
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>different events. Semis and finals (and both Doubles events, in full) run only after every group/pool match, in every event, has finished.</t>
+          <t>different events. Doubles events run once their own players are free (from 9:00 AM Aug 16); Semis and Finals for singles events wait until every group/pool match everywhere is finished.</t>
         </is>
       </c>
     </row>
@@ -982,7 +999,7 @@
       <c r="F13" s="37" t="n"/>
       <c r="G13" s="38" t="n"/>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="45" customHeight="1">
       <c r="A14" s="47" t="inlineStr">
         <is>
           <t>Aug 16</t>
@@ -990,29 +1007,29 @@
       </c>
       <c r="B14" s="51" t="inlineStr">
         <is>
+          <t>9:00 - 11:15 AM</t>
+        </is>
+      </c>
+      <c r="C14" s="52" t="inlineStr">
+        <is>
+          <t>Both Doubles events (TT Doubles, Carrom Doubles) run in full — only need their own players free, don't wait for other events' groups</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
+      <c r="A15" s="49" t="inlineStr">
+        <is>
+          <t>Aug 16</t>
+        </is>
+      </c>
+      <c r="B15" s="49" t="inlineStr">
+        <is>
           <t>12:00 - 3:00 PM</t>
         </is>
       </c>
-      <c r="C14" s="52" t="inlineStr">
+      <c r="C15" s="50" t="inlineStr">
         <is>
           <t>BREAK</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="49" t="inlineStr">
-        <is>
-          <t>Aug 16</t>
-        </is>
-      </c>
-      <c r="B15" s="49" t="inlineStr">
-        <is>
-          <t>3:00 - 3:20 PM</t>
-        </is>
-      </c>
-      <c r="C15" s="50" t="inlineStr">
-        <is>
-          <t>Remaining group-stage matches finish</t>
         </is>
       </c>
       <c r="D15" s="37" t="n"/>
@@ -1020,7 +1037,7 @@
       <c r="F15" s="37" t="n"/>
       <c r="G15" s="38" t="n"/>
     </row>
-    <row r="16" ht="60" customHeight="1">
+    <row r="16" ht="30" customHeight="1">
       <c r="A16" s="51" t="inlineStr">
         <is>
           <t>Aug 16</t>
@@ -1028,121 +1045,85 @@
       </c>
       <c r="B16" s="51" t="inlineStr">
         <is>
-          <t>3:20 - 5:35 PM</t>
+          <t>3:00 - 3:20 PM</t>
         </is>
       </c>
       <c r="C16" s="52" t="inlineStr">
         <is>
-          <t>Semis + Finals for every singles event, plus both Doubles events in full (TT Doubles, Carrom Doubles) — none of this starts until every group/pool match everywhere is done</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="27.95" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>Sports run concurrently on their own tables/boards/court and heavily share players, so each event's matches are spread across the day interleaved with other sports rather than run as one uninterrupted block. See each sport's own sheet for the exact chronological match list.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
+          <t>Remaining group-stage matches finish</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="51" t="inlineStr">
+        <is>
+          <t>Aug 16</t>
+        </is>
+      </c>
+      <c r="B17" s="51" t="inlineStr">
+        <is>
+          <t>3:20 - 5:26 PM</t>
+        </is>
+      </c>
+      <c r="C17" s="52" t="inlineStr">
+        <is>
+          <t>Semis + Finals for every singles event — starts only once every group/pool match everywhere is done</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
       <c r="A18" s="53" t="inlineStr">
         <is>
-          <t>No matches are scheduled before 8:00 AM, between 9:30-10:30 AM (Aug 15 flag hoisting), between 12:00-3:00 PM on either day, or after 10:00 PM — any match that would otherwise land in those windows rolls to the end of the window.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20.1" customHeight="1">
-      <c r="A19" s="16" t="inlineStr">
+          <t>No matches are scheduled before 8:00 AM, between 9:30-10:30 AM (Aug 15 flag hoisting), between 12:00-3:00 PM on either day, or after 10:00 PM — any match that would otherwise land in those windows rolls to the end of the window. Doubles events only need to wait for 9:00 AM Aug 16, not for other events' group stages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1"/>
+    <row r="20">
+      <c r="A20" s="55" t="inlineStr">
         <is>
           <t>EVENTS</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="54" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>Event</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Matches</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>Equipment</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Starts</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E22" s="9" t="inlineStr">
         <is>
           <t>Finishes</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>TT Women's Singles</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>2 tables</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Aug15 10:30AM</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>Aug16 3:50PM</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Table Tennis Singles Men</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="n">
-        <v>71</v>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>2 tables</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>Aug15 8:00AM</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>Aug16 5:05PM</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Table Tennis Doubles</t>
+          <t>TT Women's Singles</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
@@ -1151,23 +1132,23 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Aug16 4:05PM</t>
+          <t>Aug15 10:30AM</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Aug16 5:35PM</t>
+          <t>Aug16 3:50PM</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Pool</t>
+          <t>Table Tennis Singles Men</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
@@ -1181,47 +1162,47 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Aug16 5:00PM</t>
+          <t>Aug16 5:05PM</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Chess</t>
+          <t>Table Tennis Doubles</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>58</v>
+        <v>7</v>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>2 boards</t>
+          <t>2 tables</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Aug15 8:00AM</t>
+          <t>Aug16 9:45AM</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Aug16 5:00PM</t>
+          <t>Aug16 11:15AM</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Carrom Singles Men</t>
+          <t>Pool</t>
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>3 boards</t>
+          <t>2 tables</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -1231,22 +1212,22 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Aug16 4:05PM</t>
+          <t>Aug16 5:00PM</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Carrom Singles Women</t>
+          <t>Chess</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>11</v>
+        <v>58</v>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>3 boards (1 used)</t>
+          <t>2 boards</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1256,18 +1237,18 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Aug16 3:35PM</t>
+          <t>Aug16 5:00PM</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Carrom Doubles</t>
+          <t>Carrom Singles Men</t>
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
@@ -1276,68 +1257,120 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Aug16 3:20PM</t>
+          <t>Aug15 8:00AM</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Aug16 4:50PM</t>
+          <t>Aug16 4:05PM</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
+          <t>Carrom Singles Women</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>3 boards (1 used)</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Aug15 8:00AM</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Aug16 3:35PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Carrom Doubles</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>3 boards</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Aug16 9:00AM</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>Aug16 10:30AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
           <t>Squash</t>
         </is>
       </c>
-      <c r="B29" s="4" t="n">
+      <c r="B31" t="n">
         <v>19</v>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>1 court</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>Aug15 8:00AM</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Aug16 5:26PM</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="19" t="inlineStr">
-        <is>
-          <t>Overall tournament span: Aug 15, 8:00 AM start → Aug 16, 5:35 PM finish — comfortably inside the Aug 16, 10 PM cap.</t>
-        </is>
-      </c>
-    </row>
     <row r="33" ht="20.1" customHeight="1">
-      <c r="A33" s="16" t="inlineStr">
+      <c r="A33" s="19" t="inlineStr">
+        <is>
+          <t>Overall tournament span: Aug 15, 8:00 AM start → Aug 16, 5:26 PM finish — comfortably inside the Aug 16, 10 PM cap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1"/>
+    <row r="35">
+      <c r="A35" s="16" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1">
-      <c r="A34" s="20" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="20" t="inlineStr">
         <is>
           <t>Full match-by-match detail (exact times, table/board assignment, player groups) lives in each sport's own sheet — this tab is a summary only.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
-    <mergeCell ref="A34:E34"/>
+  <mergeCells count="22">
     <mergeCell ref="C15:G15"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="C14:G14"/>
+    <mergeCell ref="A36:E36"/>
     <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A19:G19"/>
     <mergeCell ref="C10:G10"/>
     <mergeCell ref="C16:G16"/>
     <mergeCell ref="C9:G9"/>
@@ -1347,12 +1380,12 @@
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="C11:G11"/>
     <mergeCell ref="C8:G8"/>
-    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="C17:G17"/>
     <mergeCell ref="C7:G7"/>
     <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A20:E20"/>
     <mergeCell ref="A18:G18"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A31:E31"/>
     <mergeCell ref="C13:G13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8075,12 +8108,12 @@
       </c>
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>4:05PM</t>
+          <t>9:45AM</t>
         </is>
       </c>
       <c r="C20" s="27" t="inlineStr">
         <is>
-          <t>4:20PM</t>
+          <t>10:00AM</t>
         </is>
       </c>
       <c r="D20" s="27" t="inlineStr">
@@ -8125,12 +8158,12 @@
       </c>
       <c r="B21" s="28" t="inlineStr">
         <is>
-          <t>4:20PM</t>
+          <t>10:00AM</t>
         </is>
       </c>
       <c r="C21" s="28" t="inlineStr">
         <is>
-          <t>4:35PM</t>
+          <t>10:15AM</t>
         </is>
       </c>
       <c r="D21" s="28" t="inlineStr">
@@ -8175,12 +8208,12 @@
       </c>
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>4:20PM</t>
+          <t>10:00AM</t>
         </is>
       </c>
       <c r="C22" s="27" t="inlineStr">
         <is>
-          <t>4:35PM</t>
+          <t>10:15AM</t>
         </is>
       </c>
       <c r="D22" s="27" t="inlineStr">
@@ -8225,12 +8258,12 @@
       </c>
       <c r="B23" s="28" t="inlineStr">
         <is>
-          <t>4:35PM</t>
+          <t>10:15AM</t>
         </is>
       </c>
       <c r="C23" s="28" t="inlineStr">
         <is>
-          <t>4:50PM</t>
+          <t>10:30AM</t>
         </is>
       </c>
       <c r="D23" s="28" t="inlineStr">
@@ -8275,12 +8308,12 @@
       </c>
       <c r="B24" s="27" t="inlineStr">
         <is>
-          <t>4:50PM</t>
+          <t>10:30AM</t>
         </is>
       </c>
       <c r="C24" s="27" t="inlineStr">
         <is>
-          <t>5:05PM</t>
+          <t>10:45AM</t>
         </is>
       </c>
       <c r="D24" s="27" t="inlineStr">
@@ -8325,12 +8358,12 @@
       </c>
       <c r="B25" s="28" t="inlineStr">
         <is>
-          <t>5:05PM</t>
+          <t>10:45AM</t>
         </is>
       </c>
       <c r="C25" s="28" t="inlineStr">
         <is>
-          <t>5:20PM</t>
+          <t>11:00AM</t>
         </is>
       </c>
       <c r="D25" s="28" t="inlineStr">
@@ -8375,12 +8408,12 @@
       </c>
       <c r="B26" s="27" t="inlineStr">
         <is>
-          <t>5:20PM</t>
+          <t>11:00AM</t>
         </is>
       </c>
       <c r="C26" s="27" t="inlineStr">
         <is>
-          <t>5:35PM</t>
+          <t>11:15AM</t>
         </is>
       </c>
       <c r="D26" s="27" t="inlineStr">
@@ -12434,12 +12467,12 @@
       </c>
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>3:20PM</t>
+          <t>9:00AM</t>
         </is>
       </c>
       <c r="C28" s="27" t="inlineStr">
         <is>
-          <t>3:35PM</t>
+          <t>9:15AM</t>
         </is>
       </c>
       <c r="D28" s="27" t="inlineStr">
@@ -12484,12 +12517,12 @@
       </c>
       <c r="B29" s="28" t="inlineStr">
         <is>
-          <t>3:20PM</t>
+          <t>9:00AM</t>
         </is>
       </c>
       <c r="C29" s="28" t="inlineStr">
         <is>
-          <t>3:35PM</t>
+          <t>9:15AM</t>
         </is>
       </c>
       <c r="D29" s="28" t="inlineStr">
@@ -12534,12 +12567,12 @@
       </c>
       <c r="B30" s="27" t="inlineStr">
         <is>
-          <t>3:20PM</t>
+          <t>9:00AM</t>
         </is>
       </c>
       <c r="C30" s="27" t="inlineStr">
         <is>
-          <t>3:35PM</t>
+          <t>9:15AM</t>
         </is>
       </c>
       <c r="D30" s="27" t="inlineStr">
@@ -12584,12 +12617,12 @@
       </c>
       <c r="B31" s="28" t="inlineStr">
         <is>
-          <t>3:35PM</t>
+          <t>9:15AM</t>
         </is>
       </c>
       <c r="C31" s="28" t="inlineStr">
         <is>
-          <t>3:50PM</t>
+          <t>9:30AM</t>
         </is>
       </c>
       <c r="D31" s="28" t="inlineStr">
@@ -12634,12 +12667,12 @@
       </c>
       <c r="B32" s="27" t="inlineStr">
         <is>
-          <t>3:35PM</t>
+          <t>9:15AM</t>
         </is>
       </c>
       <c r="C32" s="27" t="inlineStr">
         <is>
-          <t>3:50PM</t>
+          <t>9:30AM</t>
         </is>
       </c>
       <c r="D32" s="27" t="inlineStr">
@@ -12684,12 +12717,12 @@
       </c>
       <c r="B33" s="28" t="inlineStr">
         <is>
-          <t>3:35PM</t>
+          <t>9:15AM</t>
         </is>
       </c>
       <c r="C33" s="28" t="inlineStr">
         <is>
-          <t>3:50PM</t>
+          <t>9:30AM</t>
         </is>
       </c>
       <c r="D33" s="28" t="inlineStr">
@@ -12734,12 +12767,12 @@
       </c>
       <c r="B34" s="27" t="inlineStr">
         <is>
-          <t>3:50PM</t>
+          <t>9:30AM</t>
         </is>
       </c>
       <c r="C34" s="27" t="inlineStr">
         <is>
-          <t>4:05PM</t>
+          <t>9:45AM</t>
         </is>
       </c>
       <c r="D34" s="27" t="inlineStr">
@@ -12784,12 +12817,12 @@
       </c>
       <c r="B35" s="28" t="inlineStr">
         <is>
-          <t>3:50PM</t>
+          <t>9:30AM</t>
         </is>
       </c>
       <c r="C35" s="28" t="inlineStr">
         <is>
-          <t>4:05PM</t>
+          <t>9:45AM</t>
         </is>
       </c>
       <c r="D35" s="28" t="inlineStr">
@@ -12834,12 +12867,12 @@
       </c>
       <c r="B36" s="27" t="inlineStr">
         <is>
-          <t>3:50PM</t>
+          <t>9:30AM</t>
         </is>
       </c>
       <c r="C36" s="27" t="inlineStr">
         <is>
-          <t>4:05PM</t>
+          <t>9:45AM</t>
         </is>
       </c>
       <c r="D36" s="27" t="inlineStr">
@@ -12884,12 +12917,12 @@
       </c>
       <c r="B37" s="28" t="inlineStr">
         <is>
-          <t>4:05PM</t>
+          <t>9:45AM</t>
         </is>
       </c>
       <c r="C37" s="28" t="inlineStr">
         <is>
-          <t>4:20PM</t>
+          <t>10:00AM</t>
         </is>
       </c>
       <c r="D37" s="28" t="inlineStr">
@@ -12934,12 +12967,12 @@
       </c>
       <c r="B38" s="27" t="inlineStr">
         <is>
-          <t>4:05PM</t>
+          <t>9:45AM</t>
         </is>
       </c>
       <c r="C38" s="27" t="inlineStr">
         <is>
-          <t>4:20PM</t>
+          <t>10:00AM</t>
         </is>
       </c>
       <c r="D38" s="27" t="inlineStr">
@@ -12984,12 +13017,12 @@
       </c>
       <c r="B39" s="28" t="inlineStr">
         <is>
-          <t>4:20PM</t>
+          <t>10:00AM</t>
         </is>
       </c>
       <c r="C39" s="28" t="inlineStr">
         <is>
-          <t>4:35PM</t>
+          <t>10:15AM</t>
         </is>
       </c>
       <c r="D39" s="28" t="inlineStr">
@@ -13034,12 +13067,12 @@
       </c>
       <c r="B40" s="27" t="inlineStr">
         <is>
-          <t>4:20PM</t>
+          <t>10:00AM</t>
         </is>
       </c>
       <c r="C40" s="27" t="inlineStr">
         <is>
-          <t>4:35PM</t>
+          <t>10:15AM</t>
         </is>
       </c>
       <c r="D40" s="27" t="inlineStr">
@@ -13084,12 +13117,12 @@
       </c>
       <c r="B41" s="28" t="inlineStr">
         <is>
-          <t>4:35PM</t>
+          <t>10:15AM</t>
         </is>
       </c>
       <c r="C41" s="28" t="inlineStr">
         <is>
-          <t>4:50PM</t>
+          <t>10:30AM</t>
         </is>
       </c>
       <c r="D41" s="28" t="inlineStr">

</xml_diff>

<commit_message>
Add Trophies & Medals sheet to the schedule workbook
New "Trophies & Medals" tab: trophy count (22 finals across all 9
events -> 22 big + 22 small trophies, with per-event breakdown), plus
Under-16 medal planning (14 unique U16 players, their category
memberships, the categories that are tightest bottlenecks for them,
and the 3-14 best/worst-case medal count range depending on results).

Excel-only, per the established pattern for this thread of requests -
index.html untouched.
</commit_message>
<xml_diff>
--- a/Ekta_Schedule_With_Matchups.xlsx
+++ b/Ekta_Schedule_With_Matchups.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Pool" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Chess" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Squash" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Trophies &amp; Medals" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -155,6 +156,11 @@
       <color rgb="000F172A"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00B45309"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -219,7 +225,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -301,11 +307,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <right/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -495,6 +539,52 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -877,15 +967,11 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="57" t="inlineStr">
+      <c r="A1" s="68" t="inlineStr">
         <is>
           <t>EKTA GAMES 2026 — SCHEDULE OVERVIEW</t>
         </is>
       </c>
-      <c r="B1" s="58" t="n"/>
-      <c r="C1" s="58" t="n"/>
-      <c r="D1" s="58" t="n"/>
-      <c r="E1" s="58" t="n"/>
       <c r="F1" s="31" t="n"/>
       <c r="G1" s="31" t="n"/>
       <c r="H1" s="31" t="n"/>
@@ -893,15 +979,11 @@
       <c r="J1" s="31" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="59" t="inlineStr">
+      <c r="A2" s="69" t="inlineStr">
         <is>
           <t>Fully conflict-free: no player is ever double-booked, TT tables are shared across TT Women's/Men's/Doubles</t>
         </is>
       </c>
-      <c r="B2" s="58" t="n"/>
-      <c r="C2" s="58" t="n"/>
-      <c r="D2" s="58" t="n"/>
-      <c r="E2" s="58" t="n"/>
       <c r="F2" s="31" t="n"/>
       <c r="G2" s="31" t="n"/>
       <c r="H2" s="31" t="n"/>
@@ -909,15 +991,11 @@
       <c r="J2" s="31" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="59" t="inlineStr">
+      <c r="A3" s="69" t="inlineStr">
         <is>
           <t>and Carrom boards across Carrom Men's/Women's/Doubles, and a 10-minute break is inserted whenever a player</t>
         </is>
       </c>
-      <c r="B3" s="58" t="n"/>
-      <c r="C3" s="58" t="n"/>
-      <c r="D3" s="58" t="n"/>
-      <c r="E3" s="58" t="n"/>
       <c r="F3" s="31" t="n"/>
       <c r="G3" s="31" t="n"/>
       <c r="H3" s="31" t="n"/>
@@ -925,15 +1003,11 @@
       <c r="J3" s="31" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="59" t="inlineStr">
+      <c r="A4" s="69" t="inlineStr">
         <is>
           <t>would otherwise play back-to-back in the same event or continuously for 60+ minutes across different events.</t>
         </is>
       </c>
-      <c r="B4" s="58" t="n"/>
-      <c r="C4" s="58" t="n"/>
-      <c r="D4" s="58" t="n"/>
-      <c r="E4" s="58" t="n"/>
       <c r="F4" s="31" t="n"/>
       <c r="G4" s="31" t="n"/>
       <c r="H4" s="31" t="n"/>
@@ -941,15 +1015,11 @@
       <c r="J4" s="31" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="59" t="inlineStr">
+      <c r="A5" s="69" t="inlineStr">
         <is>
           <t>Carrom Women's Singles, TT Women's Singles, Pool, and Squash's Under 15 + 15-25 Bracket knockouts each follow</t>
         </is>
       </c>
-      <c r="B5" s="58" t="n"/>
-      <c r="C5" s="58" t="n"/>
-      <c r="D5" s="58" t="n"/>
-      <c r="E5" s="58" t="n"/>
       <c r="F5" s="31" t="n"/>
       <c r="G5" s="31" t="n"/>
       <c r="H5" s="31" t="n"/>
@@ -957,15 +1027,11 @@
       <c r="J5" s="31" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="59" t="inlineStr">
+      <c r="A6" s="69" t="inlineStr">
         <is>
           <t>immediately once that event's own league stage is done. Carrom Men's, TT Men's, Chess, and Squash's Above 25</t>
         </is>
       </c>
-      <c r="B6" s="58" t="n"/>
-      <c r="C6" s="58" t="n"/>
-      <c r="D6" s="58" t="n"/>
-      <c r="E6" s="58" t="n"/>
       <c r="F6" s="31" t="n"/>
       <c r="G6" s="31" t="n"/>
       <c r="H6" s="31" t="n"/>
@@ -973,15 +1039,11 @@
       <c r="J6" s="31" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="59" t="inlineStr">
+      <c r="A7" s="69" t="inlineStr">
         <is>
           <t>Bracket knockouts, plus both entire Doubles events (from 9:00 AM Aug 16), wait for their own gating rule.</t>
         </is>
       </c>
-      <c r="B7" s="58" t="n"/>
-      <c r="C7" s="58" t="n"/>
-      <c r="D7" s="58" t="n"/>
-      <c r="E7" s="58" t="n"/>
       <c r="F7" s="31" t="n"/>
       <c r="G7" s="31" t="n"/>
       <c r="H7" s="31" t="n"/>
@@ -1001,15 +1063,11 @@
       <c r="J8" s="31" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="60" t="inlineStr">
+      <c r="A9" s="70" t="inlineStr">
         <is>
           <t>DAY STRUCTURE</t>
         </is>
       </c>
-      <c r="B9" s="56" t="n"/>
-      <c r="C9" s="56" t="n"/>
-      <c r="D9" s="56" t="n"/>
-      <c r="E9" s="56" t="n"/>
       <c r="F9" s="31" t="n"/>
       <c r="G9" s="31" t="n"/>
       <c r="H9" s="31" t="n"/>
@@ -1027,15 +1085,11 @@
           <t>Time</t>
         </is>
       </c>
-      <c r="C10" s="61" t="inlineStr">
+      <c r="C10" s="71" t="inlineStr">
         <is>
           <t>Activity</t>
         </is>
       </c>
-      <c r="D10" s="62" t="n"/>
-      <c r="E10" s="62" t="n"/>
-      <c r="F10" s="62" t="n"/>
-      <c r="G10" s="62" t="n"/>
       <c r="H10" s="31" t="n"/>
       <c r="I10" s="31" t="n"/>
       <c r="J10" s="31" t="n"/>
@@ -1243,15 +1297,11 @@
       <c r="J21" s="31" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="60" t="inlineStr">
+      <c r="A22" s="70" t="inlineStr">
         <is>
           <t>EVENTS</t>
         </is>
       </c>
-      <c r="B22" s="56" t="n"/>
-      <c r="C22" s="56" t="n"/>
-      <c r="D22" s="56" t="n"/>
-      <c r="E22" s="56" t="n"/>
       <c r="F22" s="31" t="n"/>
       <c r="G22" s="31" t="n"/>
       <c r="H22" s="31" t="n"/>
@@ -1597,15 +1647,11 @@
       <c r="J35" s="31" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="60" t="inlineStr">
+      <c r="A36" s="70" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
       </c>
-      <c r="B36" s="56" t="n"/>
-      <c r="C36" s="56" t="n"/>
-      <c r="D36" s="56" t="n"/>
-      <c r="E36" s="56" t="n"/>
       <c r="F36" s="31" t="n"/>
       <c r="G36" s="31" t="n"/>
       <c r="H36" s="31" t="n"/>
@@ -3378,6 +3424,1251 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G71"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="72" t="inlineStr">
+        <is>
+          <t>TROPHIES &amp; MEDALS</t>
+        </is>
+      </c>
+      <c r="B1" s="58" t="n"/>
+      <c r="C1" s="58" t="n"/>
+      <c r="D1" s="58" t="n"/>
+      <c r="E1" s="58" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="73" t="inlineStr">
+        <is>
+          <t>Every final's winner gets a big trophy, runner-up gets a small trophy. Under-16 players who don't reach any final they're entered in get a medal.</t>
+        </is>
+      </c>
+      <c r="B2" s="58" t="n"/>
+      <c r="C2" s="58" t="n"/>
+      <c r="D2" s="58" t="n"/>
+      <c r="E2" s="58" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="55" t="inlineStr">
+        <is>
+          <t>TROPHY COUNT</t>
+        </is>
+      </c>
+      <c r="B4" s="56" t="n"/>
+      <c r="C4" s="56" t="n"/>
+      <c r="D4" s="56" t="n"/>
+      <c r="E4" s="56" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="74" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="B5" s="74" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C5" s="74" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="D5" s="74" t="inlineStr">
+        <is>
+          <t>Big Trophy (Winner)</t>
+        </is>
+      </c>
+      <c r="E5" s="74" t="inlineStr">
+        <is>
+          <t>Small Trophy (Runner-up)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="75" t="inlineStr">
+        <is>
+          <t>TT — Women's Singles</t>
+        </is>
+      </c>
+      <c r="B6" s="75" t="inlineStr">
+        <is>
+          <t>(single category)</t>
+        </is>
+      </c>
+      <c r="C6" s="75" t="inlineStr">
+        <is>
+          <t>FINAL</t>
+        </is>
+      </c>
+      <c r="D6" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="75" t="inlineStr">
+        <is>
+          <t>TT — Men's Singles</t>
+        </is>
+      </c>
+      <c r="B7" s="75" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="C7" s="75" t="inlineStr">
+        <is>
+          <t>SR-FINAL</t>
+        </is>
+      </c>
+      <c r="D7" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="75" t="inlineStr">
+        <is>
+          <t>TT — Men's Singles</t>
+        </is>
+      </c>
+      <c r="B8" s="75" t="inlineStr">
+        <is>
+          <t>Under 15</t>
+        </is>
+      </c>
+      <c r="C8" s="75" t="inlineStr">
+        <is>
+          <t>U15-FINAL</t>
+        </is>
+      </c>
+      <c r="D8" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="75" t="inlineStr">
+        <is>
+          <t>TT — Men's Singles</t>
+        </is>
+      </c>
+      <c r="B9" s="75" t="inlineStr">
+        <is>
+          <t>Under 32</t>
+        </is>
+      </c>
+      <c r="C9" s="75" t="inlineStr">
+        <is>
+          <t>U32-FINAL</t>
+        </is>
+      </c>
+      <c r="D9" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="75" t="inlineStr">
+        <is>
+          <t>TT — Men's Singles</t>
+        </is>
+      </c>
+      <c r="B10" s="75" t="inlineStr">
+        <is>
+          <t>Under 36</t>
+        </is>
+      </c>
+      <c r="C10" s="75" t="inlineStr">
+        <is>
+          <t>U36-FINAL</t>
+        </is>
+      </c>
+      <c r="D10" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="75" t="inlineStr">
+        <is>
+          <t>TT — Men's Singles</t>
+        </is>
+      </c>
+      <c r="B11" s="75" t="inlineStr">
+        <is>
+          <t>Under 46</t>
+        </is>
+      </c>
+      <c r="C11" s="75" t="inlineStr">
+        <is>
+          <t>U46-FINAL</t>
+        </is>
+      </c>
+      <c r="D11" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="75" t="inlineStr">
+        <is>
+          <t>TT — Doubles</t>
+        </is>
+      </c>
+      <c r="B12" s="75" t="inlineStr">
+        <is>
+          <t>(single category)</t>
+        </is>
+      </c>
+      <c r="C12" s="75" t="inlineStr">
+        <is>
+          <t>FINAL</t>
+        </is>
+      </c>
+      <c r="D12" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="75" t="inlineStr">
+        <is>
+          <t>Carrom — Women's Singles</t>
+        </is>
+      </c>
+      <c r="B13" s="75" t="inlineStr">
+        <is>
+          <t>(single category)</t>
+        </is>
+      </c>
+      <c r="C13" s="75" t="inlineStr">
+        <is>
+          <t>CW-FINAL</t>
+        </is>
+      </c>
+      <c r="D13" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="75" t="inlineStr">
+        <is>
+          <t>Carrom — Men's Singles</t>
+        </is>
+      </c>
+      <c r="B14" s="75" t="inlineStr">
+        <is>
+          <t>Above 46</t>
+        </is>
+      </c>
+      <c r="C14" s="75" t="inlineStr">
+        <is>
+          <t>A46-FINAL</t>
+        </is>
+      </c>
+      <c r="D14" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="75" t="inlineStr">
+        <is>
+          <t>Carrom — Men's Singles</t>
+        </is>
+      </c>
+      <c r="B15" s="75" t="inlineStr">
+        <is>
+          <t>Under 15</t>
+        </is>
+      </c>
+      <c r="C15" s="75" t="inlineStr">
+        <is>
+          <t>U15-FINAL</t>
+        </is>
+      </c>
+      <c r="D15" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="75" t="inlineStr">
+        <is>
+          <t>Carrom — Men's Singles</t>
+        </is>
+      </c>
+      <c r="B16" s="75" t="inlineStr">
+        <is>
+          <t>Under 46</t>
+        </is>
+      </c>
+      <c r="C16" s="75" t="inlineStr">
+        <is>
+          <t>U46-FINAL</t>
+        </is>
+      </c>
+      <c r="D16" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="75" t="inlineStr">
+        <is>
+          <t>Carrom — Doubles</t>
+        </is>
+      </c>
+      <c r="B17" s="75" t="inlineStr">
+        <is>
+          <t>(single category)</t>
+        </is>
+      </c>
+      <c r="C17" s="75" t="inlineStr">
+        <is>
+          <t>FINAL</t>
+        </is>
+      </c>
+      <c r="D17" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="75" t="inlineStr">
+        <is>
+          <t>Pool</t>
+        </is>
+      </c>
+      <c r="B18" s="75" t="inlineStr">
+        <is>
+          <t>26 to 39</t>
+        </is>
+      </c>
+      <c r="C18" s="75" t="inlineStr">
+        <is>
+          <t>2639-FINAL</t>
+        </is>
+      </c>
+      <c r="D18" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="75" t="inlineStr">
+        <is>
+          <t>Pool</t>
+        </is>
+      </c>
+      <c r="B19" s="75" t="inlineStr">
+        <is>
+          <t>40 and above</t>
+        </is>
+      </c>
+      <c r="C19" s="75" t="inlineStr">
+        <is>
+          <t>40P-FINAL</t>
+        </is>
+      </c>
+      <c r="D19" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="75" t="inlineStr">
+        <is>
+          <t>Pool</t>
+        </is>
+      </c>
+      <c r="B20" s="75" t="inlineStr">
+        <is>
+          <t>Under 26</t>
+        </is>
+      </c>
+      <c r="C20" s="75" t="inlineStr">
+        <is>
+          <t>U26-FINAL</t>
+        </is>
+      </c>
+      <c r="D20" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="75" t="inlineStr">
+        <is>
+          <t>Chess</t>
+        </is>
+      </c>
+      <c r="B21" s="75" t="inlineStr">
+        <is>
+          <t>12 to 20</t>
+        </is>
+      </c>
+      <c r="C21" s="75" t="inlineStr">
+        <is>
+          <t>1220-FINAL</t>
+        </is>
+      </c>
+      <c r="D21" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="75" t="inlineStr">
+        <is>
+          <t>Chess</t>
+        </is>
+      </c>
+      <c r="B22" s="75" t="inlineStr">
+        <is>
+          <t>21 to 40</t>
+        </is>
+      </c>
+      <c r="C22" s="75" t="inlineStr">
+        <is>
+          <t>2140-FINAL</t>
+        </is>
+      </c>
+      <c r="D22" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="75" t="inlineStr">
+        <is>
+          <t>Chess</t>
+        </is>
+      </c>
+      <c r="B23" s="75" t="inlineStr">
+        <is>
+          <t>41 and above</t>
+        </is>
+      </c>
+      <c r="C23" s="75" t="inlineStr">
+        <is>
+          <t>41P-FINAL</t>
+        </is>
+      </c>
+      <c r="D23" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="75" t="inlineStr">
+        <is>
+          <t>Chess</t>
+        </is>
+      </c>
+      <c r="B24" s="75" t="inlineStr">
+        <is>
+          <t>Under 11</t>
+        </is>
+      </c>
+      <c r="C24" s="75" t="inlineStr">
+        <is>
+          <t>U11-FINAL</t>
+        </is>
+      </c>
+      <c r="D24" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="75" t="inlineStr">
+        <is>
+          <t>Squash</t>
+        </is>
+      </c>
+      <c r="B25" s="75" t="inlineStr">
+        <is>
+          <t>15-25 Bracket</t>
+        </is>
+      </c>
+      <c r="C25" s="75" t="inlineStr">
+        <is>
+          <t>GC-FINAL</t>
+        </is>
+      </c>
+      <c r="D25" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="75" t="inlineStr">
+        <is>
+          <t>Squash</t>
+        </is>
+      </c>
+      <c r="B26" s="75" t="inlineStr">
+        <is>
+          <t>Above 25 Bracket</t>
+        </is>
+      </c>
+      <c r="C26" s="75" t="inlineStr">
+        <is>
+          <t>A25-FINAL</t>
+        </is>
+      </c>
+      <c r="D26" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="75" t="inlineStr">
+        <is>
+          <t>Squash</t>
+        </is>
+      </c>
+      <c r="B27" s="75" t="inlineStr">
+        <is>
+          <t>Under 15</t>
+        </is>
+      </c>
+      <c r="C27" s="75" t="inlineStr">
+        <is>
+          <t>U15-FINAL</t>
+        </is>
+      </c>
+      <c r="D27" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="76" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="77" t="n"/>
+      <c r="C28" s="76" t="inlineStr">
+        <is>
+          <t>22 finals</t>
+        </is>
+      </c>
+      <c r="D28" s="76" t="n">
+        <v>22</v>
+      </c>
+      <c r="E28" s="76" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="78" t="inlineStr">
+        <is>
+          <t>Per-event summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="74" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="B31" s="74" t="inlineStr">
+        <is>
+          <t>Categories (finals)</t>
+        </is>
+      </c>
+      <c r="C31" s="74" t="inlineStr">
+        <is>
+          <t>Big Trophies</t>
+        </is>
+      </c>
+      <c r="D31" s="74" t="inlineStr">
+        <is>
+          <t>Small Trophies</t>
+        </is>
+      </c>
+      <c r="E31" s="74" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="75" t="inlineStr">
+        <is>
+          <t>TT — Men's Singles</t>
+        </is>
+      </c>
+      <c r="B32" s="75" t="n">
+        <v>5</v>
+      </c>
+      <c r="C32" s="75" t="n">
+        <v>5</v>
+      </c>
+      <c r="D32" s="75" t="n">
+        <v>5</v>
+      </c>
+      <c r="E32" s="77" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="75" t="inlineStr">
+        <is>
+          <t>Chess</t>
+        </is>
+      </c>
+      <c r="B33" s="75" t="n">
+        <v>4</v>
+      </c>
+      <c r="C33" s="75" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" s="75" t="n">
+        <v>4</v>
+      </c>
+      <c r="E33" s="77" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="75" t="inlineStr">
+        <is>
+          <t>Carrom — Men's Singles</t>
+        </is>
+      </c>
+      <c r="B34" s="75" t="n">
+        <v>3</v>
+      </c>
+      <c r="C34" s="75" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" s="75" t="n">
+        <v>3</v>
+      </c>
+      <c r="E34" s="77" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="75" t="inlineStr">
+        <is>
+          <t>Pool</t>
+        </is>
+      </c>
+      <c r="B35" s="75" t="n">
+        <v>3</v>
+      </c>
+      <c r="C35" s="75" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" s="75" t="n">
+        <v>3</v>
+      </c>
+      <c r="E35" s="77" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="75" t="inlineStr">
+        <is>
+          <t>Squash</t>
+        </is>
+      </c>
+      <c r="B36" s="75" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" s="75" t="n">
+        <v>3</v>
+      </c>
+      <c r="D36" s="75" t="n">
+        <v>3</v>
+      </c>
+      <c r="E36" s="77" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="75" t="inlineStr">
+        <is>
+          <t>TT — Women's Singles</t>
+        </is>
+      </c>
+      <c r="B37" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="77" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="75" t="inlineStr">
+        <is>
+          <t>TT — Doubles</t>
+        </is>
+      </c>
+      <c r="B38" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="77" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="75" t="inlineStr">
+        <is>
+          <t>Carrom — Women's Singles</t>
+        </is>
+      </c>
+      <c r="B39" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="77" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="75" t="inlineStr">
+        <is>
+          <t>Carrom — Doubles</t>
+        </is>
+      </c>
+      <c r="B40" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="77" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="55" t="inlineStr">
+        <is>
+          <t>MEDALS — UNDER 16 PARTICIPATION</t>
+        </is>
+      </c>
+      <c r="B42" s="56" t="n"/>
+      <c r="C42" s="56" t="n"/>
+      <c r="D42" s="56" t="n"/>
+      <c r="E42" s="56" t="n"/>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="79" t="inlineStr">
+        <is>
+          <t>14 unique players across all events are under 16. A medal goes to any of them who doesn't reach a final in ANY event/category they're entered in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="74" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B45" s="74" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="C45" s="74" t="inlineStr">
+        <is>
+          <t>Categories entered</t>
+        </is>
+      </c>
+      <c r="D45" s="80" t="n"/>
+      <c r="E45" s="80" t="n"/>
+      <c r="F45" s="80" t="n"/>
+      <c r="G45" s="81" t="n"/>
+    </row>
+    <row r="46" ht="15" customHeight="1">
+      <c r="A46" s="75" t="inlineStr">
+        <is>
+          <t>Rushabh</t>
+        </is>
+      </c>
+      <c r="B46" s="75" t="n">
+        <v>8</v>
+      </c>
+      <c r="C46" s="82" t="inlineStr">
+        <is>
+          <t>Chess (Under 11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="15" customHeight="1">
+      <c r="A47" s="75" t="inlineStr">
+        <is>
+          <t>Neev Chauhan</t>
+        </is>
+      </c>
+      <c r="B47" s="75" t="n">
+        <v>8</v>
+      </c>
+      <c r="C47" s="82" t="inlineStr">
+        <is>
+          <t>Chess (Under 11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="15" customHeight="1">
+      <c r="A48" s="75" t="inlineStr">
+        <is>
+          <t>Kaira</t>
+        </is>
+      </c>
+      <c r="B48" s="75" t="n">
+        <v>8</v>
+      </c>
+      <c r="C48" s="82" t="inlineStr">
+        <is>
+          <t>Carrom — Women's Singles (single category)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="15" customHeight="1">
+      <c r="A49" s="75" t="inlineStr">
+        <is>
+          <t>Kartik Relan</t>
+        </is>
+      </c>
+      <c r="B49" s="75" t="n">
+        <v>9</v>
+      </c>
+      <c r="C49" s="82" t="inlineStr">
+        <is>
+          <t>Chess (Under 11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="75" t="inlineStr">
+        <is>
+          <t>Shaurya Tripathi</t>
+        </is>
+      </c>
+      <c r="B50" s="75" t="n">
+        <v>10</v>
+      </c>
+      <c r="C50" s="82" t="inlineStr">
+        <is>
+          <t>Carrom — Men's Singles (Under 15); Squash (Under 15); TT — Men's Singles (Under 15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="75" t="inlineStr">
+        <is>
+          <t>Parth yadav</t>
+        </is>
+      </c>
+      <c r="B51" s="75" t="n">
+        <v>10</v>
+      </c>
+      <c r="C51" s="82" t="inlineStr">
+        <is>
+          <t>Chess (Under 11); Squash (Under 15); TT — Men's Singles (Under 15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="15" customHeight="1">
+      <c r="A52" s="75" t="inlineStr">
+        <is>
+          <t>Jimit Relan</t>
+        </is>
+      </c>
+      <c r="B52" s="75" t="n">
+        <v>11</v>
+      </c>
+      <c r="C52" s="82" t="inlineStr">
+        <is>
+          <t>Chess (Under 11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="15" customHeight="1">
+      <c r="A53" s="75" t="inlineStr">
+        <is>
+          <t>Aarav Pilankar</t>
+        </is>
+      </c>
+      <c r="B53" s="75" t="n">
+        <v>11</v>
+      </c>
+      <c r="C53" s="82" t="inlineStr">
+        <is>
+          <t>Carrom — Men's Singles (Under 15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="75" t="inlineStr">
+        <is>
+          <t>Aadit Joshi</t>
+        </is>
+      </c>
+      <c r="B54" s="75" t="n">
+        <v>12</v>
+      </c>
+      <c r="C54" s="82" t="inlineStr">
+        <is>
+          <t>Chess (12 to 20); Pool (Under 26); Squash (Under 15); TT — Men's Singles (Under 15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="15" customHeight="1">
+      <c r="A55" s="75" t="inlineStr">
+        <is>
+          <t>Peher Krunal Shah</t>
+        </is>
+      </c>
+      <c r="B55" s="75" t="n">
+        <v>12</v>
+      </c>
+      <c r="C55" s="82" t="inlineStr">
+        <is>
+          <t>Squash (Under 15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="15" customHeight="1">
+      <c r="A56" s="75" t="inlineStr">
+        <is>
+          <t>Viaan Neema</t>
+        </is>
+      </c>
+      <c r="B56" s="75" t="n">
+        <v>12</v>
+      </c>
+      <c r="C56" s="82" t="inlineStr">
+        <is>
+          <t>Squash (Under 15); TT — Men's Singles (Under 15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="15" customHeight="1">
+      <c r="A57" s="75" t="inlineStr">
+        <is>
+          <t>Hridh jhala</t>
+        </is>
+      </c>
+      <c r="B57" s="75" t="n">
+        <v>13</v>
+      </c>
+      <c r="C57" s="82" t="inlineStr">
+        <is>
+          <t>Squash (Under 15); TT — Men's Singles (Under 15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="75" t="inlineStr">
+        <is>
+          <t>Yash agarwal</t>
+        </is>
+      </c>
+      <c r="B58" s="75" t="n">
+        <v>13</v>
+      </c>
+      <c r="C58" s="82" t="inlineStr">
+        <is>
+          <t>Carrom — Men's Singles (Under 15); Squash (Under 15); TT — Men's Singles (Under 15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="15" customHeight="1">
+      <c r="A59" s="75" t="inlineStr">
+        <is>
+          <t>Maitreya Manvik</t>
+        </is>
+      </c>
+      <c r="B59" s="75" t="n">
+        <v>14</v>
+      </c>
+      <c r="C59" s="82" t="inlineStr">
+        <is>
+          <t>Chess (12 to 20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="30" customHeight="1">
+      <c r="A61" s="83" t="inlineStr">
+        <is>
+          <t>Categories entirely or mostly made up of Under-16 players (tightest medal bottlenecks — only 2 final slots each)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="74" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="B62" s="74" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C62" s="74" t="inlineStr">
+        <is>
+          <t>Under-16 players in it</t>
+        </is>
+      </c>
+      <c r="D62" s="84" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="75" t="inlineStr">
+        <is>
+          <t>Squash</t>
+        </is>
+      </c>
+      <c r="B63" s="75" t="inlineStr">
+        <is>
+          <t>Under 15</t>
+        </is>
+      </c>
+      <c r="C63" s="82" t="inlineStr">
+        <is>
+          <t>7: Aadit Joshi, Hridh jhala, Parth yadav, Peher Krunal Shah, Shaurya Tripathi, Viaan Neema, Yash agarwal</t>
+        </is>
+      </c>
+      <c r="E63" s="75" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="75" t="inlineStr">
+        <is>
+          <t>TT — Men's Singles</t>
+        </is>
+      </c>
+      <c r="B64" s="75" t="inlineStr">
+        <is>
+          <t>Under 15</t>
+        </is>
+      </c>
+      <c r="C64" s="82" t="inlineStr">
+        <is>
+          <t>6: Aadit Joshi, Hridh jhala, Parth yadav, Shaurya Tripathi, Viaan Neema, Yash agarwal</t>
+        </is>
+      </c>
+      <c r="E64" s="75" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="75" t="inlineStr">
+        <is>
+          <t>Chess</t>
+        </is>
+      </c>
+      <c r="B65" s="75" t="inlineStr">
+        <is>
+          <t>Under 11</t>
+        </is>
+      </c>
+      <c r="C65" s="82" t="inlineStr">
+        <is>
+          <t>5: Jimit Relan, Kartik Relan, Neev Chauhan, Parth yadav, Rushabh</t>
+        </is>
+      </c>
+      <c r="E65" s="75" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="75" t="inlineStr">
+        <is>
+          <t>Carrom — Men's Singles</t>
+        </is>
+      </c>
+      <c r="B66" s="75" t="inlineStr">
+        <is>
+          <t>Under 15</t>
+        </is>
+      </c>
+      <c r="C66" s="82" t="inlineStr">
+        <is>
+          <t>3: Aarav Pilankar, Shaurya Tripathi, Yash agarwal</t>
+        </is>
+      </c>
+      <c r="E66" s="75" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="75" t="inlineStr">
+        <is>
+          <t>Chess</t>
+        </is>
+      </c>
+      <c r="B67" s="75" t="inlineStr">
+        <is>
+          <t>12 to 20</t>
+        </is>
+      </c>
+      <c r="C67" s="82" t="inlineStr">
+        <is>
+          <t>2: Aadit Joshi, Maitreya Manvik</t>
+        </is>
+      </c>
+      <c r="E67" s="75" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="75" t="inlineStr">
+        <is>
+          <t>Pool</t>
+        </is>
+      </c>
+      <c r="B68" s="75" t="inlineStr">
+        <is>
+          <t>Under 26</t>
+        </is>
+      </c>
+      <c r="C68" s="82" t="inlineStr">
+        <is>
+          <t>1: Aadit Joshi</t>
+        </is>
+      </c>
+      <c r="E68" s="75" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="75" t="inlineStr">
+        <is>
+          <t>Carrom — Women's Singles</t>
+        </is>
+      </c>
+      <c r="B69" s="75" t="inlineStr">
+        <is>
+          <t>(single category)</t>
+        </is>
+      </c>
+      <c r="C69" s="82" t="inlineStr">
+        <is>
+          <t>1: Kaira</t>
+        </is>
+      </c>
+      <c r="E69" s="75" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="71" ht="30" customHeight="1">
+      <c r="A71" s="85" t="inlineStr">
+        <is>
+          <t>Estimated medal count: minimum 3 (best case — every multi-category player escapes via a different event), maximum 14 (worst case — none of them reach any final). Actual count depends on match results.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="31">
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="C49:G49"/>
+    <mergeCell ref="C62:D62"/>
+    <mergeCell ref="C68:D68"/>
+    <mergeCell ref="C58:G58"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="C45:G45"/>
+    <mergeCell ref="A61:E61"/>
+    <mergeCell ref="C64:D64"/>
+    <mergeCell ref="C47:G47"/>
+    <mergeCell ref="C54:G54"/>
+    <mergeCell ref="C63:D63"/>
+    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="C50:G50"/>
+    <mergeCell ref="C55:G55"/>
+    <mergeCell ref="C56:G56"/>
+    <mergeCell ref="C59:G59"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="C46:G46"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="C51:G51"/>
+    <mergeCell ref="A71:E71"/>
+    <mergeCell ref="C52:G52"/>
+    <mergeCell ref="C48:G48"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="C67:D67"/>
+    <mergeCell ref="C57:G57"/>
+    <mergeCell ref="C66:D66"/>
+    <mergeCell ref="C53:G53"/>
+    <mergeCell ref="C69:D69"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Fix overflowing/truncated text throughout the schedule workbook
Audited every cell across all 11 sheets for content wider than its
column (or taller than its row, for already-wrapped cells). Widened
columns for the many single-field overflows (player/pair name columns
across all 9 sport sheets - especially Carrom Doubles and TT Doubles,
whose paired names run up to 39 characters; a handful of narrow
headers in Overview and Trophies & Medals). Increased row height
rather than widening for cells that were already merged+wrapped but
too short vertically (Overview's day-structure/notes text, Trophies &
Medals' banner and bottleneck-category lists). Re-audited afterward:
zero overflow findings remain.
</commit_message>
<xml_diff>
--- a/Ekta_Schedule_With_Matchups.xlsx
+++ b/Ekta_Schedule_With_Matchups.xlsx
@@ -349,7 +349,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -586,6 +586,13 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -955,7 +962,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="21" min="1" max="1"/>
-    <col width="16" bestFit="1" customWidth="1" style="14" min="2" max="2"/>
+    <col width="20" bestFit="1" customWidth="1" style="14" min="2" max="2"/>
     <col width="20" bestFit="1" customWidth="1" style="14" min="3" max="3"/>
     <col width="16" bestFit="1" customWidth="1" style="14" min="4" max="4"/>
     <col width="16" customWidth="1" style="14" min="5" max="5"/>
@@ -1194,7 +1201,7 @@
       <c r="I15" s="31" t="n"/>
       <c r="J15" s="31" t="n"/>
     </row>
-    <row r="16" ht="45" customHeight="1">
+    <row r="16" ht="68" customHeight="1">
       <c r="A16" s="63" t="inlineStr">
         <is>
           <t>Aug 16</t>
@@ -1622,8 +1629,8 @@
       <c r="I33" s="31" t="n"/>
       <c r="J33" s="31" t="n"/>
     </row>
-    <row r="34">
-      <c r="A34" s="67" t="inlineStr">
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="86" t="inlineStr">
         <is>
           <t>Overall tournament span: Aug 15, 8:00 AM start → Aug 16, 5:45 PM finish — comfortably inside the Aug 16, 10 PM cap.</t>
         </is>
@@ -1658,7 +1665,7 @@
       <c r="I36" s="31" t="n"/>
       <c r="J36" s="31" t="n"/>
     </row>
-    <row r="37">
+    <row r="37" ht="30" customHeight="1">
       <c r="A37" s="65" t="inlineStr">
         <is>
           <t>Full match-by-match detail (exact times, table/board assignment, player groups) lives in each sport's own sheet — this tab is a summary only.</t>
@@ -1985,7 +1992,7 @@
   <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="20" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
     <col width="10" customWidth="1" style="14" min="2" max="3"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" style="14" min="4" max="4"/>
@@ -3434,10 +3441,10 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
@@ -3448,21 +3455,13 @@
           <t>TROPHIES &amp; MEDALS</t>
         </is>
       </c>
-      <c r="B1" s="58" t="n"/>
-      <c r="C1" s="58" t="n"/>
-      <c r="D1" s="58" t="n"/>
-      <c r="E1" s="58" t="n"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="73" t="inlineStr">
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="87" t="inlineStr">
         <is>
           <t>Every final's winner gets a big trophy, runner-up gets a small trophy. Under-16 players who don't reach any final they're entered in get a medal.</t>
         </is>
       </c>
-      <c r="B2" s="58" t="n"/>
-      <c r="C2" s="58" t="n"/>
-      <c r="D2" s="58" t="n"/>
-      <c r="E2" s="58" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="55" t="inlineStr">
@@ -3470,10 +3469,6 @@
           <t>TROPHY COUNT</t>
         </is>
       </c>
-      <c r="B4" s="56" t="n"/>
-      <c r="C4" s="56" t="n"/>
-      <c r="D4" s="56" t="n"/>
-      <c r="E4" s="56" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="74" t="inlineStr">
@@ -4216,10 +4211,6 @@
           <t>MEDALS — UNDER 16 PARTICIPATION</t>
         </is>
       </c>
-      <c r="B42" s="56" t="n"/>
-      <c r="C42" s="56" t="n"/>
-      <c r="D42" s="56" t="n"/>
-      <c r="E42" s="56" t="n"/>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="79" t="inlineStr">
@@ -4244,10 +4235,10 @@
           <t>Categories entered</t>
         </is>
       </c>
-      <c r="D45" s="80" t="n"/>
-      <c r="E45" s="80" t="n"/>
-      <c r="F45" s="80" t="n"/>
-      <c r="G45" s="81" t="n"/>
+      <c r="D45" s="88" t="n"/>
+      <c r="E45" s="88" t="n"/>
+      <c r="F45" s="88" t="n"/>
+      <c r="G45" s="84" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="75" t="inlineStr">
@@ -4263,6 +4254,10 @@
           <t>Chess (Under 11)</t>
         </is>
       </c>
+      <c r="D46" s="88" t="n"/>
+      <c r="E46" s="88" t="n"/>
+      <c r="F46" s="88" t="n"/>
+      <c r="G46" s="84" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="75" t="inlineStr">
@@ -4278,6 +4273,10 @@
           <t>Chess (Under 11)</t>
         </is>
       </c>
+      <c r="D47" s="88" t="n"/>
+      <c r="E47" s="88" t="n"/>
+      <c r="F47" s="88" t="n"/>
+      <c r="G47" s="84" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="75" t="inlineStr">
@@ -4293,6 +4292,10 @@
           <t>Carrom — Women's Singles (single category)</t>
         </is>
       </c>
+      <c r="D48" s="88" t="n"/>
+      <c r="E48" s="88" t="n"/>
+      <c r="F48" s="88" t="n"/>
+      <c r="G48" s="84" t="n"/>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="75" t="inlineStr">
@@ -4308,6 +4311,10 @@
           <t>Chess (Under 11)</t>
         </is>
       </c>
+      <c r="D49" s="88" t="n"/>
+      <c r="E49" s="88" t="n"/>
+      <c r="F49" s="88" t="n"/>
+      <c r="G49" s="84" t="n"/>
     </row>
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="75" t="inlineStr">
@@ -4323,6 +4330,10 @@
           <t>Carrom — Men's Singles (Under 15); Squash (Under 15); TT — Men's Singles (Under 15)</t>
         </is>
       </c>
+      <c r="D50" s="88" t="n"/>
+      <c r="E50" s="88" t="n"/>
+      <c r="F50" s="88" t="n"/>
+      <c r="G50" s="84" t="n"/>
     </row>
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="75" t="inlineStr">
@@ -4338,6 +4349,10 @@
           <t>Chess (Under 11); Squash (Under 15); TT — Men's Singles (Under 15)</t>
         </is>
       </c>
+      <c r="D51" s="88" t="n"/>
+      <c r="E51" s="88" t="n"/>
+      <c r="F51" s="88" t="n"/>
+      <c r="G51" s="84" t="n"/>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="75" t="inlineStr">
@@ -4353,6 +4368,10 @@
           <t>Chess (Under 11)</t>
         </is>
       </c>
+      <c r="D52" s="88" t="n"/>
+      <c r="E52" s="88" t="n"/>
+      <c r="F52" s="88" t="n"/>
+      <c r="G52" s="84" t="n"/>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="75" t="inlineStr">
@@ -4368,6 +4387,10 @@
           <t>Carrom — Men's Singles (Under 15)</t>
         </is>
       </c>
+      <c r="D53" s="88" t="n"/>
+      <c r="E53" s="88" t="n"/>
+      <c r="F53" s="88" t="n"/>
+      <c r="G53" s="84" t="n"/>
     </row>
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="75" t="inlineStr">
@@ -4383,6 +4406,10 @@
           <t>Chess (12 to 20); Pool (Under 26); Squash (Under 15); TT — Men's Singles (Under 15)</t>
         </is>
       </c>
+      <c r="D54" s="88" t="n"/>
+      <c r="E54" s="88" t="n"/>
+      <c r="F54" s="88" t="n"/>
+      <c r="G54" s="84" t="n"/>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="75" t="inlineStr">
@@ -4398,6 +4425,10 @@
           <t>Squash (Under 15)</t>
         </is>
       </c>
+      <c r="D55" s="88" t="n"/>
+      <c r="E55" s="88" t="n"/>
+      <c r="F55" s="88" t="n"/>
+      <c r="G55" s="84" t="n"/>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="75" t="inlineStr">
@@ -4413,6 +4444,10 @@
           <t>Squash (Under 15); TT — Men's Singles (Under 15)</t>
         </is>
       </c>
+      <c r="D56" s="88" t="n"/>
+      <c r="E56" s="88" t="n"/>
+      <c r="F56" s="88" t="n"/>
+      <c r="G56" s="84" t="n"/>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="75" t="inlineStr">
@@ -4428,6 +4463,10 @@
           <t>Squash (Under 15); TT — Men's Singles (Under 15)</t>
         </is>
       </c>
+      <c r="D57" s="88" t="n"/>
+      <c r="E57" s="88" t="n"/>
+      <c r="F57" s="88" t="n"/>
+      <c r="G57" s="84" t="n"/>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="75" t="inlineStr">
@@ -4443,6 +4482,10 @@
           <t>Carrom — Men's Singles (Under 15); Squash (Under 15); TT — Men's Singles (Under 15)</t>
         </is>
       </c>
+      <c r="D58" s="88" t="n"/>
+      <c r="E58" s="88" t="n"/>
+      <c r="F58" s="88" t="n"/>
+      <c r="G58" s="84" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="75" t="inlineStr">
@@ -4458,6 +4501,10 @@
           <t>Chess (12 to 20)</t>
         </is>
       </c>
+      <c r="D59" s="88" t="n"/>
+      <c r="E59" s="88" t="n"/>
+      <c r="F59" s="88" t="n"/>
+      <c r="G59" s="84" t="n"/>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="83" t="inlineStr">
@@ -4484,7 +4531,7 @@
       </c>
       <c r="D62" s="84" t="n"/>
     </row>
-    <row r="63">
+    <row r="63" ht="50" customHeight="1">
       <c r="A63" s="75" t="inlineStr">
         <is>
           <t>Squash</t>
@@ -4500,11 +4547,12 @@
           <t>7: Aadit Joshi, Hridh jhala, Parth yadav, Peher Krunal Shah, Shaurya Tripathi, Viaan Neema, Yash agarwal</t>
         </is>
       </c>
+      <c r="D63" s="84" t="n"/>
       <c r="E63" s="75" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" ht="50" customHeight="1">
       <c r="A64" s="75" t="inlineStr">
         <is>
           <t>TT — Men's Singles</t>
@@ -4520,11 +4568,12 @@
           <t>6: Aadit Joshi, Hridh jhala, Parth yadav, Shaurya Tripathi, Viaan Neema, Yash agarwal</t>
         </is>
       </c>
+      <c r="D64" s="84" t="n"/>
       <c r="E64" s="75" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" ht="35" customHeight="1">
       <c r="A65" s="75" t="inlineStr">
         <is>
           <t>Chess</t>
@@ -4540,11 +4589,12 @@
           <t>5: Jimit Relan, Kartik Relan, Neev Chauhan, Parth yadav, Rushabh</t>
         </is>
       </c>
+      <c r="D65" s="84" t="n"/>
       <c r="E65" s="75" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" ht="35" customHeight="1">
       <c r="A66" s="75" t="inlineStr">
         <is>
           <t>Carrom — Men's Singles</t>
@@ -4560,11 +4610,12 @@
           <t>3: Aarav Pilankar, Shaurya Tripathi, Yash agarwal</t>
         </is>
       </c>
+      <c r="D66" s="84" t="n"/>
       <c r="E66" s="75" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" ht="20" customHeight="1">
       <c r="A67" s="75" t="inlineStr">
         <is>
           <t>Chess</t>
@@ -4580,11 +4631,12 @@
           <t>2: Aadit Joshi, Maitreya Manvik</t>
         </is>
       </c>
+      <c r="D67" s="84" t="n"/>
       <c r="E67" s="75" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" ht="20" customHeight="1">
       <c r="A68" s="75" t="inlineStr">
         <is>
           <t>Pool</t>
@@ -4600,11 +4652,12 @@
           <t>1: Aadit Joshi</t>
         </is>
       </c>
+      <c r="D68" s="84" t="n"/>
       <c r="E68" s="75" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" ht="20" customHeight="1">
       <c r="A69" s="75" t="inlineStr">
         <is>
           <t>Carrom — Women's Singles</t>
@@ -4620,6 +4673,7 @@
           <t>1: Kaira</t>
         </is>
       </c>
+      <c r="D69" s="84" t="n"/>
       <c r="E69" s="75" t="n">
         <v>2</v>
       </c>
@@ -4678,7 +4732,7 @@
   <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="18" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="2" max="3"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" bestFit="1" customWidth="1" style="14" min="4" max="4"/>
@@ -5635,10 +5689,10 @@
   <dimension ref="A1:J115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="19" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="2" max="3"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="20" bestFit="1" customWidth="1" style="14" min="4" max="4"/>
+    <col width="23" bestFit="1" customWidth="1" style="14" min="4" max="4"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="5" max="5"/>
     <col width="12" bestFit="1" customWidth="1" style="14" min="6" max="6"/>
     <col width="11" bestFit="1" customWidth="1" style="14" min="7" max="7"/>
@@ -9738,16 +9792,16 @@
   <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="32" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="2" max="2"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="3" max="3"/>
     <col width="20" bestFit="1" customWidth="1" style="14" min="4" max="4"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="5" max="5"/>
     <col width="12" bestFit="1" customWidth="1" style="14" min="6" max="6"/>
     <col width="11" bestFit="1" customWidth="1" style="14" min="7" max="7"/>
-    <col width="27" bestFit="1" customWidth="1" style="14" min="8" max="8"/>
+    <col width="32" bestFit="1" customWidth="1" style="14" min="8" max="8"/>
     <col width="4" bestFit="1" customWidth="1" style="14" min="9" max="9"/>
-    <col width="27" customWidth="1" style="14" min="10" max="16384"/>
+    <col width="32" customWidth="1" style="14" min="10" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.95" customHeight="1">
@@ -10300,7 +10354,7 @@
   <dimension ref="A1:J82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="21" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
     <col width="10" customWidth="1" style="14" min="2" max="3"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" style="14" min="4" max="4"/>
@@ -13287,7 +13341,7 @@
   <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="22" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="2" max="3"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" bestFit="1" customWidth="1" style="14" min="4" max="4"/>
@@ -14020,16 +14074,16 @@
   <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="42" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="2" max="3"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" bestFit="1" customWidth="1" style="14" min="4" max="4"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="5" max="5"/>
     <col width="12" bestFit="1" customWidth="1" style="14" min="6" max="6"/>
     <col width="11" bestFit="1" customWidth="1" style="14" min="7" max="7"/>
-    <col width="27" bestFit="1" customWidth="1" style="14" min="8" max="8"/>
+    <col width="42" bestFit="1" customWidth="1" style="14" min="8" max="8"/>
     <col width="4" bestFit="1" customWidth="1" style="14" min="9" max="9"/>
-    <col width="27" customWidth="1" style="14" min="10" max="16384"/>
+    <col width="42" customWidth="1" style="14" min="10" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.95" customHeight="1">
@@ -15010,7 +15064,7 @@
   <dimension ref="A1:J92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="20" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
     <col width="10" customWidth="1" style="14" min="2" max="3"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" style="14" min="4" max="4"/>
@@ -18490,7 +18544,7 @@
   <dimension ref="A1:J100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="20" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
     <col width="10" customWidth="1" style="14" min="2" max="3"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" style="14" min="4" max="4"/>

</xml_diff>

<commit_message>
Fix player names still cut off in the last column of every sport sheet
The previous overflow fix used a rough character-count heuristic that
underestimated real rendering width in some viewers - Player B (the
sheet's actual last column, with no column to its right to spill into)
was still getting clipped, worst case Carrom Doubles' 39-character
paired names. Redone with actual pixel-width measurement of every
name (Liberation Sans, metrically close to Calibri) plus a generous
40% safety margin, applied to both Player A/B schedule columns and
the Player Groups name columns across all 9 sport sheets. Widths only
ever increased from their prior values, never shrunk. Also caught and
fixed three smaller gaps found in the same pass: Carrom Men's match
code column, Carrom Women's Band column, and a negligible Overview
banner rounding gap. Re-verified with the same pixel-measurement
method: zero overflow remains anywhere in the workbook.
</commit_message>
<xml_diff>
--- a/Ekta_Schedule_With_Matchups.xlsx
+++ b/Ekta_Schedule_With_Matchups.xlsx
@@ -965,7 +965,7 @@
     <col width="20" bestFit="1" customWidth="1" style="14" min="2" max="2"/>
     <col width="20" bestFit="1" customWidth="1" style="14" min="3" max="3"/>
     <col width="16" bestFit="1" customWidth="1" style="14" min="4" max="4"/>
-    <col width="16" customWidth="1" style="14" min="5" max="5"/>
+    <col width="17" customWidth="1" style="14" min="5" max="5"/>
     <col width="9" customWidth="1" style="14" min="6" max="6"/>
     <col width="11" customWidth="1" style="14" min="7" max="7"/>
     <col width="10" customWidth="1" style="14" min="8" max="8"/>
@@ -1992,7 +1992,7 @@
   <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="24.9" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
     <col width="10" customWidth="1" style="14" min="2" max="3"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" style="14" min="4" max="4"/>
@@ -4732,10 +4732,10 @@
   <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="21.9" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="2" max="3"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="20" bestFit="1" customWidth="1" style="14" min="4" max="4"/>
+    <col width="23.1" bestFit="1" customWidth="1" style="14" min="4" max="4"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="5" max="5"/>
     <col width="12" bestFit="1" customWidth="1" style="14" min="6" max="6"/>
     <col width="11" bestFit="1" customWidth="1" style="14" min="7" max="7"/>
@@ -5689,16 +5689,16 @@
   <dimension ref="A1:J115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="24.5" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="2" max="3"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="23" bestFit="1" customWidth="1" style="14" min="4" max="4"/>
+    <col width="36.9" bestFit="1" customWidth="1" style="14" min="4" max="4"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="5" max="5"/>
     <col width="12" bestFit="1" customWidth="1" style="14" min="6" max="6"/>
     <col width="11" bestFit="1" customWidth="1" style="14" min="7" max="7"/>
-    <col width="27" bestFit="1" customWidth="1" style="14" min="8" max="8"/>
+    <col width="36.9" bestFit="1" customWidth="1" style="14" min="8" max="8"/>
     <col width="4" bestFit="1" customWidth="1" style="14" min="9" max="9"/>
-    <col width="27" customWidth="1" style="14" min="10" max="16384"/>
+    <col width="36.9" customWidth="1" style="14" min="10" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.95" customHeight="1">
@@ -9792,16 +9792,16 @@
   <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="40.1" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="2" max="2"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="3" max="3"/>
     <col width="20" bestFit="1" customWidth="1" style="14" min="4" max="4"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="5" max="5"/>
     <col width="12" bestFit="1" customWidth="1" style="14" min="6" max="6"/>
     <col width="11" bestFit="1" customWidth="1" style="14" min="7" max="7"/>
-    <col width="32" bestFit="1" customWidth="1" style="14" min="8" max="8"/>
+    <col width="40.1" bestFit="1" customWidth="1" style="14" min="8" max="8"/>
     <col width="4" bestFit="1" customWidth="1" style="14" min="9" max="9"/>
-    <col width="32" customWidth="1" style="14" min="10" max="16384"/>
+    <col width="35.5" customWidth="1" style="14" min="10" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.95" customHeight="1">
@@ -10354,12 +10354,12 @@
   <dimension ref="A1:J82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="25.1" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
     <col width="10" customWidth="1" style="14" min="2" max="3"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" style="14" min="4" max="4"/>
+    <col width="23.9" customWidth="1" style="14" min="4" max="4"/>
     <col width="10" customWidth="1" style="14" min="5" max="5"/>
-    <col width="12" bestFit="1" customWidth="1" style="14" min="6" max="6"/>
+    <col width="15" bestFit="1" customWidth="1" style="14" min="6" max="6"/>
     <col width="11" customWidth="1" style="14" min="7" max="7"/>
     <col width="27" customWidth="1" style="14" min="8" max="8"/>
     <col width="4" customWidth="1" style="14" min="9" max="9"/>
@@ -13341,16 +13341,16 @@
   <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="28.7" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="2" max="3"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="20" bestFit="1" customWidth="1" style="14" min="4" max="4"/>
+    <col width="24" bestFit="1" customWidth="1" style="14" min="4" max="4"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="5" max="5"/>
     <col width="12" bestFit="1" customWidth="1" style="14" min="6" max="6"/>
     <col width="11" bestFit="1" customWidth="1" style="14" min="7" max="7"/>
-    <col width="27" bestFit="1" customWidth="1" style="14" min="8" max="8"/>
+    <col width="28.7" bestFit="1" customWidth="1" style="14" min="8" max="8"/>
     <col width="4" bestFit="1" customWidth="1" style="14" min="9" max="9"/>
-    <col width="27" customWidth="1" style="14" min="10" max="16384"/>
+    <col width="28.7" customWidth="1" style="14" min="10" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.95" customHeight="1">
@@ -14074,16 +14074,16 @@
   <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="54.1" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="2" max="3"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" bestFit="1" customWidth="1" style="14" min="4" max="4"/>
     <col width="10" bestFit="1" customWidth="1" style="14" min="5" max="5"/>
     <col width="12" bestFit="1" customWidth="1" style="14" min="6" max="6"/>
     <col width="11" bestFit="1" customWidth="1" style="14" min="7" max="7"/>
-    <col width="42" bestFit="1" customWidth="1" style="14" min="8" max="8"/>
+    <col width="46.5" bestFit="1" customWidth="1" style="14" min="8" max="8"/>
     <col width="4" bestFit="1" customWidth="1" style="14" min="9" max="9"/>
-    <col width="42" customWidth="1" style="14" min="10" max="16384"/>
+    <col width="54.1" customWidth="1" style="14" min="10" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.95" customHeight="1">
@@ -15064,10 +15064,10 @@
   <dimension ref="A1:J92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="25.1" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
     <col width="10" customWidth="1" style="14" min="2" max="3"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" style="14" min="4" max="4"/>
+    <col width="23.9" customWidth="1" style="14" min="4" max="4"/>
     <col width="10" customWidth="1" style="14" min="5" max="5"/>
     <col width="12" customWidth="1" style="14" min="6" max="6"/>
     <col width="11" customWidth="1" style="14" min="7" max="7"/>
@@ -18544,7 +18544,7 @@
   <dimension ref="A1:J100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="25.3" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
     <col width="10" customWidth="1" style="14" min="2" max="3"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" style="14" min="4" max="4"/>

</xml_diff>

<commit_message>
Fix Carrom Doubles pairing: Vinod Agrawal, not Shalu Agarwal
Resolves the name ambiguity flagged in the original registration data
- the correct partner for Vrinda Agrawal is Vinod Agrawal, matching
his existing entries elsewhere (TT Men's Singles, Carrom Men's
Singles). Updated in index.html's SEED_DATA and both the Player
Groups listing and schedule table in the Carrom Doubles sheet.
</commit_message>
<xml_diff>
--- a/Ekta_Schedule_With_Matchups.xlsx
+++ b/Ekta_Schedule_With_Matchups.xlsx
@@ -14169,7 +14169,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Shalu Agarwal &amp; Vrinda Agrawal</t>
+          <t>Vinod Agrawal &amp; Vrinda Agrawal</t>
         </is>
       </c>
       <c r="B12" s="1" t="n">
@@ -14528,7 +14528,7 @@
       </c>
       <c r="H31" s="28" t="inlineStr">
         <is>
-          <t>Shalu Agarwal &amp; Vrinda Agrawal</t>
+          <t>Vinod Agrawal &amp; Vrinda Agrawal</t>
         </is>
       </c>
       <c r="I31" s="28" t="inlineStr">

</xml_diff>

<commit_message>
Rebuild TT Men's Singles age bands so labels match actual player ages
The old bands (Under 15/32/36/46, Senior) didn't reflect who was actually
in them - e.g. "Under 36" had players up to 39, "Under 46" had players up
to 55. Rebanded into Under 15/26/36/46/Above 46 (each label now true of
its members) and regenerated the full 71-match bracket, scheduled
conflict-free against every other event's fixed schedule (shared TT
tables, cross-sport player overlaps, the 10-min break rule, and the
tournament-wide gate that holds all semis/finals until every event's
group stage is done). Tournament finish moves from 5:45 PM to 6:14 PM
Aug 16, since the new Above 46 band now contains 4 players who are also
in Carrom Men's and Chess's own late-afternoon semis/finals.

Updated the schedule workbook (TT Men's sheet, Overview, Trophies &
Medals), index.html's SEED_DATA, and CLAUDE.md to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Ekta_Schedule_With_Matchups.xlsx
+++ b/Ekta_Schedule_With_Matchups.xlsx
@@ -1398,7 +1398,7 @@
       </c>
       <c r="E25" s="63" t="inlineStr">
         <is>
-          <t>Aug16 5:45PM</t>
+          <t>Aug16 6:14PM</t>
         </is>
       </c>
       <c r="F25" s="31" t="n"/>
@@ -3463,7 +3463,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="55" t="inlineStr">
         <is>
@@ -3529,12 +3528,12 @@
       </c>
       <c r="B7" s="75" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="C7" s="75" t="inlineStr">
         <is>
-          <t>SR-FINAL</t>
+          <t>A46-FINAL</t>
         </is>
       </c>
       <c r="D7" s="75" t="n">
@@ -3575,12 +3574,12 @@
       </c>
       <c r="B9" s="75" t="inlineStr">
         <is>
-          <t>Under 32</t>
+          <t>Under 26</t>
         </is>
       </c>
       <c r="C9" s="75" t="inlineStr">
         <is>
-          <t>U32-FINAL</t>
+          <t>U26-FINAL</t>
         </is>
       </c>
       <c r="D9" s="75" t="n">
@@ -4023,7 +4022,6 @@
         <v>22</v>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="78" t="inlineStr">
         <is>
@@ -4207,7 +4205,6 @@
       </c>
       <c r="E40" s="77" t="n"/>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="A42" s="55" t="inlineStr">
         <is>
@@ -4222,7 +4219,6 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="A45" s="74" t="inlineStr">
         <is>
@@ -4510,7 +4506,6 @@
       <c r="F59" s="88" t="n"/>
       <c r="G59" s="84" t="n"/>
     </row>
-    <row r="60"/>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="83" t="inlineStr">
         <is>
@@ -4683,7 +4678,6 @@
         <v>2</v>
       </c>
     </row>
-    <row r="70"/>
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="85" t="inlineStr">
         <is>
@@ -4772,7 +4766,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="17.1" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
         <is>
@@ -4864,8 +4857,6 @@
         <v>58</v>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
     <row r="14" ht="20.1" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
@@ -5720,7 +5711,7 @@
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="23" t="inlineStr">
         <is>
-          <t>5 age bands, each Group Stage → Semifinal → Final (Under 32 is a single Americano pool) · Best of 3, Final Best of 5 · 2 Tables</t>
+          <t>5 age bands, each Group Stage → Semifinal → Final (Under 26 is a single Americano pool) · Best of 3, Final Best of 5 · 2 Tables</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5723,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="17.1" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
         <is>
@@ -5758,7 +5748,7 @@
           <t>Shaurya Tripathi</t>
         </is>
       </c>
-      <c r="B8" s="1" t="n">
+      <c r="B8" s="4" t="n">
         <v>10</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -5766,7 +5756,7 @@
           <t>Viaan Neema</t>
         </is>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="4" t="n">
         <v>12</v>
       </c>
     </row>
@@ -5776,7 +5766,7 @@
           <t>Parth yadav</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="6" t="n">
         <v>10</v>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -5784,7 +5774,7 @@
           <t>Yash agarwal</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="6" t="n">
         <v>13</v>
       </c>
     </row>
@@ -5794,7 +5784,7 @@
           <t>Aadit Joshi</t>
         </is>
       </c>
-      <c r="B10" s="1" t="n">
+      <c r="B10" s="4" t="n">
         <v>12</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -5802,15 +5792,14 @@
           <t>Hridh jhala</t>
         </is>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E10" s="4" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="17.1" customHeight="1">
       <c r="A12" s="24" t="inlineStr">
         <is>
-          <t>Under 32 (single pool, Americano)</t>
+          <t>Under 26 (single pool, Americano)</t>
         </is>
       </c>
     </row>
@@ -5832,7 +5821,7 @@
           <t>Yuvraj jain</t>
         </is>
       </c>
-      <c r="B14" s="1" t="n">
+      <c r="B14" s="4" t="n">
         <v>16</v>
       </c>
     </row>
@@ -5842,7 +5831,7 @@
           <t>Aaditya Kumar</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B15" s="6" t="n">
         <v>17</v>
       </c>
     </row>
@@ -5852,7 +5841,7 @@
           <t>Hryday Goyal</t>
         </is>
       </c>
-      <c r="B16" s="1" t="n">
+      <c r="B16" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -5862,7 +5851,7 @@
           <t>Pranit Shriyan</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="B17" s="6" t="n">
         <v>25</v>
       </c>
     </row>
@@ -5872,11 +5861,10 @@
           <t>Rahul Garg</t>
         </is>
       </c>
-      <c r="B18" s="1" t="n">
+      <c r="B18" s="4" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="17.1" customHeight="1">
       <c r="A20" s="24" t="inlineStr">
         <is>
@@ -5902,15 +5890,15 @@
           <t>Jashit Bajaj</t>
         </is>
       </c>
-      <c r="B22" s="1" t="n">
+      <c r="B22" s="4" t="n">
         <v>28</v>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Tej</t>
-        </is>
-      </c>
-      <c r="E22" s="1" t="n">
+          <t>Prakshal Shah</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="n">
         <v>32</v>
       </c>
     </row>
@@ -5920,16 +5908,16 @@
           <t>Ravi Modi</t>
         </is>
       </c>
-      <c r="B23" s="2" t="n">
+      <c r="B23" s="6" t="n">
         <v>29</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Dr Rahul Modi</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="n">
-        <v>36</v>
+          <t>Amar Parulekar</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="24">
@@ -5938,234 +5926,242 @@
           <t>Tapabrata Dutta</t>
         </is>
       </c>
-      <c r="B24" s="1" t="n">
+      <c r="B24" s="4" t="n">
         <v>31</v>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
+          <t>Tej</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n"/>
+      <c r="B25" s="2" t="n"/>
+      <c r="D25" s="6" t="n"/>
+      <c r="E25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="24" t="inlineStr">
+        <is>
+          <t>Under 46</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Group A</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>Group B</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="17.1" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Dr Rahul Modi</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Nikunj Jhala</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
           <t>Ankur Mahante</t>
         </is>
       </c>
-      <c r="E24" s="1" t="n">
+      <c r="B29" s="6" t="n">
         <v>38</v>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Prakshal Shah</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>Sudip Parui</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="n">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Amar Parulekar</t>
-        </is>
-      </c>
-      <c r="B26" s="1" t="n">
-        <v>32</v>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>Tanmay Sharma</t>
-        </is>
-      </c>
-      <c r="E26" s="1" t="n">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="27"/>
-    <row r="28" ht="17.1" customHeight="1">
-      <c r="A28" s="24" t="inlineStr">
-        <is>
-          <t>Under 46</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="11" t="inlineStr">
-        <is>
-          <t>Group A</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="inlineStr">
-        <is>
-          <t>Group B</t>
-        </is>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Piyush Makharia</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>43</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Anuj Shah</t>
-        </is>
-      </c>
-      <c r="B30" s="1" t="n">
-        <v>39</v>
+          <t>Sudip Parui</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>38</v>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Amit Ranka</t>
-        </is>
-      </c>
-      <c r="E30" s="1" t="n">
-        <v>45</v>
+          <t>Vinit Padia</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Nikunj Jhala</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="n">
-        <v>40</v>
+          <t>Tanmay Sharma</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="n">
+        <v>39</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Mukul Joshi</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="n">
-        <v>51</v>
+          <t>Nilesh Bagaria</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Piyush Makharia</t>
-        </is>
-      </c>
-      <c r="B32" s="1" t="n">
-        <v>43</v>
+          <t>Anuj Shah</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="n">
+        <v>39</v>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
+          <t>Amit Ranka</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="D33" s="6" t="n"/>
+      <c r="E33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="24" t="inlineStr">
+        <is>
+          <t>Above 46</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>Group A</t>
+        </is>
+      </c>
+      <c r="D35" s="11" t="inlineStr">
+        <is>
+          <t>Group B</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="17.1" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Mukul Joshi</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Sanjay Kumar</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
           <t>Adil Khan</t>
         </is>
       </c>
-      <c r="E32" s="1" t="n">
+      <c r="B37" s="6" t="n">
         <v>51</v>
       </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>Vinit Padia</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>Vinod Agrawal</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="n">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>Nilesh Bagaria</t>
-        </is>
-      </c>
-      <c r="B34" s="1" t="n">
-        <v>44</v>
-      </c>
-      <c r="D34" s="4" t="n"/>
-      <c r="E34" s="1" t="n"/>
-    </row>
-    <row r="35"/>
-    <row r="36" ht="17.1" customHeight="1">
-      <c r="A36" s="24" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="11" t="inlineStr">
-        <is>
-          <t>Group A</t>
-        </is>
-      </c>
-      <c r="D37" s="11" t="inlineStr">
-        <is>
-          <t>Group B</t>
-        </is>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>Sushil Dashpute</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v>62</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Ajit nair</t>
-        </is>
-      </c>
-      <c r="B38" s="1" t="n">
-        <v>59</v>
+          <t>Vinod Agrawal</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="n">
+        <v>55</v>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Sushil Dashpute</t>
-        </is>
-      </c>
-      <c r="E38" s="1" t="n">
+          <t>HARSHAPRABHAT SHETTY</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="n">
         <v>62</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Ghansyam nawani</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="n">
-        <v>60</v>
+          <t>Ajit nair</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="n">
+        <v>59</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>HARSHAPRABHAT SHETTY</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="n">
-        <v>62</v>
+          <t>Kishore Kumar</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>Sanjay Kumar</t>
-        </is>
-      </c>
-      <c r="B40" s="1" t="n">
-        <v>61</v>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>Kishore Kumar</t>
-        </is>
-      </c>
-      <c r="E40" s="1" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="41"/>
-    <row r="42"/>
+          <t>Ghansyam nawani</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="D40" s="4" t="n"/>
+      <c r="E40" s="1" t="n"/>
+    </row>
     <row r="43" ht="20.1" customHeight="1">
       <c r="A43" s="16" t="inlineStr">
         <is>
@@ -6243,7 +6239,7 @@
       </c>
       <c r="D45" s="27" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E45" s="27" t="n">
@@ -6251,7 +6247,7 @@
       </c>
       <c r="F45" s="27" t="inlineStr">
         <is>
-          <t>SR-GA-1</t>
+          <t>A46-GA-1</t>
         </is>
       </c>
       <c r="G45" s="27" t="inlineStr">
@@ -6261,7 +6257,7 @@
       </c>
       <c r="H45" s="27" t="inlineStr">
         <is>
-          <t>Ajit nair</t>
+          <t>Mukul Joshi</t>
         </is>
       </c>
       <c r="I45" s="27" t="inlineStr">
@@ -6271,7 +6267,7 @@
       </c>
       <c r="J45" s="27" t="inlineStr">
         <is>
-          <t>Ghansyam nawani</t>
+          <t>Adil Khan</t>
         </is>
       </c>
     </row>
@@ -6293,7 +6289,7 @@
       </c>
       <c r="D46" s="28" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E46" s="28" t="n">
@@ -6301,7 +6297,7 @@
       </c>
       <c r="F46" s="28" t="inlineStr">
         <is>
-          <t>SR-GB-1</t>
+          <t>A46-GA-8</t>
         </is>
       </c>
       <c r="G46" s="28" t="inlineStr">
@@ -6311,7 +6307,7 @@
       </c>
       <c r="H46" s="28" t="inlineStr">
         <is>
-          <t>Sushil Dashpute</t>
+          <t>Vinod Agrawal</t>
         </is>
       </c>
       <c r="I46" s="28" t="inlineStr">
@@ -6321,7 +6317,7 @@
       </c>
       <c r="J46" s="28" t="inlineStr">
         <is>
-          <t>HARSHAPRABHAT SHETTY</t>
+          <t>Ajit nair</t>
         </is>
       </c>
     </row>
@@ -6333,17 +6329,17 @@
       </c>
       <c r="B47" s="27" t="inlineStr">
         <is>
-          <t>8:25AM</t>
+          <t>8:15AM</t>
         </is>
       </c>
       <c r="C47" s="27" t="inlineStr">
         <is>
-          <t>8:40AM</t>
+          <t>8:30AM</t>
         </is>
       </c>
       <c r="D47" s="27" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E47" s="27" t="n">
@@ -6351,7 +6347,7 @@
       </c>
       <c r="F47" s="27" t="inlineStr">
         <is>
-          <t>SR-GA-2</t>
+          <t>A46-GB-1</t>
         </is>
       </c>
       <c r="G47" s="27" t="inlineStr">
@@ -6361,7 +6357,7 @@
       </c>
       <c r="H47" s="27" t="inlineStr">
         <is>
-          <t>Ajit nair</t>
+          <t>Sanjay Kumar</t>
         </is>
       </c>
       <c r="I47" s="27" t="inlineStr">
@@ -6371,7 +6367,7 @@
       </c>
       <c r="J47" s="27" t="inlineStr">
         <is>
-          <t>Sanjay Kumar</t>
+          <t>Sushil Dashpute</t>
         </is>
       </c>
     </row>
@@ -6383,17 +6379,17 @@
       </c>
       <c r="B48" s="28" t="inlineStr">
         <is>
-          <t>8:25AM</t>
+          <t>8:15AM</t>
         </is>
       </c>
       <c r="C48" s="28" t="inlineStr">
         <is>
-          <t>8:40AM</t>
+          <t>8:30AM</t>
         </is>
       </c>
       <c r="D48" s="28" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E48" s="28" t="n">
@@ -6401,7 +6397,7 @@
       </c>
       <c r="F48" s="28" t="inlineStr">
         <is>
-          <t>SR-GB-2</t>
+          <t>A46-GB-6</t>
         </is>
       </c>
       <c r="G48" s="28" t="inlineStr">
@@ -6411,7 +6407,7 @@
       </c>
       <c r="H48" s="28" t="inlineStr">
         <is>
-          <t>Sushil Dashpute</t>
+          <t>HARSHAPRABHAT SHETTY</t>
         </is>
       </c>
       <c r="I48" s="28" t="inlineStr">
@@ -6433,17 +6429,17 @@
       </c>
       <c r="B49" s="27" t="inlineStr">
         <is>
-          <t>8:50AM</t>
+          <t>8:30AM</t>
         </is>
       </c>
       <c r="C49" s="27" t="inlineStr">
         <is>
-          <t>9:05AM</t>
+          <t>8:45AM</t>
         </is>
       </c>
       <c r="D49" s="27" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E49" s="27" t="n">
@@ -6451,7 +6447,7 @@
       </c>
       <c r="F49" s="27" t="inlineStr">
         <is>
-          <t>SR-GA-3</t>
+          <t>A46-GA-2</t>
         </is>
       </c>
       <c r="G49" s="27" t="inlineStr">
@@ -6461,7 +6457,7 @@
       </c>
       <c r="H49" s="27" t="inlineStr">
         <is>
-          <t>Ghansyam nawani</t>
+          <t>Mukul Joshi</t>
         </is>
       </c>
       <c r="I49" s="27" t="inlineStr">
@@ -6471,7 +6467,7 @@
       </c>
       <c r="J49" s="27" t="inlineStr">
         <is>
-          <t>Sanjay Kumar</t>
+          <t>Vinod Agrawal</t>
         </is>
       </c>
     </row>
@@ -6483,17 +6479,17 @@
       </c>
       <c r="B50" s="28" t="inlineStr">
         <is>
-          <t>8:50AM</t>
+          <t>8:30AM</t>
         </is>
       </c>
       <c r="C50" s="28" t="inlineStr">
         <is>
-          <t>9:05AM</t>
+          <t>8:45AM</t>
         </is>
       </c>
       <c r="D50" s="28" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E50" s="28" t="n">
@@ -6501,7 +6497,7 @@
       </c>
       <c r="F50" s="28" t="inlineStr">
         <is>
-          <t>SR-GB-3</t>
+          <t>A46-GA-6</t>
         </is>
       </c>
       <c r="G50" s="28" t="inlineStr">
@@ -6511,7 +6507,7 @@
       </c>
       <c r="H50" s="28" t="inlineStr">
         <is>
-          <t>HARSHAPRABHAT SHETTY</t>
+          <t>Adil Khan</t>
         </is>
       </c>
       <c r="I50" s="28" t="inlineStr">
@@ -6521,7 +6517,7 @@
       </c>
       <c r="J50" s="28" t="inlineStr">
         <is>
-          <t>Kishore Kumar</t>
+          <t>Ajit nair</t>
         </is>
       </c>
     </row>
@@ -6533,17 +6529,17 @@
       </c>
       <c r="B51" s="27" t="inlineStr">
         <is>
-          <t>4:00PM</t>
+          <t>8:45AM</t>
         </is>
       </c>
       <c r="C51" s="27" t="inlineStr">
         <is>
-          <t>4:15PM</t>
+          <t>9:00AM</t>
         </is>
       </c>
       <c r="D51" s="27" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E51" s="27" t="n">
@@ -6551,7 +6547,7 @@
       </c>
       <c r="F51" s="27" t="inlineStr">
         <is>
-          <t>U36-GA-1</t>
+          <t>A46-GB-2</t>
         </is>
       </c>
       <c r="G51" s="27" t="inlineStr">
@@ -6561,7 +6557,7 @@
       </c>
       <c r="H51" s="27" t="inlineStr">
         <is>
-          <t>Tapabrata Dutta</t>
+          <t>Sanjay Kumar</t>
         </is>
       </c>
       <c r="I51" s="27" t="inlineStr">
@@ -6571,7 +6567,7 @@
       </c>
       <c r="J51" s="27" t="inlineStr">
         <is>
-          <t>Prakshal Shah</t>
+          <t>HARSHAPRABHAT SHETTY</t>
         </is>
       </c>
     </row>
@@ -6583,17 +6579,17 @@
       </c>
       <c r="B52" s="28" t="inlineStr">
         <is>
-          <t>4:30PM</t>
+          <t>8:45AM</t>
         </is>
       </c>
       <c r="C52" s="28" t="inlineStr">
         <is>
-          <t>4:45PM</t>
+          <t>9:00AM</t>
         </is>
       </c>
       <c r="D52" s="28" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E52" s="28" t="n">
@@ -6601,17 +6597,17 @@
       </c>
       <c r="F52" s="28" t="inlineStr">
         <is>
-          <t>U36-GA-2</t>
+          <t>A46-GB-5</t>
         </is>
       </c>
       <c r="G52" s="28" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H52" s="28" t="inlineStr">
         <is>
-          <t>Jashit Bajaj</t>
+          <t>Sushil Dashpute</t>
         </is>
       </c>
       <c r="I52" s="28" t="inlineStr">
@@ -6621,7 +6617,7 @@
       </c>
       <c r="J52" s="28" t="inlineStr">
         <is>
-          <t>Ravi Modi</t>
+          <t>Kishore Kumar</t>
         </is>
       </c>
     </row>
@@ -6633,17 +6629,17 @@
       </c>
       <c r="B53" s="27" t="inlineStr">
         <is>
-          <t>4:30PM</t>
+          <t>9:00AM</t>
         </is>
       </c>
       <c r="C53" s="27" t="inlineStr">
         <is>
-          <t>4:45PM</t>
+          <t>9:15AM</t>
         </is>
       </c>
       <c r="D53" s="27" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E53" s="27" t="n">
@@ -6651,17 +6647,17 @@
       </c>
       <c r="F53" s="27" t="inlineStr">
         <is>
-          <t>U36-GB-1</t>
+          <t>A46-GA-3</t>
         </is>
       </c>
       <c r="G53" s="27" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H53" s="27" t="inlineStr">
         <is>
-          <t>Tej</t>
+          <t>Mukul Joshi</t>
         </is>
       </c>
       <c r="I53" s="27" t="inlineStr">
@@ -6671,7 +6667,7 @@
       </c>
       <c r="J53" s="27" t="inlineStr">
         <is>
-          <t>Dr Rahul Modi</t>
+          <t>Ajit nair</t>
         </is>
       </c>
     </row>
@@ -6683,17 +6679,17 @@
       </c>
       <c r="B54" s="28" t="inlineStr">
         <is>
-          <t>4:45PM</t>
+          <t>9:00AM</t>
         </is>
       </c>
       <c r="C54" s="28" t="inlineStr">
         <is>
-          <t>5:00PM</t>
+          <t>9:15AM</t>
         </is>
       </c>
       <c r="D54" s="28" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E54" s="28" t="n">
@@ -6701,7 +6697,7 @@
       </c>
       <c r="F54" s="28" t="inlineStr">
         <is>
-          <t>U36-GB-2</t>
+          <t>A46-GA-5</t>
         </is>
       </c>
       <c r="G54" s="28" t="inlineStr">
@@ -6711,7 +6707,7 @@
       </c>
       <c r="H54" s="28" t="inlineStr">
         <is>
-          <t>Ankur Mahante</t>
+          <t>Adil Khan</t>
         </is>
       </c>
       <c r="I54" s="28" t="inlineStr">
@@ -6721,7 +6717,7 @@
       </c>
       <c r="J54" s="28" t="inlineStr">
         <is>
-          <t>Sudip Parui</t>
+          <t>Vinod Agrawal</t>
         </is>
       </c>
     </row>
@@ -6733,17 +6729,17 @@
       </c>
       <c r="B55" s="27" t="inlineStr">
         <is>
-          <t>4:55PM</t>
+          <t>9:15AM</t>
         </is>
       </c>
       <c r="C55" s="27" t="inlineStr">
         <is>
-          <t>5:10PM</t>
+          <t>9:30AM</t>
         </is>
       </c>
       <c r="D55" s="27" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E55" s="27" t="n">
@@ -6751,7 +6747,7 @@
       </c>
       <c r="F55" s="27" t="inlineStr">
         <is>
-          <t>U36-GA-3</t>
+          <t>A46-GB-3</t>
         </is>
       </c>
       <c r="G55" s="27" t="inlineStr">
@@ -6761,7 +6757,7 @@
       </c>
       <c r="H55" s="27" t="inlineStr">
         <is>
-          <t>Ravi Modi</t>
+          <t>Sanjay Kumar</t>
         </is>
       </c>
       <c r="I55" s="27" t="inlineStr">
@@ -6771,7 +6767,7 @@
       </c>
       <c r="J55" s="27" t="inlineStr">
         <is>
-          <t>Amar Parulekar</t>
+          <t>Kishore Kumar</t>
         </is>
       </c>
     </row>
@@ -6783,17 +6779,17 @@
       </c>
       <c r="B56" s="28" t="inlineStr">
         <is>
-          <t>5:10PM</t>
+          <t>9:15AM</t>
         </is>
       </c>
       <c r="C56" s="28" t="inlineStr">
         <is>
-          <t>5:25PM</t>
+          <t>9:30AM</t>
         </is>
       </c>
       <c r="D56" s="28" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E56" s="28" t="n">
@@ -6801,17 +6797,17 @@
       </c>
       <c r="F56" s="28" t="inlineStr">
         <is>
-          <t>U36-GA-4</t>
+          <t>A46-GB-4</t>
         </is>
       </c>
       <c r="G56" s="28" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H56" s="28" t="inlineStr">
         <is>
-          <t>Jashit Bajaj</t>
+          <t>Sushil Dashpute</t>
         </is>
       </c>
       <c r="I56" s="28" t="inlineStr">
@@ -6821,7 +6817,7 @@
       </c>
       <c r="J56" s="28" t="inlineStr">
         <is>
-          <t>Tapabrata Dutta</t>
+          <t>HARSHAPRABHAT SHETTY</t>
         </is>
       </c>
     </row>
@@ -6833,17 +6829,17 @@
       </c>
       <c r="B57" s="27" t="inlineStr">
         <is>
-          <t>5:20PM</t>
+          <t>11:50AM</t>
         </is>
       </c>
       <c r="C57" s="27" t="inlineStr">
         <is>
-          <t>5:35PM</t>
+          <t>12:05PM</t>
         </is>
       </c>
       <c r="D57" s="27" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E57" s="27" t="n">
@@ -6851,17 +6847,17 @@
       </c>
       <c r="F57" s="27" t="inlineStr">
         <is>
-          <t>U36-GA-5</t>
+          <t>A46-GA-4</t>
         </is>
       </c>
       <c r="G57" s="27" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H57" s="27" t="inlineStr">
         <is>
-          <t>Prakshal Shah</t>
+          <t>Mukul Joshi</t>
         </is>
       </c>
       <c r="I57" s="27" t="inlineStr">
@@ -6871,7 +6867,7 @@
       </c>
       <c r="J57" s="27" t="inlineStr">
         <is>
-          <t>Amar Parulekar</t>
+          <t>Ghansyam nawani</t>
         </is>
       </c>
     </row>
@@ -6883,17 +6879,17 @@
       </c>
       <c r="B58" s="28" t="inlineStr">
         <is>
-          <t>5:45PM</t>
+          <t>11:50AM</t>
         </is>
       </c>
       <c r="C58" s="28" t="inlineStr">
         <is>
-          <t>6:00PM</t>
+          <t>12:05PM</t>
         </is>
       </c>
       <c r="D58" s="28" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Under 15</t>
         </is>
       </c>
       <c r="E58" s="28" t="n">
@@ -6901,17 +6897,17 @@
       </c>
       <c r="F58" s="28" t="inlineStr">
         <is>
-          <t>U36-GA-6</t>
+          <t>U15-GA-2</t>
         </is>
       </c>
       <c r="G58" s="28" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H58" s="28" t="inlineStr">
         <is>
-          <t>Jashit Bajaj</t>
+          <t>Shaurya Tripathi</t>
         </is>
       </c>
       <c r="I58" s="28" t="inlineStr">
@@ -6921,7 +6917,7 @@
       </c>
       <c r="J58" s="28" t="inlineStr">
         <is>
-          <t>Prakshal Shah</t>
+          <t>Aadit Joshi</t>
         </is>
       </c>
     </row>
@@ -6933,17 +6929,17 @@
       </c>
       <c r="B59" s="27" t="inlineStr">
         <is>
-          <t>5:53PM</t>
+          <t>3:55PM</t>
         </is>
       </c>
       <c r="C59" s="27" t="inlineStr">
         <is>
-          <t>6:08PM</t>
+          <t>4:10PM</t>
         </is>
       </c>
       <c r="D59" s="27" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E59" s="27" t="n">
@@ -6951,17 +6947,17 @@
       </c>
       <c r="F59" s="27" t="inlineStr">
         <is>
-          <t>U36-GB-3</t>
+          <t>A46-GA-7</t>
         </is>
       </c>
       <c r="G59" s="27" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H59" s="27" t="inlineStr">
         <is>
-          <t>Dr Rahul Modi</t>
+          <t>Adil Khan</t>
         </is>
       </c>
       <c r="I59" s="27" t="inlineStr">
@@ -6971,7 +6967,7 @@
       </c>
       <c r="J59" s="27" t="inlineStr">
         <is>
-          <t>Tanmay Sharma</t>
+          <t>Ghansyam nawani</t>
         </is>
       </c>
     </row>
@@ -6983,17 +6979,17 @@
       </c>
       <c r="B60" s="28" t="inlineStr">
         <is>
-          <t>6:00PM</t>
+          <t>4:10PM</t>
         </is>
       </c>
       <c r="C60" s="28" t="inlineStr">
         <is>
-          <t>6:15PM</t>
+          <t>4:25PM</t>
         </is>
       </c>
       <c r="D60" s="28" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Under 15</t>
         </is>
       </c>
       <c r="E60" s="28" t="n">
@@ -7001,17 +6997,17 @@
       </c>
       <c r="F60" s="28" t="inlineStr">
         <is>
-          <t>U36-GB-4</t>
+          <t>U15-GA-3</t>
         </is>
       </c>
       <c r="G60" s="28" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H60" s="28" t="inlineStr">
         <is>
-          <t>Tej</t>
+          <t>Parth yadav</t>
         </is>
       </c>
       <c r="I60" s="28" t="inlineStr">
@@ -7021,7 +7017,7 @@
       </c>
       <c r="J60" s="28" t="inlineStr">
         <is>
-          <t>Ankur Mahante</t>
+          <t>Aadit Joshi</t>
         </is>
       </c>
     </row>
@@ -7033,17 +7029,17 @@
       </c>
       <c r="B61" s="27" t="inlineStr">
         <is>
-          <t>6:15PM</t>
+          <t>4:20PM</t>
         </is>
       </c>
       <c r="C61" s="27" t="inlineStr">
         <is>
-          <t>6:30PM</t>
+          <t>4:35PM</t>
         </is>
       </c>
       <c r="D61" s="27" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E61" s="27" t="n">
@@ -7051,7 +7047,7 @@
       </c>
       <c r="F61" s="27" t="inlineStr">
         <is>
-          <t>U36-GA-7</t>
+          <t>A46-GA-9</t>
         </is>
       </c>
       <c r="G61" s="27" t="inlineStr">
@@ -7061,7 +7057,7 @@
       </c>
       <c r="H61" s="27" t="inlineStr">
         <is>
-          <t>Ravi Modi</t>
+          <t>Vinod Agrawal</t>
         </is>
       </c>
       <c r="I61" s="27" t="inlineStr">
@@ -7071,7 +7067,7 @@
       </c>
       <c r="J61" s="27" t="inlineStr">
         <is>
-          <t>Tapabrata Dutta</t>
+          <t>Ghansyam nawani</t>
         </is>
       </c>
     </row>
@@ -7083,17 +7079,17 @@
       </c>
       <c r="B62" s="28" t="inlineStr">
         <is>
-          <t>6:18PM</t>
+          <t>4:25PM</t>
         </is>
       </c>
       <c r="C62" s="28" t="inlineStr">
         <is>
-          <t>6:33PM</t>
+          <t>4:40PM</t>
         </is>
       </c>
       <c r="D62" s="28" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Under 15</t>
         </is>
       </c>
       <c r="E62" s="28" t="n">
@@ -7101,7 +7097,7 @@
       </c>
       <c r="F62" s="28" t="inlineStr">
         <is>
-          <t>U36-GB-5</t>
+          <t>U15-GB-2</t>
         </is>
       </c>
       <c r="G62" s="28" t="inlineStr">
@@ -7111,7 +7107,7 @@
       </c>
       <c r="H62" s="28" t="inlineStr">
         <is>
-          <t>Sudip Parui</t>
+          <t>Viaan Neema</t>
         </is>
       </c>
       <c r="I62" s="28" t="inlineStr">
@@ -7121,7 +7117,7 @@
       </c>
       <c r="J62" s="28" t="inlineStr">
         <is>
-          <t>Tanmay Sharma</t>
+          <t>Hridh jhala</t>
         </is>
       </c>
     </row>
@@ -7133,17 +7129,17 @@
       </c>
       <c r="B63" s="27" t="inlineStr">
         <is>
-          <t>6:33PM</t>
+          <t>4:40PM</t>
         </is>
       </c>
       <c r="C63" s="27" t="inlineStr">
         <is>
-          <t>6:48PM</t>
+          <t>4:55PM</t>
         </is>
       </c>
       <c r="D63" s="27" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Under 26</t>
         </is>
       </c>
       <c r="E63" s="27" t="n">
@@ -7151,7 +7147,7 @@
       </c>
       <c r="F63" s="27" t="inlineStr">
         <is>
-          <t>U36-GB-6</t>
+          <t>U26-1</t>
         </is>
       </c>
       <c r="G63" s="27" t="inlineStr">
@@ -7161,7 +7157,7 @@
       </c>
       <c r="H63" s="27" t="inlineStr">
         <is>
-          <t>Dr Rahul Modi</t>
+          <t>Yuvraj jain</t>
         </is>
       </c>
       <c r="I63" s="27" t="inlineStr">
@@ -7171,7 +7167,7 @@
       </c>
       <c r="J63" s="27" t="inlineStr">
         <is>
-          <t>Ankur Mahante</t>
+          <t>Aaditya Kumar</t>
         </is>
       </c>
     </row>
@@ -7183,17 +7179,17 @@
       </c>
       <c r="B64" s="28" t="inlineStr">
         <is>
-          <t>6:40PM</t>
+          <t>4:45PM</t>
         </is>
       </c>
       <c r="C64" s="28" t="inlineStr">
         <is>
-          <t>6:55PM</t>
+          <t>5:00PM</t>
         </is>
       </c>
       <c r="D64" s="28" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E64" s="28" t="n">
@@ -7201,7 +7197,7 @@
       </c>
       <c r="F64" s="28" t="inlineStr">
         <is>
-          <t>U36-GA-8</t>
+          <t>A46-GA-10</t>
         </is>
       </c>
       <c r="G64" s="28" t="inlineStr">
@@ -7211,7 +7207,7 @@
       </c>
       <c r="H64" s="28" t="inlineStr">
         <is>
-          <t>Tapabrata Dutta</t>
+          <t>Ajit nair</t>
         </is>
       </c>
       <c r="I64" s="28" t="inlineStr">
@@ -7221,7 +7217,7 @@
       </c>
       <c r="J64" s="28" t="inlineStr">
         <is>
-          <t>Amar Parulekar</t>
+          <t>Ghansyam nawani</t>
         </is>
       </c>
     </row>
@@ -7233,17 +7229,17 @@
       </c>
       <c r="B65" s="27" t="inlineStr">
         <is>
-          <t>6:58PM</t>
+          <t>4:55PM</t>
         </is>
       </c>
       <c r="C65" s="27" t="inlineStr">
         <is>
-          <t>7:13PM</t>
+          <t>5:10PM</t>
         </is>
       </c>
       <c r="D65" s="27" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Under 26</t>
         </is>
       </c>
       <c r="E65" s="27" t="n">
@@ -7251,7 +7247,7 @@
       </c>
       <c r="F65" s="27" t="inlineStr">
         <is>
-          <t>U36-GB-7</t>
+          <t>U26-8</t>
         </is>
       </c>
       <c r="G65" s="27" t="inlineStr">
@@ -7261,7 +7257,7 @@
       </c>
       <c r="H65" s="27" t="inlineStr">
         <is>
-          <t>Ankur Mahante</t>
+          <t>Hryday Goyal</t>
         </is>
       </c>
       <c r="I65" s="27" t="inlineStr">
@@ -7271,7 +7267,7 @@
       </c>
       <c r="J65" s="27" t="inlineStr">
         <is>
-          <t>Tanmay Sharma</t>
+          <t>Pranit Shriyan</t>
         </is>
       </c>
     </row>
@@ -7283,12 +7279,12 @@
       </c>
       <c r="B66" s="28" t="inlineStr">
         <is>
-          <t>7:05PM</t>
+          <t>5:00PM</t>
         </is>
       </c>
       <c r="C66" s="28" t="inlineStr">
         <is>
-          <t>7:20PM</t>
+          <t>5:15PM</t>
         </is>
       </c>
       <c r="D66" s="28" t="inlineStr">
@@ -7301,7 +7297,7 @@
       </c>
       <c r="F66" s="28" t="inlineStr">
         <is>
-          <t>U36-GA-9</t>
+          <t>U36-GA-1</t>
         </is>
       </c>
       <c r="G66" s="28" t="inlineStr">
@@ -7321,7 +7317,7 @@
       </c>
       <c r="J66" s="28" t="inlineStr">
         <is>
-          <t>Amar Parulekar</t>
+          <t>Ravi Modi</t>
         </is>
       </c>
     </row>
@@ -7333,17 +7329,17 @@
       </c>
       <c r="B67" s="27" t="inlineStr">
         <is>
-          <t>7:15PM</t>
+          <t>5:10PM</t>
         </is>
       </c>
       <c r="C67" s="27" t="inlineStr">
         <is>
-          <t>7:30PM</t>
+          <t>5:25PM</t>
         </is>
       </c>
       <c r="D67" s="27" t="inlineStr">
         <is>
-          <t>Under 46</t>
+          <t>Under 15</t>
         </is>
       </c>
       <c r="E67" s="27" t="n">
@@ -7351,7 +7347,7 @@
       </c>
       <c r="F67" s="27" t="inlineStr">
         <is>
-          <t>U46-GB-1</t>
+          <t>U15-GA-1</t>
         </is>
       </c>
       <c r="G67" s="27" t="inlineStr">
@@ -7361,7 +7357,7 @@
       </c>
       <c r="H67" s="27" t="inlineStr">
         <is>
-          <t>Mukul Joshi</t>
+          <t>Shaurya Tripathi</t>
         </is>
       </c>
       <c r="I67" s="27" t="inlineStr">
@@ -7371,7 +7367,7 @@
       </c>
       <c r="J67" s="27" t="inlineStr">
         <is>
-          <t>Vinod Agrawal</t>
+          <t>Parth yadav</t>
         </is>
       </c>
     </row>
@@ -7383,17 +7379,17 @@
       </c>
       <c r="B68" s="28" t="inlineStr">
         <is>
-          <t>7:40PM</t>
+          <t>5:15PM</t>
         </is>
       </c>
       <c r="C68" s="28" t="inlineStr">
         <is>
-          <t>7:55PM</t>
+          <t>5:30PM</t>
         </is>
       </c>
       <c r="D68" s="28" t="inlineStr">
         <is>
-          <t>Under 46</t>
+          <t>Under 15</t>
         </is>
       </c>
       <c r="E68" s="28" t="n">
@@ -7401,7 +7397,7 @@
       </c>
       <c r="F68" s="28" t="inlineStr">
         <is>
-          <t>U46-GB-2</t>
+          <t>U15-GB-1</t>
         </is>
       </c>
       <c r="G68" s="28" t="inlineStr">
@@ -7411,7 +7407,7 @@
       </c>
       <c r="H68" s="28" t="inlineStr">
         <is>
-          <t>Amit Ranka</t>
+          <t>Viaan Neema</t>
         </is>
       </c>
       <c r="I68" s="28" t="inlineStr">
@@ -7421,7 +7417,7 @@
       </c>
       <c r="J68" s="28" t="inlineStr">
         <is>
-          <t>Mukul Joshi</t>
+          <t>Yash agarwal</t>
         </is>
       </c>
     </row>
@@ -7433,17 +7429,17 @@
       </c>
       <c r="B69" s="27" t="inlineStr">
         <is>
-          <t>7:50PM</t>
+          <t>5:25PM</t>
         </is>
       </c>
       <c r="C69" s="27" t="inlineStr">
         <is>
-          <t>8:05PM</t>
+          <t>5:40PM</t>
         </is>
       </c>
       <c r="D69" s="27" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Under 26</t>
         </is>
       </c>
       <c r="E69" s="27" t="n">
@@ -7451,7 +7447,7 @@
       </c>
       <c r="F69" s="27" t="inlineStr">
         <is>
-          <t>U36-GB-8</t>
+          <t>U26-2</t>
         </is>
       </c>
       <c r="G69" s="27" t="inlineStr">
@@ -7461,7 +7457,7 @@
       </c>
       <c r="H69" s="27" t="inlineStr">
         <is>
-          <t>Tej</t>
+          <t>Yuvraj jain</t>
         </is>
       </c>
       <c r="I69" s="27" t="inlineStr">
@@ -7471,7 +7467,7 @@
       </c>
       <c r="J69" s="27" t="inlineStr">
         <is>
-          <t>Sudip Parui</t>
+          <t>Hryday Goyal</t>
         </is>
       </c>
     </row>
@@ -7483,17 +7479,17 @@
       </c>
       <c r="B70" s="28" t="inlineStr">
         <is>
-          <t>7:55PM</t>
+          <t>5:30PM</t>
         </is>
       </c>
       <c r="C70" s="28" t="inlineStr">
         <is>
-          <t>8:10PM</t>
+          <t>5:45PM</t>
         </is>
       </c>
       <c r="D70" s="28" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Under 26</t>
         </is>
       </c>
       <c r="E70" s="28" t="n">
@@ -7501,7 +7497,7 @@
       </c>
       <c r="F70" s="28" t="inlineStr">
         <is>
-          <t>U36-GA-10</t>
+          <t>U26-6</t>
         </is>
       </c>
       <c r="G70" s="28" t="inlineStr">
@@ -7511,7 +7507,7 @@
       </c>
       <c r="H70" s="28" t="inlineStr">
         <is>
-          <t>Ravi Modi</t>
+          <t>Aaditya Kumar</t>
         </is>
       </c>
       <c r="I70" s="28" t="inlineStr">
@@ -7521,7 +7517,7 @@
       </c>
       <c r="J70" s="28" t="inlineStr">
         <is>
-          <t>Prakshal Shah</t>
+          <t>Pranit Shriyan</t>
         </is>
       </c>
     </row>
@@ -7533,17 +7529,17 @@
       </c>
       <c r="B71" s="27" t="inlineStr">
         <is>
-          <t>8:05PM</t>
+          <t>5:40PM</t>
         </is>
       </c>
       <c r="C71" s="27" t="inlineStr">
         <is>
-          <t>8:20PM</t>
+          <t>5:55PM</t>
         </is>
       </c>
       <c r="D71" s="27" t="inlineStr">
         <is>
-          <t>Under 46</t>
+          <t>Under 15</t>
         </is>
       </c>
       <c r="E71" s="27" t="n">
@@ -7551,7 +7547,7 @@
       </c>
       <c r="F71" s="27" t="inlineStr">
         <is>
-          <t>U46-GA-1</t>
+          <t>U15-GB-3</t>
         </is>
       </c>
       <c r="G71" s="27" t="inlineStr">
@@ -7561,7 +7557,7 @@
       </c>
       <c r="H71" s="27" t="inlineStr">
         <is>
-          <t>Anuj Shah</t>
+          <t>Yash agarwal</t>
         </is>
       </c>
       <c r="I71" s="27" t="inlineStr">
@@ -7571,7 +7567,7 @@
       </c>
       <c r="J71" s="27" t="inlineStr">
         <is>
-          <t>Nikunj Jhala</t>
+          <t>Hridh jhala</t>
         </is>
       </c>
     </row>
@@ -7583,17 +7579,17 @@
       </c>
       <c r="B72" s="28" t="inlineStr">
         <is>
-          <t>8:20PM</t>
+          <t>5:45PM</t>
         </is>
       </c>
       <c r="C72" s="28" t="inlineStr">
         <is>
-          <t>8:35PM</t>
+          <t>6:00PM</t>
         </is>
       </c>
       <c r="D72" s="28" t="inlineStr">
         <is>
-          <t>Under 46</t>
+          <t>Under 36</t>
         </is>
       </c>
       <c r="E72" s="28" t="n">
@@ -7601,17 +7597,17 @@
       </c>
       <c r="F72" s="28" t="inlineStr">
         <is>
-          <t>U46-GB-3</t>
+          <t>U36-GA-2</t>
         </is>
       </c>
       <c r="G72" s="28" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H72" s="28" t="inlineStr">
         <is>
-          <t>Amit Ranka</t>
+          <t>Jashit Bajaj</t>
         </is>
       </c>
       <c r="I72" s="28" t="inlineStr">
@@ -7621,7 +7617,7 @@
       </c>
       <c r="J72" s="28" t="inlineStr">
         <is>
-          <t>Vinod Agrawal</t>
+          <t>Tapabrata Dutta</t>
         </is>
       </c>
     </row>
@@ -7633,17 +7629,17 @@
       </c>
       <c r="B73" s="27" t="inlineStr">
         <is>
-          <t>8:30PM</t>
+          <t>5:55PM</t>
         </is>
       </c>
       <c r="C73" s="27" t="inlineStr">
         <is>
-          <t>8:45PM</t>
+          <t>6:10PM</t>
         </is>
       </c>
       <c r="D73" s="27" t="inlineStr">
         <is>
-          <t>Under 46</t>
+          <t>Under 26</t>
         </is>
       </c>
       <c r="E73" s="27" t="n">
@@ -7651,17 +7647,17 @@
       </c>
       <c r="F73" s="27" t="inlineStr">
         <is>
-          <t>U46-GA-2</t>
+          <t>U26-3</t>
         </is>
       </c>
       <c r="G73" s="27" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H73" s="27" t="inlineStr">
         <is>
-          <t>Nikunj Jhala</t>
+          <t>Yuvraj jain</t>
         </is>
       </c>
       <c r="I73" s="27" t="inlineStr">
@@ -7671,7 +7667,7 @@
       </c>
       <c r="J73" s="27" t="inlineStr">
         <is>
-          <t>Nilesh Bagaria</t>
+          <t>Pranit Shriyan</t>
         </is>
       </c>
     </row>
@@ -7683,17 +7679,17 @@
       </c>
       <c r="B74" s="28" t="inlineStr">
         <is>
-          <t>8:35PM</t>
+          <t>6:00PM</t>
         </is>
       </c>
       <c r="C74" s="28" t="inlineStr">
         <is>
-          <t>8:50PM</t>
+          <t>6:15PM</t>
         </is>
       </c>
       <c r="D74" s="28" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Under 26</t>
         </is>
       </c>
       <c r="E74" s="28" t="n">
@@ -7701,17 +7697,17 @@
       </c>
       <c r="F74" s="28" t="inlineStr">
         <is>
-          <t>U36-GB-9</t>
+          <t>U26-5</t>
         </is>
       </c>
       <c r="G74" s="28" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H74" s="28" t="inlineStr">
         <is>
-          <t>Dr Rahul Modi</t>
+          <t>Aaditya Kumar</t>
         </is>
       </c>
       <c r="I74" s="28" t="inlineStr">
@@ -7721,7 +7717,7 @@
       </c>
       <c r="J74" s="28" t="inlineStr">
         <is>
-          <t>Sudip Parui</t>
+          <t>Hryday Goyal</t>
         </is>
       </c>
     </row>
@@ -7733,12 +7729,12 @@
       </c>
       <c r="B75" s="27" t="inlineStr">
         <is>
-          <t>8:45PM</t>
+          <t>6:10PM</t>
         </is>
       </c>
       <c r="C75" s="27" t="inlineStr">
         <is>
-          <t>9:00PM</t>
+          <t>6:25PM</t>
         </is>
       </c>
       <c r="D75" s="27" t="inlineStr">
@@ -7751,17 +7747,17 @@
       </c>
       <c r="F75" s="27" t="inlineStr">
         <is>
-          <t>U36-GB-10</t>
+          <t>U36-GB-1</t>
         </is>
       </c>
       <c r="G75" s="27" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H75" s="27" t="inlineStr">
         <is>
-          <t>Tej</t>
+          <t>Prakshal Shah</t>
         </is>
       </c>
       <c r="I75" s="27" t="inlineStr">
@@ -7771,7 +7767,7 @@
       </c>
       <c r="J75" s="27" t="inlineStr">
         <is>
-          <t>Tanmay Sharma</t>
+          <t>Amar Parulekar</t>
         </is>
       </c>
     </row>
@@ -7783,17 +7779,17 @@
       </c>
       <c r="B76" s="28" t="inlineStr">
         <is>
-          <t>8:50PM</t>
+          <t>6:15PM</t>
         </is>
       </c>
       <c r="C76" s="28" t="inlineStr">
         <is>
-          <t>9:05PM</t>
+          <t>6:30PM</t>
         </is>
       </c>
       <c r="D76" s="28" t="inlineStr">
         <is>
-          <t>Under 15</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E76" s="28" t="n">
@@ -7801,17 +7797,17 @@
       </c>
       <c r="F76" s="28" t="inlineStr">
         <is>
-          <t>U15-GA-1</t>
+          <t>U46-GA-1</t>
         </is>
       </c>
       <c r="G76" s="28" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H76" s="28" t="inlineStr">
         <is>
-          <t>Shaurya Tripathi</t>
+          <t>Dr Rahul Modi</t>
         </is>
       </c>
       <c r="I76" s="28" t="inlineStr">
@@ -7821,7 +7817,7 @@
       </c>
       <c r="J76" s="28" t="inlineStr">
         <is>
-          <t>Parth yadav</t>
+          <t>Ankur Mahante</t>
         </is>
       </c>
     </row>
@@ -7833,17 +7829,17 @@
       </c>
       <c r="B77" s="27" t="inlineStr">
         <is>
-          <t>9:00PM</t>
+          <t>6:25PM</t>
         </is>
       </c>
       <c r="C77" s="27" t="inlineStr">
         <is>
-          <t>9:15PM</t>
+          <t>6:40PM</t>
         </is>
       </c>
       <c r="D77" s="27" t="inlineStr">
         <is>
-          <t>Under 46</t>
+          <t>Under 26</t>
         </is>
       </c>
       <c r="E77" s="27" t="n">
@@ -7851,17 +7847,17 @@
       </c>
       <c r="F77" s="27" t="inlineStr">
         <is>
-          <t>U46-GA-3</t>
+          <t>U26-4</t>
         </is>
       </c>
       <c r="G77" s="27" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H77" s="27" t="inlineStr">
         <is>
-          <t>Vinit Padia</t>
+          <t>Yuvraj jain</t>
         </is>
       </c>
       <c r="I77" s="27" t="inlineStr">
@@ -7871,7 +7867,7 @@
       </c>
       <c r="J77" s="27" t="inlineStr">
         <is>
-          <t>Nilesh Bagaria</t>
+          <t>Rahul Garg</t>
         </is>
       </c>
     </row>
@@ -7883,17 +7879,17 @@
       </c>
       <c r="B78" s="28" t="inlineStr">
         <is>
-          <t>9:25PM</t>
+          <t>6:30PM</t>
         </is>
       </c>
       <c r="C78" s="28" t="inlineStr">
         <is>
-          <t>9:40PM</t>
+          <t>6:45PM</t>
         </is>
       </c>
       <c r="D78" s="28" t="inlineStr">
         <is>
-          <t>Under 46</t>
+          <t>Under 36</t>
         </is>
       </c>
       <c r="E78" s="28" t="n">
@@ -7901,7 +7897,7 @@
       </c>
       <c r="F78" s="28" t="inlineStr">
         <is>
-          <t>U46-GB-4</t>
+          <t>U36-GA-3</t>
         </is>
       </c>
       <c r="G78" s="28" t="inlineStr">
@@ -7911,7 +7907,7 @@
       </c>
       <c r="H78" s="28" t="inlineStr">
         <is>
-          <t>Adil Khan</t>
+          <t>Ravi Modi</t>
         </is>
       </c>
       <c r="I78" s="28" t="inlineStr">
@@ -7921,7 +7917,7 @@
       </c>
       <c r="J78" s="28" t="inlineStr">
         <is>
-          <t>Vinod Agrawal</t>
+          <t>Tapabrata Dutta</t>
         </is>
       </c>
     </row>
@@ -7933,12 +7929,12 @@
       </c>
       <c r="B79" s="27" t="inlineStr">
         <is>
-          <t>9:25PM</t>
+          <t>6:40PM</t>
         </is>
       </c>
       <c r="C79" s="27" t="inlineStr">
         <is>
-          <t>9:40PM</t>
+          <t>6:55PM</t>
         </is>
       </c>
       <c r="D79" s="27" t="inlineStr">
@@ -7951,7 +7947,7 @@
       </c>
       <c r="F79" s="27" t="inlineStr">
         <is>
-          <t>U46-GA-4</t>
+          <t>U46-GA-2</t>
         </is>
       </c>
       <c r="G79" s="27" t="inlineStr">
@@ -7961,7 +7957,7 @@
       </c>
       <c r="H79" s="27" t="inlineStr">
         <is>
-          <t>Anuj Shah</t>
+          <t>Dr Rahul Modi</t>
         </is>
       </c>
       <c r="I79" s="27" t="inlineStr">
@@ -7971,7 +7967,7 @@
       </c>
       <c r="J79" s="27" t="inlineStr">
         <is>
-          <t>Nilesh Bagaria</t>
+          <t>Sudip Parui</t>
         </is>
       </c>
     </row>
@@ -7983,17 +7979,17 @@
       </c>
       <c r="B80" s="28" t="inlineStr">
         <is>
-          <t>9:40PM</t>
+          <t>6:45PM</t>
         </is>
       </c>
       <c r="C80" s="28" t="inlineStr">
         <is>
-          <t>9:55PM</t>
+          <t>7:00PM</t>
         </is>
       </c>
       <c r="D80" s="28" t="inlineStr">
         <is>
-          <t>Under 15</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E80" s="28" t="n">
@@ -8001,17 +7997,17 @@
       </c>
       <c r="F80" s="28" t="inlineStr">
         <is>
-          <t>U15-GB-1</t>
+          <t>U46-GA-6</t>
         </is>
       </c>
       <c r="G80" s="28" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H80" s="28" t="inlineStr">
         <is>
-          <t>Viaan Neema</t>
+          <t>Ankur Mahante</t>
         </is>
       </c>
       <c r="I80" s="28" t="inlineStr">
@@ -8021,7 +8017,7 @@
       </c>
       <c r="J80" s="28" t="inlineStr">
         <is>
-          <t>Yash agarwal</t>
+          <t>Tanmay Sharma</t>
         </is>
       </c>
     </row>
@@ -8033,12 +8029,12 @@
       </c>
       <c r="B81" s="27" t="inlineStr">
         <is>
-          <t>9:50PM</t>
+          <t>6:55PM</t>
         </is>
       </c>
       <c r="C81" s="27" t="inlineStr">
         <is>
-          <t>10:05PM</t>
+          <t>7:10PM</t>
         </is>
       </c>
       <c r="D81" s="27" t="inlineStr">
@@ -8051,17 +8047,17 @@
       </c>
       <c r="F81" s="27" t="inlineStr">
         <is>
-          <t>U46-GB-5</t>
+          <t>U46-GB-8</t>
         </is>
       </c>
       <c r="G81" s="27" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H81" s="27" t="inlineStr">
         <is>
-          <t>Amit Ranka</t>
+          <t>Vinit Padia</t>
         </is>
       </c>
       <c r="I81" s="27" t="inlineStr">
@@ -8071,7 +8067,7 @@
       </c>
       <c r="J81" s="27" t="inlineStr">
         <is>
-          <t>Adil Khan</t>
+          <t>Nilesh Bagaria</t>
         </is>
       </c>
     </row>
@@ -8083,17 +8079,17 @@
       </c>
       <c r="B82" s="28" t="inlineStr">
         <is>
-          <t>9:55PM</t>
+          <t>7:05PM</t>
         </is>
       </c>
       <c r="C82" s="28" t="inlineStr">
         <is>
-          <t>10:10PM</t>
+          <t>7:20PM</t>
         </is>
       </c>
       <c r="D82" s="28" t="inlineStr">
         <is>
-          <t>Under 15</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E82" s="28" t="n">
@@ -8101,17 +8097,17 @@
       </c>
       <c r="F82" s="28" t="inlineStr">
         <is>
-          <t>U15-GA-2</t>
+          <t>U46-GA-4</t>
         </is>
       </c>
       <c r="G82" s="28" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H82" s="28" t="inlineStr">
         <is>
-          <t>Shaurya Tripathi</t>
+          <t>Dr Rahul Modi</t>
         </is>
       </c>
       <c r="I82" s="28" t="inlineStr">
@@ -8121,24 +8117,24 @@
       </c>
       <c r="J82" s="28" t="inlineStr">
         <is>
-          <t>Aadit Joshi</t>
+          <t>Anuj Shah</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="27" t="inlineStr">
         <is>
-          <t>Aug 16</t>
+          <t>Aug 15</t>
         </is>
       </c>
       <c r="B83" s="27" t="inlineStr">
         <is>
-          <t>8:00AM</t>
+          <t>7:10PM</t>
         </is>
       </c>
       <c r="C83" s="27" t="inlineStr">
         <is>
-          <t>8:15AM</t>
+          <t>7:25PM</t>
         </is>
       </c>
       <c r="D83" s="27" t="inlineStr">
@@ -8151,17 +8147,17 @@
       </c>
       <c r="F83" s="27" t="inlineStr">
         <is>
-          <t>U46-GB-6</t>
+          <t>U46-GA-5</t>
         </is>
       </c>
       <c r="G83" s="27" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H83" s="27" t="inlineStr">
         <is>
-          <t>Mukul Joshi</t>
+          <t>Ankur Mahante</t>
         </is>
       </c>
       <c r="I83" s="27" t="inlineStr">
@@ -8171,29 +8167,29 @@
       </c>
       <c r="J83" s="27" t="inlineStr">
         <is>
-          <t>Adil Khan</t>
+          <t>Sudip Parui</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="28" t="inlineStr">
         <is>
-          <t>Aug 16</t>
+          <t>Aug 15</t>
         </is>
       </c>
       <c r="B84" s="28" t="inlineStr">
         <is>
-          <t>8:00AM</t>
+          <t>7:35PM</t>
         </is>
       </c>
       <c r="C84" s="28" t="inlineStr">
         <is>
-          <t>8:15AM</t>
+          <t>7:50PM</t>
         </is>
       </c>
       <c r="D84" s="28" t="inlineStr">
         <is>
-          <t>Under 15</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E84" s="28" t="n">
@@ -8201,17 +8197,17 @@
       </c>
       <c r="F84" s="28" t="inlineStr">
         <is>
-          <t>U15-GA-3</t>
+          <t>U46-GA-7</t>
         </is>
       </c>
       <c r="G84" s="28" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H84" s="28" t="inlineStr">
         <is>
-          <t>Parth yadav</t>
+          <t>Ankur Mahante</t>
         </is>
       </c>
       <c r="I84" s="28" t="inlineStr">
@@ -8221,29 +8217,29 @@
       </c>
       <c r="J84" s="28" t="inlineStr">
         <is>
-          <t>Aadit Joshi</t>
+          <t>Anuj Shah</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="27" t="inlineStr">
         <is>
-          <t>Aug 16</t>
+          <t>Aug 15</t>
         </is>
       </c>
       <c r="B85" s="27" t="inlineStr">
         <is>
-          <t>8:15AM</t>
+          <t>7:40PM</t>
         </is>
       </c>
       <c r="C85" s="27" t="inlineStr">
         <is>
-          <t>8:30AM</t>
+          <t>7:55PM</t>
         </is>
       </c>
       <c r="D85" s="27" t="inlineStr">
         <is>
-          <t>Under 46</t>
+          <t>Under 26</t>
         </is>
       </c>
       <c r="E85" s="27" t="n">
@@ -8251,17 +8247,17 @@
       </c>
       <c r="F85" s="27" t="inlineStr">
         <is>
-          <t>U46-GA-5</t>
+          <t>U26-10</t>
         </is>
       </c>
       <c r="G85" s="27" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H85" s="27" t="inlineStr">
         <is>
-          <t>Piyush Makharia</t>
+          <t>Pranit Shriyan</t>
         </is>
       </c>
       <c r="I85" s="27" t="inlineStr">
@@ -8271,24 +8267,24 @@
       </c>
       <c r="J85" s="27" t="inlineStr">
         <is>
-          <t>Vinit Padia</t>
+          <t>Rahul Garg</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="28" t="inlineStr">
         <is>
-          <t>Aug 16</t>
+          <t>Aug 15</t>
         </is>
       </c>
       <c r="B86" s="28" t="inlineStr">
         <is>
-          <t>8:40AM</t>
+          <t>7:50PM</t>
         </is>
       </c>
       <c r="C86" s="28" t="inlineStr">
         <is>
-          <t>8:55AM</t>
+          <t>8:05PM</t>
         </is>
       </c>
       <c r="D86" s="28" t="inlineStr">
@@ -8301,7 +8297,7 @@
       </c>
       <c r="F86" s="28" t="inlineStr">
         <is>
-          <t>U46-GA-6</t>
+          <t>U46-GB-9</t>
         </is>
       </c>
       <c r="G86" s="28" t="inlineStr">
@@ -8311,7 +8307,7 @@
       </c>
       <c r="H86" s="28" t="inlineStr">
         <is>
-          <t>Anuj Shah</t>
+          <t>Vinit Padia</t>
         </is>
       </c>
       <c r="I86" s="28" t="inlineStr">
@@ -8321,29 +8317,29 @@
       </c>
       <c r="J86" s="28" t="inlineStr">
         <is>
-          <t>Piyush Makharia</t>
+          <t>Amit Ranka</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="27" t="inlineStr">
         <is>
-          <t>Aug 16</t>
+          <t>Aug 15</t>
         </is>
       </c>
       <c r="B87" s="27" t="inlineStr">
         <is>
-          <t>8:40AM</t>
+          <t>8:00PM</t>
         </is>
       </c>
       <c r="C87" s="27" t="inlineStr">
         <is>
-          <t>8:55AM</t>
+          <t>8:15PM</t>
         </is>
       </c>
       <c r="D87" s="27" t="inlineStr">
         <is>
-          <t>Under 46</t>
+          <t>Under 36</t>
         </is>
       </c>
       <c r="E87" s="27" t="n">
@@ -8351,7 +8347,7 @@
       </c>
       <c r="F87" s="27" t="inlineStr">
         <is>
-          <t>U46-GA-7</t>
+          <t>U36-GB-2</t>
         </is>
       </c>
       <c r="G87" s="27" t="inlineStr">
@@ -8361,7 +8357,7 @@
       </c>
       <c r="H87" s="27" t="inlineStr">
         <is>
-          <t>Nikunj Jhala</t>
+          <t>Prakshal Shah</t>
         </is>
       </c>
       <c r="I87" s="27" t="inlineStr">
@@ -8371,29 +8367,29 @@
       </c>
       <c r="J87" s="27" t="inlineStr">
         <is>
-          <t>Vinit Padia</t>
+          <t>Tej</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="28" t="inlineStr">
         <is>
-          <t>Aug 16</t>
+          <t>Aug 15</t>
         </is>
       </c>
       <c r="B88" s="28" t="inlineStr">
         <is>
-          <t>9:05AM</t>
+          <t>8:05PM</t>
         </is>
       </c>
       <c r="C88" s="28" t="inlineStr">
         <is>
-          <t>9:20AM</t>
+          <t>8:20PM</t>
         </is>
       </c>
       <c r="D88" s="28" t="inlineStr">
         <is>
-          <t>Under 46</t>
+          <t>Under 26</t>
         </is>
       </c>
       <c r="E88" s="28" t="n">
@@ -8401,7 +8397,7 @@
       </c>
       <c r="F88" s="28" t="inlineStr">
         <is>
-          <t>U46-GA-8</t>
+          <t>U26-7</t>
         </is>
       </c>
       <c r="G88" s="28" t="inlineStr">
@@ -8411,7 +8407,7 @@
       </c>
       <c r="H88" s="28" t="inlineStr">
         <is>
-          <t>Nikunj Jhala</t>
+          <t>Aaditya Kumar</t>
         </is>
       </c>
       <c r="I88" s="28" t="inlineStr">
@@ -8421,24 +8417,24 @@
       </c>
       <c r="J88" s="28" t="inlineStr">
         <is>
-          <t>Piyush Makharia</t>
+          <t>Rahul Garg</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="27" t="inlineStr">
         <is>
-          <t>Aug 16</t>
+          <t>Aug 15</t>
         </is>
       </c>
       <c r="B89" s="27" t="inlineStr">
         <is>
-          <t>9:05AM</t>
+          <t>8:15PM</t>
         </is>
       </c>
       <c r="C89" s="27" t="inlineStr">
         <is>
-          <t>9:20AM</t>
+          <t>8:30PM</t>
         </is>
       </c>
       <c r="D89" s="27" t="inlineStr">
@@ -8451,7 +8447,7 @@
       </c>
       <c r="F89" s="27" t="inlineStr">
         <is>
-          <t>U46-GA-9</t>
+          <t>U46-GA-3</t>
         </is>
       </c>
       <c r="G89" s="27" t="inlineStr">
@@ -8461,7 +8457,7 @@
       </c>
       <c r="H89" s="27" t="inlineStr">
         <is>
-          <t>Anuj Shah</t>
+          <t>Dr Rahul Modi</t>
         </is>
       </c>
       <c r="I89" s="27" t="inlineStr">
@@ -8471,29 +8467,29 @@
       </c>
       <c r="J89" s="27" t="inlineStr">
         <is>
-          <t>Vinit Padia</t>
+          <t>Tanmay Sharma</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="28" t="inlineStr">
         <is>
-          <t>Aug 16</t>
+          <t>Aug 15</t>
         </is>
       </c>
       <c r="B90" s="28" t="inlineStr">
         <is>
-          <t>9:20AM</t>
+          <t>8:20PM</t>
         </is>
       </c>
       <c r="C90" s="28" t="inlineStr">
         <is>
-          <t>9:35AM</t>
+          <t>8:35PM</t>
         </is>
       </c>
       <c r="D90" s="28" t="inlineStr">
         <is>
-          <t>Under 15</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E90" s="28" t="n">
@@ -8501,17 +8497,17 @@
       </c>
       <c r="F90" s="28" t="inlineStr">
         <is>
-          <t>U15-GB-2</t>
+          <t>U46-GA-9</t>
         </is>
       </c>
       <c r="G90" s="28" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H90" s="28" t="inlineStr">
         <is>
-          <t>Viaan Neema</t>
+          <t>Sudip Parui</t>
         </is>
       </c>
       <c r="I90" s="28" t="inlineStr">
@@ -8521,29 +8517,29 @@
       </c>
       <c r="J90" s="28" t="inlineStr">
         <is>
-          <t>Hridh jhala</t>
+          <t>Anuj Shah</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="27" t="inlineStr">
         <is>
-          <t>Aug 16</t>
+          <t>Aug 15</t>
         </is>
       </c>
       <c r="B91" s="27" t="inlineStr">
         <is>
-          <t>9:30AM</t>
+          <t>8:30PM</t>
         </is>
       </c>
       <c r="C91" s="27" t="inlineStr">
         <is>
-          <t>9:45AM</t>
+          <t>8:45PM</t>
         </is>
       </c>
       <c r="D91" s="27" t="inlineStr">
         <is>
-          <t>Under 46</t>
+          <t>Under 36</t>
         </is>
       </c>
       <c r="E91" s="27" t="n">
@@ -8551,17 +8547,17 @@
       </c>
       <c r="F91" s="27" t="inlineStr">
         <is>
-          <t>U46-GA-10</t>
+          <t>U36-GB-3</t>
         </is>
       </c>
       <c r="G91" s="27" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H91" s="27" t="inlineStr">
         <is>
-          <t>Piyush Makharia</t>
+          <t>Amar Parulekar</t>
         </is>
       </c>
       <c r="I91" s="27" t="inlineStr">
@@ -8571,29 +8567,29 @@
       </c>
       <c r="J91" s="27" t="inlineStr">
         <is>
-          <t>Nilesh Bagaria</t>
+          <t>Tej</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="28" t="inlineStr">
         <is>
-          <t>Aug 16</t>
+          <t>Aug 15</t>
         </is>
       </c>
       <c r="B92" s="28" t="inlineStr">
         <is>
-          <t>9:35AM</t>
+          <t>8:35PM</t>
         </is>
       </c>
       <c r="C92" s="28" t="inlineStr">
         <is>
-          <t>9:50AM</t>
+          <t>8:50PM</t>
         </is>
       </c>
       <c r="D92" s="28" t="inlineStr">
         <is>
-          <t>Under 32</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E92" s="28" t="n">
@@ -8601,17 +8597,17 @@
       </c>
       <c r="F92" s="28" t="inlineStr">
         <is>
-          <t>U32-1</t>
+          <t>U46-GB-3</t>
         </is>
       </c>
       <c r="G92" s="28" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H92" s="28" t="inlineStr">
         <is>
-          <t>Yuvraj jain</t>
+          <t>Nikunj Jhala</t>
         </is>
       </c>
       <c r="I92" s="28" t="inlineStr">
@@ -8621,29 +8617,29 @@
       </c>
       <c r="J92" s="28" t="inlineStr">
         <is>
-          <t>Aaditya Kumar</t>
+          <t>Nilesh Bagaria</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="27" t="inlineStr">
         <is>
-          <t>Aug 16</t>
+          <t>Aug 15</t>
         </is>
       </c>
       <c r="B93" s="27" t="inlineStr">
         <is>
-          <t>9:45AM</t>
+          <t>8:45PM</t>
         </is>
       </c>
       <c r="C93" s="27" t="inlineStr">
         <is>
-          <t>10:00AM</t>
+          <t>9:00PM</t>
         </is>
       </c>
       <c r="D93" s="27" t="inlineStr">
         <is>
-          <t>Under 15</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E93" s="27" t="n">
@@ -8651,17 +8647,17 @@
       </c>
       <c r="F93" s="27" t="inlineStr">
         <is>
-          <t>U15-GB-3</t>
+          <t>U46-GA-8</t>
         </is>
       </c>
       <c r="G93" s="27" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H93" s="27" t="inlineStr">
         <is>
-          <t>Yash agarwal</t>
+          <t>Sudip Parui</t>
         </is>
       </c>
       <c r="I93" s="27" t="inlineStr">
@@ -8671,29 +8667,29 @@
       </c>
       <c r="J93" s="27" t="inlineStr">
         <is>
-          <t>Hridh jhala</t>
+          <t>Tanmay Sharma</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="28" t="inlineStr">
         <is>
-          <t>Aug 16</t>
+          <t>Aug 15</t>
         </is>
       </c>
       <c r="B94" s="28" t="inlineStr">
         <is>
-          <t>10:00AM</t>
+          <t>9:00PM</t>
         </is>
       </c>
       <c r="C94" s="28" t="inlineStr">
         <is>
-          <t>10:15AM</t>
+          <t>9:15PM</t>
         </is>
       </c>
       <c r="D94" s="28" t="inlineStr">
         <is>
-          <t>Under 32</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E94" s="28" t="n">
@@ -8701,7 +8697,7 @@
       </c>
       <c r="F94" s="28" t="inlineStr">
         <is>
-          <t>U32-3</t>
+          <t>U46-GB-4</t>
         </is>
       </c>
       <c r="G94" s="28" t="inlineStr">
@@ -8711,7 +8707,7 @@
       </c>
       <c r="H94" s="28" t="inlineStr">
         <is>
-          <t>Hryday Goyal</t>
+          <t>Nikunj Jhala</t>
         </is>
       </c>
       <c r="I94" s="28" t="inlineStr">
@@ -8721,29 +8717,29 @@
       </c>
       <c r="J94" s="28" t="inlineStr">
         <is>
-          <t>Pranit Shriyan</t>
+          <t>Amit Ranka</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="27" t="inlineStr">
         <is>
-          <t>Aug 16</t>
+          <t>Aug 15</t>
         </is>
       </c>
       <c r="B95" s="27" t="inlineStr">
         <is>
-          <t>10:00AM</t>
+          <t>9:10PM</t>
         </is>
       </c>
       <c r="C95" s="27" t="inlineStr">
         <is>
-          <t>10:15AM</t>
+          <t>9:25PM</t>
         </is>
       </c>
       <c r="D95" s="27" t="inlineStr">
         <is>
-          <t>Under 32</t>
+          <t>Under 26</t>
         </is>
       </c>
       <c r="E95" s="27" t="n">
@@ -8751,7 +8747,7 @@
       </c>
       <c r="F95" s="27" t="inlineStr">
         <is>
-          <t>U32-2</t>
+          <t>U26-9</t>
         </is>
       </c>
       <c r="G95" s="27" t="inlineStr">
@@ -8761,7 +8757,7 @@
       </c>
       <c r="H95" s="27" t="inlineStr">
         <is>
-          <t>Yuvraj jain</t>
+          <t>Hryday Goyal</t>
         </is>
       </c>
       <c r="I95" s="27" t="inlineStr">
@@ -8778,22 +8774,22 @@
     <row r="96">
       <c r="A96" s="28" t="inlineStr">
         <is>
-          <t>Aug 16</t>
+          <t>Aug 15</t>
         </is>
       </c>
       <c r="B96" s="28" t="inlineStr">
         <is>
-          <t>10:25AM</t>
+          <t>9:15PM</t>
         </is>
       </c>
       <c r="C96" s="28" t="inlineStr">
         <is>
-          <t>10:40AM</t>
+          <t>9:30PM</t>
         </is>
       </c>
       <c r="D96" s="28" t="inlineStr">
         <is>
-          <t>Under 32</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E96" s="28" t="n">
@@ -8801,17 +8797,17 @@
       </c>
       <c r="F96" s="28" t="inlineStr">
         <is>
-          <t>U32-4</t>
+          <t>U46-GA-10</t>
         </is>
       </c>
       <c r="G96" s="28" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H96" s="28" t="inlineStr">
         <is>
-          <t>Yuvraj jain</t>
+          <t>Tanmay Sharma</t>
         </is>
       </c>
       <c r="I96" s="28" t="inlineStr">
@@ -8821,29 +8817,29 @@
       </c>
       <c r="J96" s="28" t="inlineStr">
         <is>
-          <t>Hryday Goyal</t>
+          <t>Anuj Shah</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="27" t="inlineStr">
         <is>
-          <t>Aug 16</t>
+          <t>Aug 15</t>
         </is>
       </c>
       <c r="B97" s="27" t="inlineStr">
         <is>
-          <t>10:40AM</t>
+          <t>9:25PM</t>
         </is>
       </c>
       <c r="C97" s="27" t="inlineStr">
         <is>
-          <t>10:55AM</t>
+          <t>9:40PM</t>
         </is>
       </c>
       <c r="D97" s="27" t="inlineStr">
         <is>
-          <t>Under 32</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E97" s="27" t="n">
@@ -8851,7 +8847,7 @@
       </c>
       <c r="F97" s="27" t="inlineStr">
         <is>
-          <t>U32-5</t>
+          <t>U46-GB-10</t>
         </is>
       </c>
       <c r="G97" s="27" t="inlineStr">
@@ -8861,7 +8857,7 @@
       </c>
       <c r="H97" s="27" t="inlineStr">
         <is>
-          <t>Aaditya Kumar</t>
+          <t>Nilesh Bagaria</t>
         </is>
       </c>
       <c r="I97" s="27" t="inlineStr">
@@ -8871,7 +8867,7 @@
       </c>
       <c r="J97" s="27" t="inlineStr">
         <is>
-          <t>Pranit Shriyan</t>
+          <t>Amit Ranka</t>
         </is>
       </c>
     </row>
@@ -8883,17 +8879,17 @@
       </c>
       <c r="B98" s="28" t="inlineStr">
         <is>
-          <t>10:50AM</t>
+          <t>8:00AM</t>
         </is>
       </c>
       <c r="C98" s="28" t="inlineStr">
         <is>
-          <t>11:05AM</t>
+          <t>8:15AM</t>
         </is>
       </c>
       <c r="D98" s="28" t="inlineStr">
         <is>
-          <t>Under 32</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E98" s="28" t="n">
@@ -8901,7 +8897,7 @@
       </c>
       <c r="F98" s="28" t="inlineStr">
         <is>
-          <t>U32-6</t>
+          <t>U46-GB-1</t>
         </is>
       </c>
       <c r="G98" s="28" t="inlineStr">
@@ -8911,7 +8907,7 @@
       </c>
       <c r="H98" s="28" t="inlineStr">
         <is>
-          <t>Hryday Goyal</t>
+          <t>Nikunj Jhala</t>
         </is>
       </c>
       <c r="I98" s="28" t="inlineStr">
@@ -8921,7 +8917,7 @@
       </c>
       <c r="J98" s="28" t="inlineStr">
         <is>
-          <t>Rahul Garg</t>
+          <t>Piyush Makharia</t>
         </is>
       </c>
     </row>
@@ -8933,17 +8929,17 @@
       </c>
       <c r="B99" s="27" t="inlineStr">
         <is>
-          <t>11:05AM</t>
+          <t>8:25AM</t>
         </is>
       </c>
       <c r="C99" s="27" t="inlineStr">
         <is>
-          <t>11:20AM</t>
+          <t>8:40AM</t>
         </is>
       </c>
       <c r="D99" s="27" t="inlineStr">
         <is>
-          <t>Under 32</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E99" s="27" t="n">
@@ -8951,17 +8947,17 @@
       </c>
       <c r="F99" s="27" t="inlineStr">
         <is>
-          <t>U32-7</t>
+          <t>U46-GB-2</t>
         </is>
       </c>
       <c r="G99" s="27" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H99" s="27" t="inlineStr">
         <is>
-          <t>Yuvraj jain</t>
+          <t>Nikunj Jhala</t>
         </is>
       </c>
       <c r="I99" s="27" t="inlineStr">
@@ -8971,7 +8967,7 @@
       </c>
       <c r="J99" s="27" t="inlineStr">
         <is>
-          <t>Pranit Shriyan</t>
+          <t>Vinit Padia</t>
         </is>
       </c>
     </row>
@@ -8983,17 +8979,17 @@
       </c>
       <c r="B100" s="28" t="inlineStr">
         <is>
-          <t>11:15AM</t>
+          <t>8:25AM</t>
         </is>
       </c>
       <c r="C100" s="28" t="inlineStr">
         <is>
-          <t>11:30AM</t>
+          <t>8:40AM</t>
         </is>
       </c>
       <c r="D100" s="28" t="inlineStr">
         <is>
-          <t>Under 32</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E100" s="28" t="n">
@@ -9001,17 +8997,17 @@
       </c>
       <c r="F100" s="28" t="inlineStr">
         <is>
-          <t>U32-8</t>
+          <t>U46-GB-6</t>
         </is>
       </c>
       <c r="G100" s="28" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H100" s="28" t="inlineStr">
         <is>
-          <t>Aaditya Kumar</t>
+          <t>Piyush Makharia</t>
         </is>
       </c>
       <c r="I100" s="28" t="inlineStr">
@@ -9021,7 +9017,7 @@
       </c>
       <c r="J100" s="28" t="inlineStr">
         <is>
-          <t>Rahul Garg</t>
+          <t>Nilesh Bagaria</t>
         </is>
       </c>
     </row>
@@ -9033,17 +9029,17 @@
       </c>
       <c r="B101" s="27" t="inlineStr">
         <is>
-          <t>11:40AM</t>
+          <t>8:50AM</t>
         </is>
       </c>
       <c r="C101" s="27" t="inlineStr">
         <is>
-          <t>11:55AM</t>
+          <t>9:05AM</t>
         </is>
       </c>
       <c r="D101" s="27" t="inlineStr">
         <is>
-          <t>Under 32</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E101" s="27" t="n">
@@ -9051,7 +9047,7 @@
       </c>
       <c r="F101" s="27" t="inlineStr">
         <is>
-          <t>U32-10</t>
+          <t>U46-GB-5</t>
         </is>
       </c>
       <c r="G101" s="27" t="inlineStr">
@@ -9061,7 +9057,7 @@
       </c>
       <c r="H101" s="27" t="inlineStr">
         <is>
-          <t>Aaditya Kumar</t>
+          <t>Piyush Makharia</t>
         </is>
       </c>
       <c r="I101" s="27" t="inlineStr">
@@ -9071,7 +9067,7 @@
       </c>
       <c r="J101" s="27" t="inlineStr">
         <is>
-          <t>Hryday Goyal</t>
+          <t>Vinit Padia</t>
         </is>
       </c>
     </row>
@@ -9083,17 +9079,17 @@
       </c>
       <c r="B102" s="28" t="inlineStr">
         <is>
-          <t>11:40AM</t>
+          <t>9:15AM</t>
         </is>
       </c>
       <c r="C102" s="28" t="inlineStr">
         <is>
-          <t>11:55AM</t>
+          <t>9:30AM</t>
         </is>
       </c>
       <c r="D102" s="28" t="inlineStr">
         <is>
-          <t>Under 32</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E102" s="28" t="n">
@@ -9101,17 +9097,17 @@
       </c>
       <c r="F102" s="28" t="inlineStr">
         <is>
-          <t>U32-9</t>
+          <t>U46-GB-7</t>
         </is>
       </c>
       <c r="G102" s="28" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H102" s="28" t="inlineStr">
         <is>
-          <t>Pranit Shriyan</t>
+          <t>Piyush Makharia</t>
         </is>
       </c>
       <c r="I102" s="28" t="inlineStr">
@@ -9121,7 +9117,7 @@
       </c>
       <c r="J102" s="28" t="inlineStr">
         <is>
-          <t>Rahul Garg</t>
+          <t>Amit Ranka</t>
         </is>
       </c>
     </row>
@@ -9133,17 +9129,17 @@
       </c>
       <c r="B103" s="27" t="inlineStr">
         <is>
-          <t>3:20PM</t>
+          <t>3:50PM</t>
         </is>
       </c>
       <c r="C103" s="27" t="inlineStr">
         <is>
-          <t>3:35PM</t>
+          <t>4:05PM</t>
         </is>
       </c>
       <c r="D103" s="27" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Under 15</t>
         </is>
       </c>
       <c r="E103" s="27" t="n">
@@ -9151,7 +9147,7 @@
       </c>
       <c r="F103" s="27" t="inlineStr">
         <is>
-          <t>SR-SF1</t>
+          <t>U15-SF1</t>
         </is>
       </c>
       <c r="G103" s="27" t="inlineStr">
@@ -9183,17 +9179,17 @@
       </c>
       <c r="B104" s="28" t="inlineStr">
         <is>
-          <t>3:35PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="C104" s="28" t="inlineStr">
         <is>
-          <t>3:50PM</t>
+          <t>4:15PM</t>
         </is>
       </c>
       <c r="D104" s="28" t="inlineStr">
         <is>
-          <t>Under 46</t>
+          <t>Under 15</t>
         </is>
       </c>
       <c r="E104" s="28" t="n">
@@ -9201,17 +9197,17 @@
       </c>
       <c r="F104" s="28" t="inlineStr">
         <is>
-          <t>U46-SF1</t>
+          <t>U15-SF2</t>
         </is>
       </c>
       <c r="G104" s="28" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H104" s="28" t="inlineStr">
         <is>
-          <t>Group B 1st</t>
+          <t>Group A 1st</t>
         </is>
       </c>
       <c r="I104" s="28" t="inlineStr">
@@ -9221,7 +9217,7 @@
       </c>
       <c r="J104" s="28" t="inlineStr">
         <is>
-          <t>Group A 2nd</t>
+          <t>Group B 2nd</t>
         </is>
       </c>
     </row>
@@ -9233,17 +9229,17 @@
       </c>
       <c r="B105" s="27" t="inlineStr">
         <is>
-          <t>3:50PM</t>
+          <t>4:15PM</t>
         </is>
       </c>
       <c r="C105" s="27" t="inlineStr">
         <is>
-          <t>4:05PM</t>
+          <t>4:30PM</t>
         </is>
       </c>
       <c r="D105" s="27" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Under 26</t>
         </is>
       </c>
       <c r="E105" s="27" t="n">
@@ -9251,17 +9247,17 @@
       </c>
       <c r="F105" s="27" t="inlineStr">
         <is>
-          <t>U36-SF1</t>
+          <t>U26-FINAL</t>
         </is>
       </c>
       <c r="G105" s="27" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H105" s="27" t="inlineStr">
         <is>
-          <t>Group B 1st</t>
+          <t>Pool 1st</t>
         </is>
       </c>
       <c r="I105" s="27" t="inlineStr">
@@ -9271,7 +9267,7 @@
       </c>
       <c r="J105" s="27" t="inlineStr">
         <is>
-          <t>Group A 2nd</t>
+          <t>Pool 2nd</t>
         </is>
       </c>
     </row>
@@ -9283,17 +9279,17 @@
       </c>
       <c r="B106" s="28" t="inlineStr">
         <is>
-          <t>4:00PM</t>
+          <t>4:24PM</t>
         </is>
       </c>
       <c r="C106" s="28" t="inlineStr">
         <is>
-          <t>4:15PM</t>
+          <t>4:39PM</t>
         </is>
       </c>
       <c r="D106" s="28" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Under 36</t>
         </is>
       </c>
       <c r="E106" s="28" t="n">
@@ -9301,17 +9297,17 @@
       </c>
       <c r="F106" s="28" t="inlineStr">
         <is>
-          <t>SR-SF2</t>
+          <t>U36-SF1</t>
         </is>
       </c>
       <c r="G106" s="28" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H106" s="28" t="inlineStr">
         <is>
-          <t>Group A 1st</t>
+          <t>Group B 1st</t>
         </is>
       </c>
       <c r="I106" s="28" t="inlineStr">
@@ -9321,7 +9317,7 @@
       </c>
       <c r="J106" s="28" t="inlineStr">
         <is>
-          <t>Group B 2nd</t>
+          <t>Group A 2nd</t>
         </is>
       </c>
     </row>
@@ -9333,17 +9329,17 @@
       </c>
       <c r="B107" s="27" t="inlineStr">
         <is>
-          <t>4:05PM</t>
+          <t>4:30PM</t>
         </is>
       </c>
       <c r="C107" s="27" t="inlineStr">
         <is>
-          <t>4:20PM</t>
+          <t>4:45PM</t>
         </is>
       </c>
       <c r="D107" s="27" t="inlineStr">
         <is>
-          <t>Under 32</t>
+          <t>Under 15</t>
         </is>
       </c>
       <c r="E107" s="27" t="n">
@@ -9351,17 +9347,17 @@
       </c>
       <c r="F107" s="27" t="inlineStr">
         <is>
-          <t>U32-FINAL</t>
+          <t>U15-FINAL</t>
         </is>
       </c>
       <c r="G107" s="27" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H107" s="27" t="inlineStr">
         <is>
-          <t>Pool 1st</t>
+          <t>Winner SF1</t>
         </is>
       </c>
       <c r="I107" s="27" t="inlineStr">
@@ -9371,7 +9367,7 @@
       </c>
       <c r="J107" s="27" t="inlineStr">
         <is>
-          <t>Pool 2nd</t>
+          <t>Winner SF2</t>
         </is>
       </c>
     </row>
@@ -9383,17 +9379,17 @@
       </c>
       <c r="B108" s="28" t="inlineStr">
         <is>
-          <t>4:15PM</t>
+          <t>4:39PM</t>
         </is>
       </c>
       <c r="C108" s="28" t="inlineStr">
         <is>
-          <t>4:30PM</t>
+          <t>4:54PM</t>
         </is>
       </c>
       <c r="D108" s="28" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Under 36</t>
         </is>
       </c>
       <c r="E108" s="28" t="n">
@@ -9401,17 +9397,17 @@
       </c>
       <c r="F108" s="28" t="inlineStr">
         <is>
-          <t>SR-FINAL</t>
+          <t>U36-SF2</t>
         </is>
       </c>
       <c r="G108" s="28" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H108" s="28" t="inlineStr">
         <is>
-          <t>Winner SF1</t>
+          <t>Group A 1st</t>
         </is>
       </c>
       <c r="I108" s="28" t="inlineStr">
@@ -9421,7 +9417,7 @@
       </c>
       <c r="J108" s="28" t="inlineStr">
         <is>
-          <t>Winner SF2</t>
+          <t>Group B 2nd</t>
         </is>
       </c>
     </row>
@@ -9433,17 +9429,17 @@
       </c>
       <c r="B109" s="27" t="inlineStr">
         <is>
-          <t>4:20PM</t>
+          <t>5:04PM</t>
         </is>
       </c>
       <c r="C109" s="27" t="inlineStr">
         <is>
-          <t>4:35PM</t>
+          <t>5:19PM</t>
         </is>
       </c>
       <c r="D109" s="27" t="inlineStr">
         <is>
-          <t>Under 15</t>
+          <t>Under 36</t>
         </is>
       </c>
       <c r="E109" s="27" t="n">
@@ -9451,17 +9447,17 @@
       </c>
       <c r="F109" s="27" t="inlineStr">
         <is>
-          <t>U15-SF1</t>
+          <t>U36-FINAL</t>
         </is>
       </c>
       <c r="G109" s="27" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H109" s="27" t="inlineStr">
         <is>
-          <t>Group B 1st</t>
+          <t>Winner SF1</t>
         </is>
       </c>
       <c r="I109" s="27" t="inlineStr">
@@ -9471,7 +9467,7 @@
       </c>
       <c r="J109" s="27" t="inlineStr">
         <is>
-          <t>Group A 2nd</t>
+          <t>Winner SF2</t>
         </is>
       </c>
     </row>
@@ -9483,12 +9479,12 @@
       </c>
       <c r="B110" s="28" t="inlineStr">
         <is>
-          <t>4:30PM</t>
+          <t>5:10PM</t>
         </is>
       </c>
       <c r="C110" s="28" t="inlineStr">
         <is>
-          <t>4:45PM</t>
+          <t>5:25PM</t>
         </is>
       </c>
       <c r="D110" s="28" t="inlineStr">
@@ -9501,17 +9497,17 @@
       </c>
       <c r="F110" s="28" t="inlineStr">
         <is>
-          <t>U46-SF2</t>
+          <t>U46-SF1</t>
         </is>
       </c>
       <c r="G110" s="28" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H110" s="28" t="inlineStr">
         <is>
-          <t>Group A 1st</t>
+          <t>Group B 1st</t>
         </is>
       </c>
       <c r="I110" s="28" t="inlineStr">
@@ -9521,7 +9517,7 @@
       </c>
       <c r="J110" s="28" t="inlineStr">
         <is>
-          <t>Group B 2nd</t>
+          <t>Group A 2nd</t>
         </is>
       </c>
     </row>
@@ -9533,17 +9529,17 @@
       </c>
       <c r="B111" s="27" t="inlineStr">
         <is>
-          <t>4:45PM</t>
+          <t>5:19PM</t>
         </is>
       </c>
       <c r="C111" s="27" t="inlineStr">
         <is>
-          <t>5:00PM</t>
+          <t>5:34PM</t>
         </is>
       </c>
       <c r="D111" s="27" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E111" s="27" t="n">
@@ -9551,7 +9547,7 @@
       </c>
       <c r="F111" s="27" t="inlineStr">
         <is>
-          <t>U36-SF2</t>
+          <t>U46-SF2</t>
         </is>
       </c>
       <c r="G111" s="27" t="inlineStr">
@@ -9583,17 +9579,17 @@
       </c>
       <c r="B112" s="28" t="inlineStr">
         <is>
-          <t>5:00PM</t>
+          <t>5:25PM</t>
         </is>
       </c>
       <c r="C112" s="28" t="inlineStr">
         <is>
-          <t>5:15PM</t>
+          <t>5:40PM</t>
         </is>
       </c>
       <c r="D112" s="28" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E112" s="28" t="n">
@@ -9601,17 +9597,17 @@
       </c>
       <c r="F112" s="28" t="inlineStr">
         <is>
-          <t>U36-FINAL</t>
+          <t>A46-SF1</t>
         </is>
       </c>
       <c r="G112" s="28" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H112" s="28" t="inlineStr">
         <is>
-          <t>Winner SF1</t>
+          <t>Group B 1st</t>
         </is>
       </c>
       <c r="I112" s="28" t="inlineStr">
@@ -9621,7 +9617,7 @@
       </c>
       <c r="J112" s="28" t="inlineStr">
         <is>
-          <t>Winner SF2</t>
+          <t>Group A 2nd</t>
         </is>
       </c>
     </row>
@@ -9633,17 +9629,17 @@
       </c>
       <c r="B113" s="27" t="inlineStr">
         <is>
-          <t>5:15PM</t>
+          <t>5:34PM</t>
         </is>
       </c>
       <c r="C113" s="27" t="inlineStr">
         <is>
-          <t>5:30PM</t>
+          <t>5:49PM</t>
         </is>
       </c>
       <c r="D113" s="27" t="inlineStr">
         <is>
-          <t>Under 15</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E113" s="27" t="n">
@@ -9651,7 +9647,7 @@
       </c>
       <c r="F113" s="27" t="inlineStr">
         <is>
-          <t>U15-SF2</t>
+          <t>A46-SF2</t>
         </is>
       </c>
       <c r="G113" s="27" t="inlineStr">
@@ -9683,12 +9679,12 @@
       </c>
       <c r="B114" s="28" t="inlineStr">
         <is>
-          <t>5:30PM</t>
+          <t>5:44PM</t>
         </is>
       </c>
       <c r="C114" s="28" t="inlineStr">
         <is>
-          <t>5:45PM</t>
+          <t>5:59PM</t>
         </is>
       </c>
       <c r="D114" s="28" t="inlineStr">
@@ -9706,7 +9702,7 @@
       </c>
       <c r="G114" s="28" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H114" s="28" t="inlineStr">
@@ -9733,17 +9729,17 @@
       </c>
       <c r="B115" s="27" t="inlineStr">
         <is>
-          <t>5:30PM</t>
+          <t>5:59PM</t>
         </is>
       </c>
       <c r="C115" s="27" t="inlineStr">
         <is>
-          <t>5:45PM</t>
+          <t>6:14PM</t>
         </is>
       </c>
       <c r="D115" s="27" t="inlineStr">
         <is>
-          <t>Under 15</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E115" s="27" t="n">
@@ -9751,12 +9747,12 @@
       </c>
       <c r="F115" s="27" t="inlineStr">
         <is>
-          <t>U15-FINAL</t>
+          <t>A46-FINAL</t>
         </is>
       </c>
       <c r="G115" s="27" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H115" s="27" t="inlineStr">
@@ -9779,20 +9775,20 @@
   <mergeCells count="17">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A36:J36"/>
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="A34:J34"/>
     <mergeCell ref="A12:J12"/>
     <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A43:J43"/>
     <mergeCell ref="A20:J20"/>
-    <mergeCell ref="A43:J43"/>
     <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A28:J28"/>
+    <mergeCell ref="A26:J26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="D35:E35"/>
     <mergeCell ref="D21:E21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9834,7 +9830,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="20.1" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -9842,7 +9837,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="17.1" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
         <is>
@@ -9942,8 +9936,6 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17"/>
     <row r="18" ht="20.1" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
@@ -10408,7 +10400,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="17.1" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
         <is>
@@ -10458,7 +10449,6 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="17.1" customHeight="1">
       <c r="A12" s="24" t="inlineStr">
         <is>
@@ -10586,7 +10576,6 @@
         <v>45</v>
       </c>
     </row>
-    <row r="20"/>
     <row r="21" ht="17.1" customHeight="1">
       <c r="A21" s="24" t="inlineStr">
         <is>
@@ -10678,8 +10667,6 @@
         <v>65</v>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
     <row r="29" ht="20.1" customHeight="1">
       <c r="A29" s="16" t="inlineStr">
         <is>
@@ -13400,7 +13387,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="17.1" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
         <is>
@@ -13470,8 +13456,6 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
     <row r="15" ht="20.1" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
@@ -14128,7 +14112,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="20.1" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -14136,7 +14119,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="17.1" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
         <is>
@@ -14306,7 +14288,6 @@
         <v>47</v>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="25" t="inlineStr">
         <is>
@@ -14314,7 +14295,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26" ht="20.1" customHeight="1">
       <c r="A26" s="16" t="inlineStr">
         <is>
@@ -15122,7 +15102,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="20.1" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
@@ -15130,7 +15109,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="17.1" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
         <is>
@@ -15240,7 +15218,6 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="17.1" customHeight="1">
       <c r="A14" s="24" t="inlineStr">
         <is>
@@ -15350,7 +15327,6 @@
         <v>61</v>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="17.1" customHeight="1">
       <c r="A22" s="24" t="inlineStr">
         <is>
@@ -15442,8 +15418,6 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
     <row r="30" ht="20.1" customHeight="1">
       <c r="A30" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Reprioritize TT Men's Above 46 knockout to lead off the morning at 8am
Above 46 (Sanjay Kumar's bye bracket) now grabs Table 1 as the very
first TT match of the day (Match 1, Aug 15 8:00 AM) whenever it ties
with another band for earliest achievable start, since none of its 9
players have any other-event commitment before Aug 15 evening. Same
dependency-based reflow as before, just with tie-breaking changed to
favor Above 46 over other TT bands/events.

Net effect: TT Women's Singles now 8:00-11:15 AM, TT Men's Singles
8:00 AM-4:00 PM Aug 16 (was 10:45 AM-4:45 PM), TT Doubles now wraps
4:30 PM Aug 16. Overall tournament finish unchanged at 5:00 PM Aug 16
(still gated by Chess). Verified zero venue conflicts and zero
player-continuity/break-rule violations.

Updates index.html SEED_DATA, the schedule workbook's TT sheets +
Overview summary, CLAUDE.md, and the Firestore import file — Firestore
has already been re-synced to match.
</commit_message>
<xml_diff>
--- a/Ekta_Schedule_With_Matchups.xlsx
+++ b/Ekta_Schedule_With_Matchups.xlsx
@@ -1242,7 +1242,7 @@
       </c>
       <c r="C15" s="64" t="inlineStr">
         <is>
-          <t>League stage continues. Carrom Women's Singles (done ~11:00 AM) and TT Women's Singles (done ~11:00 AM) each finish in full today — their knockouts run right after their own league stage ends, no waiting for other events.</t>
+          <t>League stage continues. Carrom Women's Singles (done ~11:00 AM) and TT Women's Singles (done ~11:15 AM) each finish in full today — their knockouts run right after their own league stage ends, no waiting for other events. TT Men's Above 46 knockout leads off the morning on Table 1 at 8:00 AM.</t>
         </is>
       </c>
       <c r="H15" s="31" t="n"/>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="C17" s="64" t="inlineStr">
         <is>
-          <t>Both Doubles events run once their own players are free — Carrom Doubles 9:30-11:50 AM; TT Doubles starts 9:05 AM and interleaves with TT Men's Singles on the shared tables, wrapping by 3:45 PM.</t>
+          <t>Both Doubles events run once their own players are free — Carrom Doubles 9:30-11:50 AM; TT Doubles starts 9:05 AM and interleaves with TT Men's Singles on the shared tables, wrapping by 4:30 PM.</t>
         </is>
       </c>
       <c r="H17" s="31" t="n"/>
@@ -1416,7 +1416,7 @@
       </c>
       <c r="E24" s="63" t="inlineStr">
         <is>
-          <t>Aug15 11:00AM</t>
+          <t>Aug15 11:15AM</t>
         </is>
       </c>
       <c r="F24" s="31" t="n"/>
@@ -1441,12 +1441,12 @@
       </c>
       <c r="D25" s="63" t="inlineStr">
         <is>
-          <t>Aug15 10:45AM</t>
+          <t>Aug15 8:00AM</t>
         </is>
       </c>
       <c r="E25" s="63" t="inlineStr">
         <is>
-          <t>Aug16 4:45PM</t>
+          <t>Aug16 4:00PM</t>
         </is>
       </c>
       <c r="F25" s="31" t="n"/>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="E26" s="63" t="inlineStr">
         <is>
-          <t>Aug16 3:45PM</t>
+          <t>Aug16 4:30PM</t>
         </is>
       </c>
       <c r="F26" s="31" t="n"/>
@@ -4995,7 +4995,7 @@
       </c>
       <c r="G16" s="94" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H16" s="94" t="inlineStr">
@@ -5022,12 +5022,12 @@
       </c>
       <c r="B17" s="95" t="inlineStr">
         <is>
-          <t>8:00AM</t>
+          <t>8:15AM</t>
         </is>
       </c>
       <c r="C17" s="95" t="inlineStr">
         <is>
-          <t>8:15AM</t>
+          <t>8:30AM</t>
         </is>
       </c>
       <c r="D17" s="95" t="inlineStr">
@@ -5045,7 +5045,7 @@
       </c>
       <c r="G17" s="95" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H17" s="95" t="inlineStr">
@@ -5095,7 +5095,7 @@
       </c>
       <c r="G18" s="94" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H18" s="94" t="inlineStr">
@@ -5122,12 +5122,12 @@
       </c>
       <c r="B19" s="95" t="inlineStr">
         <is>
-          <t>8:15AM</t>
+          <t>8:30AM</t>
         </is>
       </c>
       <c r="C19" s="95" t="inlineStr">
         <is>
-          <t>8:30AM</t>
+          <t>8:45AM</t>
         </is>
       </c>
       <c r="D19" s="95" t="inlineStr">
@@ -5145,7 +5145,7 @@
       </c>
       <c r="G19" s="95" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H19" s="95" t="inlineStr">
@@ -5172,12 +5172,12 @@
       </c>
       <c r="B20" s="94" t="inlineStr">
         <is>
-          <t>8:30AM</t>
+          <t>8:45AM</t>
         </is>
       </c>
       <c r="C20" s="94" t="inlineStr">
         <is>
-          <t>8:45AM</t>
+          <t>9:00AM</t>
         </is>
       </c>
       <c r="D20" s="94" t="inlineStr">
@@ -5222,12 +5222,12 @@
       </c>
       <c r="B21" s="95" t="inlineStr">
         <is>
-          <t>8:30AM</t>
+          <t>8:45AM</t>
         </is>
       </c>
       <c r="C21" s="95" t="inlineStr">
         <is>
-          <t>8:45AM</t>
+          <t>9:00AM</t>
         </is>
       </c>
       <c r="D21" s="95" t="inlineStr">
@@ -5272,12 +5272,12 @@
       </c>
       <c r="B22" s="94" t="inlineStr">
         <is>
-          <t>8:45AM</t>
+          <t>9:00AM</t>
         </is>
       </c>
       <c r="C22" s="94" t="inlineStr">
         <is>
-          <t>9:00AM</t>
+          <t>9:15AM</t>
         </is>
       </c>
       <c r="D22" s="94" t="inlineStr">
@@ -5322,12 +5322,12 @@
       </c>
       <c r="B23" s="95" t="inlineStr">
         <is>
-          <t>8:45AM</t>
+          <t>9:00AM</t>
         </is>
       </c>
       <c r="C23" s="95" t="inlineStr">
         <is>
-          <t>9:00AM</t>
+          <t>9:15AM</t>
         </is>
       </c>
       <c r="D23" s="95" t="inlineStr">
@@ -5372,12 +5372,12 @@
       </c>
       <c r="B24" s="94" t="inlineStr">
         <is>
-          <t>9:00AM</t>
+          <t>9:15AM</t>
         </is>
       </c>
       <c r="C24" s="94" t="inlineStr">
         <is>
-          <t>9:15AM</t>
+          <t>9:30AM</t>
         </is>
       </c>
       <c r="D24" s="94" t="inlineStr">
@@ -5422,12 +5422,12 @@
       </c>
       <c r="B25" s="95" t="inlineStr">
         <is>
-          <t>9:00AM</t>
+          <t>9:15AM</t>
         </is>
       </c>
       <c r="C25" s="95" t="inlineStr">
         <is>
-          <t>9:15AM</t>
+          <t>9:30AM</t>
         </is>
       </c>
       <c r="D25" s="95" t="inlineStr">
@@ -5472,12 +5472,12 @@
       </c>
       <c r="B26" s="94" t="inlineStr">
         <is>
-          <t>9:15AM</t>
+          <t>10:30AM</t>
         </is>
       </c>
       <c r="C26" s="94" t="inlineStr">
         <is>
-          <t>9:30AM</t>
+          <t>10:45AM</t>
         </is>
       </c>
       <c r="D26" s="94" t="inlineStr">
@@ -5522,12 +5522,12 @@
       </c>
       <c r="B27" s="95" t="inlineStr">
         <is>
-          <t>9:15AM</t>
+          <t>10:30AM</t>
         </is>
       </c>
       <c r="C27" s="95" t="inlineStr">
         <is>
-          <t>9:30AM</t>
+          <t>10:45AM</t>
         </is>
       </c>
       <c r="D27" s="95" t="inlineStr">
@@ -5572,12 +5572,12 @@
       </c>
       <c r="B28" s="94" t="inlineStr">
         <is>
-          <t>10:30AM</t>
+          <t>10:45AM</t>
         </is>
       </c>
       <c r="C28" s="94" t="inlineStr">
         <is>
-          <t>10:45AM</t>
+          <t>11:00AM</t>
         </is>
       </c>
       <c r="D28" s="94" t="inlineStr">
@@ -5622,12 +5622,12 @@
       </c>
       <c r="B29" s="95" t="inlineStr">
         <is>
-          <t>10:30AM</t>
+          <t>10:45AM</t>
         </is>
       </c>
       <c r="C29" s="95" t="inlineStr">
         <is>
-          <t>10:45AM</t>
+          <t>11:00AM</t>
         </is>
       </c>
       <c r="D29" s="95" t="inlineStr">
@@ -5672,12 +5672,12 @@
       </c>
       <c r="B30" s="94" t="inlineStr">
         <is>
-          <t>10:45AM</t>
+          <t>11:00AM</t>
         </is>
       </c>
       <c r="C30" s="94" t="inlineStr">
         <is>
-          <t>11:00AM</t>
+          <t>11:15AM</t>
         </is>
       </c>
       <c r="D30" s="94" t="inlineStr">
@@ -6448,17 +6448,17 @@
       </c>
       <c r="B49" s="94" t="inlineStr">
         <is>
-          <t>10:45AM</t>
+          <t>8:00AM</t>
         </is>
       </c>
       <c r="C49" s="94" t="inlineStr">
         <is>
-          <t>11:00AM</t>
+          <t>8:15AM</t>
         </is>
       </c>
       <c r="D49" s="94" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E49" s="94" t="n">
@@ -6466,17 +6466,17 @@
       </c>
       <c r="F49" s="94" t="inlineStr">
         <is>
-          <t>U36-GB-1</t>
+          <t>A46-QF3</t>
         </is>
       </c>
       <c r="G49" s="94" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H49" s="94" t="inlineStr">
         <is>
-          <t>Prakshal Shah</t>
+          <t>Ghansyam nawani</t>
         </is>
       </c>
       <c r="I49" s="94" t="inlineStr">
@@ -6486,7 +6486,7 @@
       </c>
       <c r="J49" s="94" t="inlineStr">
         <is>
-          <t>Amar Parulekar</t>
+          <t>HARSHAPRABHAT SHETTY</t>
         </is>
       </c>
     </row>
@@ -6498,17 +6498,17 @@
       </c>
       <c r="B50" s="95" t="inlineStr">
         <is>
-          <t>11:00AM</t>
+          <t>8:30AM</t>
         </is>
       </c>
       <c r="C50" s="95" t="inlineStr">
         <is>
-          <t>11:15AM</t>
+          <t>8:45AM</t>
         </is>
       </c>
       <c r="D50" s="95" t="inlineStr">
         <is>
-          <t>Above 46</t>
+          <t>Under 36</t>
         </is>
       </c>
       <c r="E50" s="95" t="n">
@@ -6516,17 +6516,17 @@
       </c>
       <c r="F50" s="95" t="inlineStr">
         <is>
-          <t>A46-QF3</t>
+          <t>U36-GB-1</t>
         </is>
       </c>
       <c r="G50" s="95" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H50" s="95" t="inlineStr">
         <is>
-          <t>Ghansyam nawani</t>
+          <t>Prakshal Shah</t>
         </is>
       </c>
       <c r="I50" s="95" t="inlineStr">
@@ -6536,7 +6536,7 @@
       </c>
       <c r="J50" s="95" t="inlineStr">
         <is>
-          <t>HARSHAPRABHAT SHETTY</t>
+          <t>Amar Parulekar</t>
         </is>
       </c>
     </row>
@@ -7808,7 +7808,7 @@
       </c>
       <c r="D76" s="95" t="inlineStr">
         <is>
-          <t>Under 36</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E76" s="95" t="n">
@@ -7816,7 +7816,7 @@
       </c>
       <c r="F76" s="95" t="inlineStr">
         <is>
-          <t>U36-FINAL</t>
+          <t>A46-QF4</t>
         </is>
       </c>
       <c r="G76" s="95" t="inlineStr">
@@ -7826,7 +7826,7 @@
       </c>
       <c r="H76" s="95" t="inlineStr">
         <is>
-          <t>Winner SF1</t>
+          <t>Mukul Joshi</t>
         </is>
       </c>
       <c r="I76" s="95" t="inlineStr">
@@ -7836,7 +7836,7 @@
       </c>
       <c r="J76" s="95" t="inlineStr">
         <is>
-          <t>Winner SF2</t>
+          <t>Sushil Dashpute</t>
         </is>
       </c>
     </row>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="D77" s="94" t="inlineStr">
         <is>
-          <t>Above 46</t>
+          <t>Under 36</t>
         </is>
       </c>
       <c r="E77" s="94" t="n">
@@ -7866,7 +7866,7 @@
       </c>
       <c r="F77" s="94" t="inlineStr">
         <is>
-          <t>A46-QF4</t>
+          <t>U36-FINAL</t>
         </is>
       </c>
       <c r="G77" s="94" t="inlineStr">
@@ -7876,7 +7876,7 @@
       </c>
       <c r="H77" s="94" t="inlineStr">
         <is>
-          <t>Mukul Joshi</t>
+          <t>Winner SF1</t>
         </is>
       </c>
       <c r="I77" s="94" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="J77" s="94" t="inlineStr">
         <is>
-          <t>Sushil Dashpute</t>
+          <t>Winner SF2</t>
         </is>
       </c>
     </row>
@@ -7908,7 +7908,7 @@
       </c>
       <c r="D78" s="95" t="inlineStr">
         <is>
-          <t>Under 46</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E78" s="95" t="n">
@@ -7916,7 +7916,7 @@
       </c>
       <c r="F78" s="95" t="inlineStr">
         <is>
-          <t>U46-GA-10</t>
+          <t>A46-SF2</t>
         </is>
       </c>
       <c r="G78" s="95" t="inlineStr">
@@ -7926,7 +7926,7 @@
       </c>
       <c r="H78" s="95" t="inlineStr">
         <is>
-          <t>Tanmay Sharma</t>
+          <t>Winner QF3</t>
         </is>
       </c>
       <c r="I78" s="95" t="inlineStr">
@@ -7936,7 +7936,7 @@
       </c>
       <c r="J78" s="95" t="inlineStr">
         <is>
-          <t>Anuj Shah</t>
+          <t>Winner QF4</t>
         </is>
       </c>
     </row>
@@ -7958,7 +7958,7 @@
       </c>
       <c r="D79" s="94" t="inlineStr">
         <is>
-          <t>Above 46</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E79" s="94" t="n">
@@ -7966,7 +7966,7 @@
       </c>
       <c r="F79" s="94" t="inlineStr">
         <is>
-          <t>A46-SF2</t>
+          <t>U46-GA-10</t>
         </is>
       </c>
       <c r="G79" s="94" t="inlineStr">
@@ -7976,7 +7976,7 @@
       </c>
       <c r="H79" s="94" t="inlineStr">
         <is>
-          <t>Winner QF3</t>
+          <t>Tanmay Sharma</t>
         </is>
       </c>
       <c r="I79" s="94" t="inlineStr">
@@ -7986,7 +7986,7 @@
       </c>
       <c r="J79" s="94" t="inlineStr">
         <is>
-          <t>Winner QF4</t>
+          <t>Anuj Shah</t>
         </is>
       </c>
     </row>
@@ -9058,7 +9058,7 @@
       </c>
       <c r="D101" s="94" t="inlineStr">
         <is>
-          <t>Under 46</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E101" s="94" t="n">
@@ -9066,7 +9066,7 @@
       </c>
       <c r="F101" s="94" t="inlineStr">
         <is>
-          <t>U46-GB-7</t>
+          <t>A46-R1</t>
         </is>
       </c>
       <c r="G101" s="94" t="inlineStr">
@@ -9076,7 +9076,7 @@
       </c>
       <c r="H101" s="94" t="inlineStr">
         <is>
-          <t>Piyush Makharia</t>
+          <t>Adil Khan</t>
         </is>
       </c>
       <c r="I101" s="94" t="inlineStr">
@@ -9086,7 +9086,7 @@
       </c>
       <c r="J101" s="94" t="inlineStr">
         <is>
-          <t>Amit Ranka</t>
+          <t>Ajit nair</t>
         </is>
       </c>
     </row>
@@ -9098,12 +9098,12 @@
       </c>
       <c r="B102" s="95" t="inlineStr">
         <is>
+          <t>3:00PM</t>
+        </is>
+      </c>
+      <c r="C102" s="95" t="inlineStr">
+        <is>
           <t>3:15PM</t>
-        </is>
-      </c>
-      <c r="C102" s="95" t="inlineStr">
-        <is>
-          <t>3:30PM</t>
         </is>
       </c>
       <c r="D102" s="95" t="inlineStr">
@@ -9116,17 +9116,17 @@
       </c>
       <c r="F102" s="95" t="inlineStr">
         <is>
-          <t>U46-SF1</t>
+          <t>U46-GB-7</t>
         </is>
       </c>
       <c r="G102" s="95" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H102" s="95" t="inlineStr">
         <is>
-          <t>Group B 1st</t>
+          <t>Piyush Makharia</t>
         </is>
       </c>
       <c r="I102" s="95" t="inlineStr">
@@ -9136,7 +9136,7 @@
       </c>
       <c r="J102" s="95" t="inlineStr">
         <is>
-          <t>Group A 2nd</t>
+          <t>Amit Ranka</t>
         </is>
       </c>
     </row>
@@ -9158,7 +9158,7 @@
       </c>
       <c r="D103" s="94" t="inlineStr">
         <is>
-          <t>Under 46</t>
+          <t>Above 46</t>
         </is>
       </c>
       <c r="E103" s="94" t="n">
@@ -9166,17 +9166,17 @@
       </c>
       <c r="F103" s="94" t="inlineStr">
         <is>
-          <t>U46-SF2</t>
+          <t>A46-QF1</t>
         </is>
       </c>
       <c r="G103" s="94" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H103" s="94" t="inlineStr">
         <is>
-          <t>Group A 1st</t>
+          <t>Winner R1</t>
         </is>
       </c>
       <c r="I103" s="94" t="inlineStr">
@@ -9186,7 +9186,7 @@
       </c>
       <c r="J103" s="94" t="inlineStr">
         <is>
-          <t>Group B 2nd</t>
+          <t>Sanjay Kumar</t>
         </is>
       </c>
     </row>
@@ -9198,12 +9198,12 @@
       </c>
       <c r="B104" s="95" t="inlineStr">
         <is>
+          <t>3:15PM</t>
+        </is>
+      </c>
+      <c r="C104" s="95" t="inlineStr">
+        <is>
           <t>3:30PM</t>
-        </is>
-      </c>
-      <c r="C104" s="95" t="inlineStr">
-        <is>
-          <t>3:45PM</t>
         </is>
       </c>
       <c r="D104" s="95" t="inlineStr">
@@ -9216,17 +9216,17 @@
       </c>
       <c r="F104" s="95" t="inlineStr">
         <is>
-          <t>U46-FINAL</t>
+          <t>U46-SF1</t>
         </is>
       </c>
       <c r="G104" s="95" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H104" s="95" t="inlineStr">
         <is>
-          <t>Winner SF1</t>
+          <t>Group B 1st</t>
         </is>
       </c>
       <c r="I104" s="95" t="inlineStr">
@@ -9236,7 +9236,7 @@
       </c>
       <c r="J104" s="95" t="inlineStr">
         <is>
-          <t>Winner SF2</t>
+          <t>Group A 2nd</t>
         </is>
       </c>
     </row>
@@ -9248,12 +9248,12 @@
       </c>
       <c r="B105" s="94" t="inlineStr">
         <is>
+          <t>3:30PM</t>
+        </is>
+      </c>
+      <c r="C105" s="94" t="inlineStr">
+        <is>
           <t>3:45PM</t>
-        </is>
-      </c>
-      <c r="C105" s="94" t="inlineStr">
-        <is>
-          <t>4:00PM</t>
         </is>
       </c>
       <c r="D105" s="94" t="inlineStr">
@@ -9266,7 +9266,7 @@
       </c>
       <c r="F105" s="94" t="inlineStr">
         <is>
-          <t>A46-R1</t>
+          <t>A46-SF1</t>
         </is>
       </c>
       <c r="G105" s="94" t="inlineStr">
@@ -9276,7 +9276,7 @@
       </c>
       <c r="H105" s="94" t="inlineStr">
         <is>
-          <t>Adil Khan</t>
+          <t>Winner QF1</t>
         </is>
       </c>
       <c r="I105" s="94" t="inlineStr">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="J105" s="94" t="inlineStr">
         <is>
-          <t>Ajit nair</t>
+          <t>Winner QF2</t>
         </is>
       </c>
     </row>
@@ -9298,17 +9298,17 @@
       </c>
       <c r="B106" s="95" t="inlineStr">
         <is>
-          <t>4:00PM</t>
+          <t>3:30PM</t>
         </is>
       </c>
       <c r="C106" s="95" t="inlineStr">
         <is>
-          <t>4:15PM</t>
+          <t>3:45PM</t>
         </is>
       </c>
       <c r="D106" s="95" t="inlineStr">
         <is>
-          <t>Above 46</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E106" s="95" t="n">
@@ -9316,17 +9316,17 @@
       </c>
       <c r="F106" s="95" t="inlineStr">
         <is>
-          <t>A46-QF1</t>
+          <t>U46-SF2</t>
         </is>
       </c>
       <c r="G106" s="95" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H106" s="95" t="inlineStr">
         <is>
-          <t>Winner R1</t>
+          <t>Group A 1st</t>
         </is>
       </c>
       <c r="I106" s="95" t="inlineStr">
@@ -9336,7 +9336,7 @@
       </c>
       <c r="J106" s="95" t="inlineStr">
         <is>
-          <t>Sanjay Kumar</t>
+          <t>Group B 2nd</t>
         </is>
       </c>
     </row>
@@ -9348,12 +9348,12 @@
       </c>
       <c r="B107" s="94" t="inlineStr">
         <is>
-          <t>4:15PM</t>
+          <t>3:45PM</t>
         </is>
       </c>
       <c r="C107" s="94" t="inlineStr">
         <is>
-          <t>4:30PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="D107" s="94" t="inlineStr">
@@ -9366,7 +9366,7 @@
       </c>
       <c r="F107" s="94" t="inlineStr">
         <is>
-          <t>A46-SF1</t>
+          <t>A46-FINAL</t>
         </is>
       </c>
       <c r="G107" s="94" t="inlineStr">
@@ -9376,7 +9376,7 @@
       </c>
       <c r="H107" s="94" t="inlineStr">
         <is>
-          <t>Winner QF1</t>
+          <t>Winner SF1</t>
         </is>
       </c>
       <c r="I107" s="94" t="inlineStr">
@@ -9386,7 +9386,7 @@
       </c>
       <c r="J107" s="94" t="inlineStr">
         <is>
-          <t>Winner QF2</t>
+          <t>Winner SF2</t>
         </is>
       </c>
     </row>
@@ -9398,17 +9398,17 @@
       </c>
       <c r="B108" s="95" t="inlineStr">
         <is>
-          <t>4:30PM</t>
+          <t>3:45PM</t>
         </is>
       </c>
       <c r="C108" s="95" t="inlineStr">
         <is>
-          <t>4:45PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="D108" s="95" t="inlineStr">
         <is>
-          <t>Above 46</t>
+          <t>Under 46</t>
         </is>
       </c>
       <c r="E108" s="95" t="n">
@@ -9416,12 +9416,12 @@
       </c>
       <c r="F108" s="95" t="inlineStr">
         <is>
-          <t>A46-FINAL</t>
+          <t>U46-FINAL</t>
         </is>
       </c>
       <c r="G108" s="95" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Table 2</t>
         </is>
       </c>
       <c r="H108" s="95" t="inlineStr">
@@ -9533,7 +9533,7 @@
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A6:J6"/>
     <mergeCell ref="A35:H35"/>
-    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="A34:H34"/>
     <mergeCell ref="D27:E27"/>
     <mergeCell ref="A12:J12"/>
     <mergeCell ref="A4:J4"/>
@@ -9541,7 +9541,7 @@
     <mergeCell ref="A26:J26"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="D21:E21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10005,12 +10005,12 @@
       </c>
       <c r="B25" s="95" t="inlineStr">
         <is>
-          <t>3:00PM</t>
+          <t>4:00PM</t>
         </is>
       </c>
       <c r="C25" s="95" t="inlineStr">
         <is>
-          <t>3:15PM</t>
+          <t>4:15PM</t>
         </is>
       </c>
       <c r="D25" s="95" t="inlineStr">
@@ -10028,7 +10028,7 @@
       </c>
       <c r="G25" s="95" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H25" s="95" t="inlineStr">
@@ -10055,12 +10055,12 @@
       </c>
       <c r="B26" s="94" t="inlineStr">
         <is>
-          <t>3:30PM</t>
+          <t>4:15PM</t>
         </is>
       </c>
       <c r="C26" s="94" t="inlineStr">
         <is>
-          <t>3:45PM</t>
+          <t>4:30PM</t>
         </is>
       </c>
       <c r="D26" s="94" t="inlineStr">
@@ -10078,7 +10078,7 @@
       </c>
       <c r="G26" s="94" t="inlineStr">
         <is>
-          <t>Table 2</t>
+          <t>Table 1</t>
         </is>
       </c>
       <c r="H26" s="94" t="inlineStr">

</xml_diff>